<commit_message>
code for new scenarios
</commit_message>
<xml_diff>
--- a/data/data_analysis/policy_effectiveness.xlsx
+++ b/data/data_analysis/policy_effectiveness.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\data\data_analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E02A2FD5-683E-4502-AEF9-4D95388A35C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3088B160-18C9-4CF8-8A6D-F1F0B698A7DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{5B094011-67C9-461D-BBBF-A6D3FE50B4AB}"/>
   </bookViews>
@@ -16,6 +16,9 @@
     <sheet name="Low" sheetId="1" r:id="rId1"/>
     <sheet name="High" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Low!$A$3:$AP$3</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -720,7 +723,6 @@
         <v>7</v>
       </c>
       <c r="B4" s="3">
-        <f>E$4</f>
         <v>293793.7861481891</v>
       </c>
       <c r="C4" s="3">
@@ -883,7 +885,6 @@
         <v>8</v>
       </c>
       <c r="B5" s="3">
-        <f>E$4</f>
         <v>293793.7861481891</v>
       </c>
       <c r="C5" s="3">
@@ -1046,7 +1047,6 @@
         <v>9</v>
       </c>
       <c r="B6" s="3">
-        <f>E$4</f>
         <v>293793.7861481891</v>
       </c>
       <c r="C6" s="3">
@@ -1209,7 +1209,6 @@
         <v>10</v>
       </c>
       <c r="B7" s="3">
-        <f>E$4</f>
         <v>293793.7861481891</v>
       </c>
       <c r="C7" s="3">
@@ -1372,7 +1371,6 @@
         <v>11</v>
       </c>
       <c r="B8" s="3">
-        <f>E$4</f>
         <v>293793.7861481891</v>
       </c>
       <c r="C8" s="3">
@@ -1535,7 +1533,6 @@
         <v>12</v>
       </c>
       <c r="B9" s="3">
-        <f>E$4</f>
         <v>293793.7861481891</v>
       </c>
       <c r="C9" s="3">
@@ -1698,7 +1695,6 @@
         <v>13</v>
       </c>
       <c r="B10" s="3">
-        <f>E$4</f>
         <v>293793.7861481891</v>
       </c>
       <c r="C10" s="3">
@@ -1861,7 +1857,6 @@
         <v>14</v>
       </c>
       <c r="B11" s="3">
-        <f>E$4</f>
         <v>293793.7861481891</v>
       </c>
       <c r="C11" s="3">
@@ -2024,7 +2019,6 @@
         <v>15</v>
       </c>
       <c r="B12" s="3">
-        <f>E$4</f>
         <v>293793.7861481891</v>
       </c>
       <c r="C12" s="3">
@@ -2187,7 +2181,6 @@
         <v>16</v>
       </c>
       <c r="B13" s="3">
-        <f>E$4</f>
         <v>293793.7861481891</v>
       </c>
       <c r="C13" s="3">
@@ -2350,7 +2343,6 @@
         <v>17</v>
       </c>
       <c r="B14" s="3">
-        <f>E$4</f>
         <v>293793.7861481891</v>
       </c>
       <c r="C14" s="3">
@@ -2509,6 +2501,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A3:AP3" xr:uid="{E1B4DBF1-F2D7-44F8-977D-1BE3C41C10B1}"/>
   <mergeCells count="5">
     <mergeCell ref="K2:P2"/>
     <mergeCell ref="E2:G2"/>
@@ -2736,15 +2729,15 @@
         <v>18</v>
       </c>
       <c r="B4" s="3">
-        <f>E$4</f>
+        <f t="shared" ref="B4:B13" si="0">E$4</f>
         <v>709776.91212891659</v>
       </c>
       <c r="C4" s="3">
-        <f>F$4</f>
+        <f t="shared" ref="C4:C13" si="1">F$4</f>
         <v>219041.54431546232</v>
       </c>
       <c r="D4" s="3">
-        <f>G$4</f>
+        <f t="shared" ref="D4:D13" si="2">G$4</f>
         <v>79692.853169511349</v>
       </c>
       <c r="E4" s="3">
@@ -2760,15 +2753,15 @@
         <v>79692.853169511349</v>
       </c>
       <c r="H4" s="3">
-        <f>E4-$B4</f>
+        <f t="shared" ref="H4:H13" si="3">E4-$B4</f>
         <v>0</v>
       </c>
       <c r="I4" s="3">
-        <f>F4-$C4</f>
+        <f t="shared" ref="I4:I13" si="4">F4-$C4</f>
         <v>0</v>
       </c>
       <c r="J4" s="3">
-        <f>G4-$D4</f>
+        <f t="shared" ref="J4:J13" si="5">G4-$D4</f>
         <v>0</v>
       </c>
       <c r="K4">
@@ -2790,107 +2783,107 @@
         <v>316331</v>
       </c>
       <c r="Q4">
-        <f>K4</f>
+        <f t="shared" ref="Q4:Q13" si="6">K4</f>
         <v>4773</v>
       </c>
       <c r="R4">
-        <f>Q4+0.2*(V4-Q4)</f>
+        <f t="shared" ref="R4:R13" si="7">Q4+0.2*(V4-Q4)</f>
         <v>5848.8</v>
       </c>
       <c r="S4">
-        <f>Q4+0.4*(V4-Q4)</f>
+        <f t="shared" ref="S4:S13" si="8">Q4+0.4*(V4-Q4)</f>
         <v>6924.6</v>
       </c>
       <c r="T4">
-        <f>Q4+0.6*(V4-Q4)</f>
+        <f t="shared" ref="T4:T13" si="9">Q4+0.6*(V4-Q4)</f>
         <v>8000.4</v>
       </c>
       <c r="U4">
-        <f>Q4+0.8*(V4-Q4)</f>
+        <f t="shared" ref="U4:U13" si="10">Q4+0.8*(V4-Q4)</f>
         <v>9076.2000000000007</v>
       </c>
       <c r="V4">
-        <f>L4</f>
+        <f t="shared" ref="V4:V13" si="11">L4</f>
         <v>10152</v>
       </c>
       <c r="W4">
-        <f>V4+0.2*(AA4-V4)</f>
+        <f t="shared" ref="W4:W13" si="12">V4+0.2*(AA4-V4)</f>
         <v>12063</v>
       </c>
       <c r="X4">
-        <f>V4+0.4*(AA4-V4)</f>
+        <f t="shared" ref="X4:X13" si="13">V4+0.4*(AA4-V4)</f>
         <v>13974</v>
       </c>
       <c r="Y4">
-        <f>V4+0.6*(AA4-V4)</f>
+        <f t="shared" ref="Y4:Y13" si="14">V4+0.6*(AA4-V4)</f>
         <v>15885</v>
       </c>
       <c r="Z4">
-        <f>V4+0.8*(AA4-V4)</f>
+        <f t="shared" ref="Z4:Z13" si="15">V4+0.8*(AA4-V4)</f>
         <v>17796</v>
       </c>
       <c r="AA4">
-        <f>M4</f>
+        <f t="shared" ref="AA4:AA13" si="16">M4</f>
         <v>19707</v>
       </c>
       <c r="AB4">
-        <f>AA4+0.2*(AF4-AA4)</f>
+        <f t="shared" ref="AB4:AB13" si="17">AA4+0.2*(AF4-AA4)</f>
         <v>25136.6</v>
       </c>
       <c r="AC4">
-        <f>AA4+0.4*(AF4-AA4)</f>
+        <f t="shared" ref="AC4:AC13" si="18">AA4+0.4*(AF4-AA4)</f>
         <v>30566.2</v>
       </c>
       <c r="AD4">
-        <f>AA4+0.6*(AF4-AA4)</f>
+        <f t="shared" ref="AD4:AD13" si="19">AA4+0.6*(AF4-AA4)</f>
         <v>35995.800000000003</v>
       </c>
       <c r="AE4">
-        <f>AA4+0.8*(AF4-AA4)</f>
+        <f t="shared" ref="AE4:AE13" si="20">AA4+0.8*(AF4-AA4)</f>
         <v>41425.4</v>
       </c>
       <c r="AF4">
-        <f>N4</f>
+        <f t="shared" ref="AF4:AF13" si="21">N4</f>
         <v>46855</v>
       </c>
       <c r="AG4">
-        <f>AF4+0.2*(AK4-AF4)</f>
+        <f t="shared" ref="AG4:AG13" si="22">AF4+0.2*(AK4-AF4)</f>
         <v>60533.8</v>
       </c>
       <c r="AH4">
-        <f>AF4+0.4*(AK4-AF4)</f>
+        <f t="shared" ref="AH4:AH13" si="23">AF4+0.4*(AK4-AF4)</f>
         <v>74212.600000000006</v>
       </c>
       <c r="AI4">
-        <f>AF4+0.6*(AK4-AF4)</f>
+        <f t="shared" ref="AI4:AI13" si="24">AF4+0.6*(AK4-AF4)</f>
         <v>87891.4</v>
       </c>
       <c r="AJ4">
-        <f>AF4+0.8*(AK4-AF4)</f>
+        <f t="shared" ref="AJ4:AJ13" si="25">AF4+0.8*(AK4-AF4)</f>
         <v>101570.20000000001</v>
       </c>
       <c r="AK4">
-        <f>O4</f>
+        <f t="shared" ref="AK4:AK13" si="26">O4</f>
         <v>115249</v>
       </c>
       <c r="AL4">
-        <f>AK4+0.2*(AP4-AK4)</f>
+        <f t="shared" ref="AL4:AL13" si="27">AK4+0.2*(AP4-AK4)</f>
         <v>155465.4</v>
       </c>
       <c r="AM4">
-        <f>AK4+0.4*(AP4-AK4)</f>
+        <f t="shared" ref="AM4:AM13" si="28">AK4+0.4*(AP4-AK4)</f>
         <v>195681.8</v>
       </c>
       <c r="AN4">
-        <f>AK4+0.6*(AP4-AK4)</f>
+        <f t="shared" ref="AN4:AN13" si="29">AK4+0.6*(AP4-AK4)</f>
         <v>235898.2</v>
       </c>
       <c r="AO4">
-        <f>AK4+0.8*(AP4-AK4)</f>
+        <f t="shared" ref="AO4:AO13" si="30">AK4+0.8*(AP4-AK4)</f>
         <v>276114.59999999998</v>
       </c>
       <c r="AP4">
-        <f>P4</f>
+        <f t="shared" ref="AP4:AP13" si="31">P4</f>
         <v>316331</v>
       </c>
     </row>
@@ -2899,15 +2892,15 @@
         <v>19</v>
       </c>
       <c r="B5" s="3">
-        <f>E$4</f>
+        <f t="shared" si="0"/>
         <v>709776.91212891659</v>
       </c>
       <c r="C5" s="3">
-        <f>F$4</f>
+        <f t="shared" si="1"/>
         <v>219041.54431546232</v>
       </c>
       <c r="D5" s="3">
-        <f>G$4</f>
+        <f t="shared" si="2"/>
         <v>79692.853169511349</v>
       </c>
       <c r="E5" s="3">
@@ -2923,15 +2916,15 @@
         <v>77596.349178421689</v>
       </c>
       <c r="H5" s="3">
-        <f>E5-$B5</f>
+        <f t="shared" si="3"/>
         <v>-39943.03500922746</v>
       </c>
       <c r="I5" s="3">
-        <f>F5-$C5</f>
+        <f t="shared" si="4"/>
         <v>-9787.8374870478001</v>
       </c>
       <c r="J5" s="3">
-        <f>G5-$D5</f>
+        <f t="shared" si="5"/>
         <v>-2096.5039910896594</v>
       </c>
       <c r="K5">
@@ -2953,107 +2946,107 @@
         <v>292688</v>
       </c>
       <c r="Q5">
-        <f>K5</f>
+        <f t="shared" si="6"/>
         <v>5267</v>
       </c>
       <c r="R5">
-        <f>Q5+0.2*(V5-Q5)</f>
+        <f t="shared" si="7"/>
         <v>6197.8</v>
       </c>
       <c r="S5">
-        <f>Q5+0.4*(V5-Q5)</f>
+        <f t="shared" si="8"/>
         <v>7128.6</v>
       </c>
       <c r="T5">
-        <f>Q5+0.6*(V5-Q5)</f>
+        <f t="shared" si="9"/>
         <v>8059.4</v>
       </c>
       <c r="U5">
-        <f>Q5+0.8*(V5-Q5)</f>
+        <f t="shared" si="10"/>
         <v>8990.2000000000007</v>
       </c>
       <c r="V5">
-        <f>L5</f>
+        <f t="shared" si="11"/>
         <v>9921</v>
       </c>
       <c r="W5">
-        <f>V5+0.2*(AA5-V5)</f>
+        <f t="shared" si="12"/>
         <v>11750.6</v>
       </c>
       <c r="X5">
-        <f>V5+0.4*(AA5-V5)</f>
+        <f t="shared" si="13"/>
         <v>13580.2</v>
       </c>
       <c r="Y5">
-        <f>V5+0.6*(AA5-V5)</f>
+        <f t="shared" si="14"/>
         <v>15409.8</v>
       </c>
       <c r="Z5">
-        <f>V5+0.8*(AA5-V5)</f>
+        <f t="shared" si="15"/>
         <v>17239.400000000001</v>
       </c>
       <c r="AA5">
-        <f>M5</f>
+        <f t="shared" si="16"/>
         <v>19069</v>
       </c>
       <c r="AB5">
-        <f>AA5+0.2*(AF5-AA5)</f>
+        <f t="shared" si="17"/>
         <v>24202.2</v>
       </c>
       <c r="AC5">
-        <f>AA5+0.4*(AF5-AA5)</f>
+        <f t="shared" si="18"/>
         <v>29335.4</v>
       </c>
       <c r="AD5">
-        <f>AA5+0.6*(AF5-AA5)</f>
+        <f t="shared" si="19"/>
         <v>34468.6</v>
       </c>
       <c r="AE5">
-        <f>AA5+0.8*(AF5-AA5)</f>
+        <f t="shared" si="20"/>
         <v>39601.800000000003</v>
       </c>
       <c r="AF5">
-        <f>N5</f>
+        <f t="shared" si="21"/>
         <v>44735</v>
       </c>
       <c r="AG5">
-        <f>AF5+0.2*(AK5-AF5)</f>
+        <f t="shared" si="22"/>
         <v>57471.4</v>
       </c>
       <c r="AH5">
-        <f>AF5+0.4*(AK5-AF5)</f>
+        <f t="shared" si="23"/>
         <v>70207.8</v>
       </c>
       <c r="AI5">
-        <f>AF5+0.6*(AK5-AF5)</f>
+        <f t="shared" si="24"/>
         <v>82944.2</v>
       </c>
       <c r="AJ5">
-        <f>AF5+0.8*(AK5-AF5)</f>
+        <f t="shared" si="25"/>
         <v>95680.6</v>
       </c>
       <c r="AK5">
-        <f>O5</f>
+        <f t="shared" si="26"/>
         <v>108417</v>
       </c>
       <c r="AL5">
-        <f>AK5+0.2*(AP5-AK5)</f>
+        <f t="shared" si="27"/>
         <v>145271.20000000001</v>
       </c>
       <c r="AM5">
-        <f>AK5+0.4*(AP5-AK5)</f>
+        <f t="shared" si="28"/>
         <v>182125.40000000002</v>
       </c>
       <c r="AN5">
-        <f>AK5+0.6*(AP5-AK5)</f>
+        <f t="shared" si="29"/>
         <v>218979.59999999998</v>
       </c>
       <c r="AO5">
-        <f>AK5+0.8*(AP5-AK5)</f>
+        <f t="shared" si="30"/>
         <v>255833.80000000002</v>
       </c>
       <c r="AP5">
-        <f>P5</f>
+        <f t="shared" si="31"/>
         <v>292688</v>
       </c>
     </row>
@@ -3062,15 +3055,15 @@
         <v>20</v>
       </c>
       <c r="B6" s="3">
-        <f>E$4</f>
+        <f t="shared" si="0"/>
         <v>709776.91212891659</v>
       </c>
       <c r="C6" s="3">
-        <f>F$4</f>
+        <f t="shared" si="1"/>
         <v>219041.54431546232</v>
       </c>
       <c r="D6" s="3">
-        <f>G$4</f>
+        <f t="shared" si="2"/>
         <v>79692.853169511349</v>
       </c>
       <c r="E6" s="3">
@@ -3086,15 +3079,15 @@
         <v>76722.386938542259</v>
       </c>
       <c r="H6" s="3">
-        <f>E6-$B6</f>
+        <f t="shared" si="3"/>
         <v>-38345.769465351477</v>
       </c>
       <c r="I6" s="3">
-        <f>F6-$C6</f>
+        <f t="shared" si="4"/>
         <v>-10466.963344462827</v>
       </c>
       <c r="J6" s="3">
-        <f>G6-$D6</f>
+        <f t="shared" si="5"/>
         <v>-2970.4662309690902</v>
       </c>
       <c r="K6">
@@ -3116,107 +3109,107 @@
         <v>297418</v>
       </c>
       <c r="Q6">
-        <f>K6</f>
+        <f t="shared" si="6"/>
         <v>4818</v>
       </c>
       <c r="R6">
-        <f>Q6+0.2*(V6-Q6)</f>
+        <f t="shared" si="7"/>
         <v>5859.6</v>
       </c>
       <c r="S6">
-        <f>Q6+0.4*(V6-Q6)</f>
+        <f t="shared" si="8"/>
         <v>6901.2000000000007</v>
       </c>
       <c r="T6">
-        <f>Q6+0.6*(V6-Q6)</f>
+        <f t="shared" si="9"/>
         <v>7942.7999999999993</v>
       </c>
       <c r="U6">
-        <f>Q6+0.8*(V6-Q6)</f>
+        <f t="shared" si="10"/>
         <v>8984.4000000000015</v>
       </c>
       <c r="V6">
-        <f>L6</f>
+        <f t="shared" si="11"/>
         <v>10026</v>
       </c>
       <c r="W6">
-        <f>V6+0.2*(AA6-V6)</f>
+        <f t="shared" si="12"/>
         <v>11789.8</v>
       </c>
       <c r="X6">
-        <f>V6+0.4*(AA6-V6)</f>
+        <f t="shared" si="13"/>
         <v>13553.6</v>
       </c>
       <c r="Y6">
-        <f>V6+0.6*(AA6-V6)</f>
+        <f t="shared" si="14"/>
         <v>15317.4</v>
       </c>
       <c r="Z6">
-        <f>V6+0.8*(AA6-V6)</f>
+        <f t="shared" si="15"/>
         <v>17081.2</v>
       </c>
       <c r="AA6">
-        <f>M6</f>
+        <f t="shared" si="16"/>
         <v>18845</v>
       </c>
       <c r="AB6">
-        <f>AA6+0.2*(AF6-AA6)</f>
+        <f t="shared" si="17"/>
         <v>23904.2</v>
       </c>
       <c r="AC6">
-        <f>AA6+0.4*(AF6-AA6)</f>
+        <f t="shared" si="18"/>
         <v>28963.4</v>
       </c>
       <c r="AD6">
-        <f>AA6+0.6*(AF6-AA6)</f>
+        <f t="shared" si="19"/>
         <v>34022.6</v>
       </c>
       <c r="AE6">
-        <f>AA6+0.8*(AF6-AA6)</f>
+        <f t="shared" si="20"/>
         <v>39081.800000000003</v>
       </c>
       <c r="AF6">
-        <f>N6</f>
+        <f t="shared" si="21"/>
         <v>44141</v>
       </c>
       <c r="AG6">
-        <f>AF6+0.2*(AK6-AF6)</f>
+        <f t="shared" si="22"/>
         <v>57014.6</v>
       </c>
       <c r="AH6">
-        <f>AF6+0.4*(AK6-AF6)</f>
+        <f t="shared" si="23"/>
         <v>69888.2</v>
       </c>
       <c r="AI6">
-        <f>AF6+0.6*(AK6-AF6)</f>
+        <f t="shared" si="24"/>
         <v>82761.799999999988</v>
       </c>
       <c r="AJ6">
-        <f>AF6+0.8*(AK6-AF6)</f>
+        <f t="shared" si="25"/>
         <v>95635.4</v>
       </c>
       <c r="AK6">
-        <f>O6</f>
+        <f t="shared" si="26"/>
         <v>108509</v>
       </c>
       <c r="AL6">
-        <f>AK6+0.2*(AP6-AK6)</f>
+        <f t="shared" si="27"/>
         <v>146290.79999999999</v>
       </c>
       <c r="AM6">
-        <f>AK6+0.4*(AP6-AK6)</f>
+        <f t="shared" si="28"/>
         <v>184072.6</v>
       </c>
       <c r="AN6">
-        <f>AK6+0.6*(AP6-AK6)</f>
+        <f t="shared" si="29"/>
         <v>221854.4</v>
       </c>
       <c r="AO6">
-        <f>AK6+0.8*(AP6-AK6)</f>
+        <f t="shared" si="30"/>
         <v>259636.2</v>
       </c>
       <c r="AP6">
-        <f>P6</f>
+        <f t="shared" si="31"/>
         <v>297418</v>
       </c>
     </row>
@@ -3225,15 +3218,15 @@
         <v>21</v>
       </c>
       <c r="B7" s="3">
-        <f>E$4</f>
+        <f t="shared" si="0"/>
         <v>709776.91212891659</v>
       </c>
       <c r="C7" s="3">
-        <f>F$4</f>
+        <f t="shared" si="1"/>
         <v>219041.54431546232</v>
       </c>
       <c r="D7" s="3">
-        <f>G$4</f>
+        <f t="shared" si="2"/>
         <v>79692.853169511349</v>
       </c>
       <c r="E7" s="3">
@@ -3249,15 +3242,15 @@
         <v>75916.94206260475</v>
       </c>
       <c r="H7" s="3">
-        <f>E7-$B7</f>
+        <f t="shared" si="3"/>
         <v>-49695.559744336875</v>
       </c>
       <c r="I7" s="3">
-        <f>F7-$C7</f>
+        <f t="shared" si="4"/>
         <v>-13629.288795838074</v>
       </c>
       <c r="J7" s="3">
-        <f>G7-$D7</f>
+        <f t="shared" si="5"/>
         <v>-3775.9111069065984</v>
       </c>
       <c r="K7">
@@ -3279,107 +3272,107 @@
         <v>293947</v>
       </c>
       <c r="Q7">
-        <f>K7</f>
+        <f t="shared" si="6"/>
         <v>4760</v>
       </c>
       <c r="R7">
-        <f>Q7+0.2*(V7-Q7)</f>
+        <f t="shared" si="7"/>
         <v>5868.6</v>
       </c>
       <c r="S7">
-        <f>Q7+0.4*(V7-Q7)</f>
+        <f t="shared" si="8"/>
         <v>6977.2000000000007</v>
       </c>
       <c r="T7">
-        <f>Q7+0.6*(V7-Q7)</f>
+        <f t="shared" si="9"/>
         <v>8085.7999999999993</v>
       </c>
       <c r="U7">
-        <f>Q7+0.8*(V7-Q7)</f>
+        <f t="shared" si="10"/>
         <v>9194.4000000000015</v>
       </c>
       <c r="V7">
-        <f>L7</f>
+        <f t="shared" si="11"/>
         <v>10303</v>
       </c>
       <c r="W7">
-        <f>V7+0.2*(AA7-V7)</f>
+        <f t="shared" si="12"/>
         <v>11918.6</v>
       </c>
       <c r="X7">
-        <f>V7+0.4*(AA7-V7)</f>
+        <f t="shared" si="13"/>
         <v>13534.2</v>
       </c>
       <c r="Y7">
-        <f>V7+0.6*(AA7-V7)</f>
+        <f t="shared" si="14"/>
         <v>15149.8</v>
       </c>
       <c r="Z7">
-        <f>V7+0.8*(AA7-V7)</f>
+        <f t="shared" si="15"/>
         <v>16765.400000000001</v>
       </c>
       <c r="AA7">
-        <f>M7</f>
+        <f t="shared" si="16"/>
         <v>18381</v>
       </c>
       <c r="AB7">
-        <f>AA7+0.2*(AF7-AA7)</f>
+        <f t="shared" si="17"/>
         <v>23201.200000000001</v>
       </c>
       <c r="AC7">
-        <f>AA7+0.4*(AF7-AA7)</f>
+        <f t="shared" si="18"/>
         <v>28021.4</v>
       </c>
       <c r="AD7">
-        <f>AA7+0.6*(AF7-AA7)</f>
+        <f t="shared" si="19"/>
         <v>32841.599999999999</v>
       </c>
       <c r="AE7">
-        <f>AA7+0.8*(AF7-AA7)</f>
+        <f t="shared" si="20"/>
         <v>37661.800000000003</v>
       </c>
       <c r="AF7">
-        <f>N7</f>
+        <f t="shared" si="21"/>
         <v>42482</v>
       </c>
       <c r="AG7">
-        <f>AF7+0.2*(AK7-AF7)</f>
+        <f t="shared" si="22"/>
         <v>55252.6</v>
       </c>
       <c r="AH7">
-        <f>AF7+0.4*(AK7-AF7)</f>
+        <f t="shared" si="23"/>
         <v>68023.199999999997</v>
       </c>
       <c r="AI7">
-        <f>AF7+0.6*(AK7-AF7)</f>
+        <f t="shared" si="24"/>
         <v>80793.799999999988</v>
       </c>
       <c r="AJ7">
-        <f>AF7+0.8*(AK7-AF7)</f>
+        <f t="shared" si="25"/>
         <v>93564.4</v>
       </c>
       <c r="AK7">
-        <f>O7</f>
+        <f t="shared" si="26"/>
         <v>106335</v>
       </c>
       <c r="AL7">
-        <f>AK7+0.2*(AP7-AK7)</f>
+        <f t="shared" si="27"/>
         <v>143857.4</v>
       </c>
       <c r="AM7">
-        <f>AK7+0.4*(AP7-AK7)</f>
+        <f t="shared" si="28"/>
         <v>181379.8</v>
       </c>
       <c r="AN7">
-        <f>AK7+0.6*(AP7-AK7)</f>
+        <f t="shared" si="29"/>
         <v>218902.2</v>
       </c>
       <c r="AO7">
-        <f>AK7+0.8*(AP7-AK7)</f>
+        <f t="shared" si="30"/>
         <v>256424.6</v>
       </c>
       <c r="AP7">
-        <f>P7</f>
+        <f t="shared" si="31"/>
         <v>293947</v>
       </c>
     </row>
@@ -3388,15 +3381,15 @@
         <v>22</v>
       </c>
       <c r="B8" s="3">
-        <f>E$4</f>
+        <f t="shared" si="0"/>
         <v>709776.91212891659</v>
       </c>
       <c r="C8" s="3">
-        <f>F$4</f>
+        <f t="shared" si="1"/>
         <v>219041.54431546232</v>
       </c>
       <c r="D8" s="3">
-        <f>G$4</f>
+        <f t="shared" si="2"/>
         <v>79692.853169511349</v>
       </c>
       <c r="E8" s="3">
@@ -3412,15 +3405,15 @@
         <v>72371.19339976694</v>
       </c>
       <c r="H8" s="3">
-        <f>E8-$B8</f>
+        <f t="shared" si="3"/>
         <v>-99383.500741741736</v>
       </c>
       <c r="I8" s="3">
-        <f>F8-$C8</f>
+        <f t="shared" si="4"/>
         <v>-27200.233395238378</v>
       </c>
       <c r="J8" s="3">
-        <f>G8-$D8</f>
+        <f t="shared" si="5"/>
         <v>-7321.6597697444085</v>
       </c>
       <c r="K8">
@@ -3442,107 +3435,107 @@
         <v>273786</v>
       </c>
       <c r="Q8">
-        <f>K8</f>
+        <f t="shared" si="6"/>
         <v>4760</v>
       </c>
       <c r="R8">
-        <f>Q8+0.2*(V8-Q8)</f>
+        <f t="shared" si="7"/>
         <v>5963.6</v>
       </c>
       <c r="S8">
-        <f>Q8+0.4*(V8-Q8)</f>
+        <f t="shared" si="8"/>
         <v>7167.2000000000007</v>
       </c>
       <c r="T8">
-        <f>Q8+0.6*(V8-Q8)</f>
+        <f t="shared" si="9"/>
         <v>8370.7999999999993</v>
       </c>
       <c r="U8">
-        <f>Q8+0.8*(V8-Q8)</f>
+        <f t="shared" si="10"/>
         <v>9574.4000000000015</v>
       </c>
       <c r="V8">
-        <f>L8</f>
+        <f t="shared" si="11"/>
         <v>10778</v>
       </c>
       <c r="W8">
-        <f>V8+0.2*(AA8-V8)</f>
+        <f t="shared" si="12"/>
         <v>12000.4</v>
       </c>
       <c r="X8">
-        <f>V8+0.4*(AA8-V8)</f>
+        <f t="shared" si="13"/>
         <v>13222.8</v>
       </c>
       <c r="Y8">
-        <f>V8+0.6*(AA8-V8)</f>
+        <f t="shared" si="14"/>
         <v>14445.2</v>
       </c>
       <c r="Z8">
-        <f>V8+0.8*(AA8-V8)</f>
+        <f t="shared" si="15"/>
         <v>15667.6</v>
       </c>
       <c r="AA8">
-        <f>M8</f>
+        <f t="shared" si="16"/>
         <v>16890</v>
       </c>
       <c r="AB8">
-        <f>AA8+0.2*(AF8-AA8)</f>
+        <f t="shared" si="17"/>
         <v>20913</v>
       </c>
       <c r="AC8">
-        <f>AA8+0.4*(AF8-AA8)</f>
+        <f t="shared" si="18"/>
         <v>24936</v>
       </c>
       <c r="AD8">
-        <f>AA8+0.6*(AF8-AA8)</f>
+        <f t="shared" si="19"/>
         <v>28959</v>
       </c>
       <c r="AE8">
-        <f>AA8+0.8*(AF8-AA8)</f>
+        <f t="shared" si="20"/>
         <v>32982</v>
       </c>
       <c r="AF8">
-        <f>N8</f>
+        <f t="shared" si="21"/>
         <v>37005</v>
       </c>
       <c r="AG8">
-        <f>AF8+0.2*(AK8-AF8)</f>
+        <f t="shared" si="22"/>
         <v>49063.6</v>
       </c>
       <c r="AH8">
-        <f>AF8+0.4*(AK8-AF8)</f>
+        <f t="shared" si="23"/>
         <v>61122.2</v>
       </c>
       <c r="AI8">
-        <f>AF8+0.6*(AK8-AF8)</f>
+        <f t="shared" si="24"/>
         <v>73180.799999999988</v>
       </c>
       <c r="AJ8">
-        <f>AF8+0.8*(AK8-AF8)</f>
+        <f t="shared" si="25"/>
         <v>85239.4</v>
       </c>
       <c r="AK8">
-        <f>O8</f>
+        <f t="shared" si="26"/>
         <v>97298</v>
       </c>
       <c r="AL8">
-        <f>AK8+0.2*(AP8-AK8)</f>
+        <f t="shared" si="27"/>
         <v>132595.6</v>
       </c>
       <c r="AM8">
-        <f>AK8+0.4*(AP8-AK8)</f>
+        <f t="shared" si="28"/>
         <v>167893.2</v>
       </c>
       <c r="AN8">
-        <f>AK8+0.6*(AP8-AK8)</f>
+        <f t="shared" si="29"/>
         <v>203190.8</v>
       </c>
       <c r="AO8">
-        <f>AK8+0.8*(AP8-AK8)</f>
+        <f t="shared" si="30"/>
         <v>238488.4</v>
       </c>
       <c r="AP8">
-        <f>P8</f>
+        <f t="shared" si="31"/>
         <v>273786</v>
       </c>
     </row>
@@ -3551,15 +3544,15 @@
         <v>23</v>
       </c>
       <c r="B9" s="3">
-        <f>E$4</f>
+        <f t="shared" si="0"/>
         <v>709776.91212891659</v>
       </c>
       <c r="C9" s="3">
-        <f>F$4</f>
+        <f t="shared" si="1"/>
         <v>219041.54431546232</v>
       </c>
       <c r="D9" s="3">
-        <f>G$4</f>
+        <f t="shared" si="2"/>
         <v>79692.853169511349</v>
       </c>
       <c r="E9" s="3">
@@ -3575,15 +3568,15 @@
         <v>75499.851497461423</v>
       </c>
       <c r="H9" s="3">
-        <f>E9-$B9</f>
+        <f t="shared" si="3"/>
         <v>-55983.648403950618</v>
       </c>
       <c r="I9" s="3">
-        <f>F9-$C9</f>
+        <f t="shared" si="4"/>
         <v>-15270.056494475401</v>
       </c>
       <c r="J9" s="3">
-        <f>G9-$D9</f>
+        <f t="shared" si="5"/>
         <v>-4193.0016720499261</v>
       </c>
       <c r="K9">
@@ -3605,107 +3598,107 @@
         <v>289957</v>
       </c>
       <c r="Q9">
-        <f>K9</f>
+        <f t="shared" si="6"/>
         <v>4983</v>
       </c>
       <c r="R9">
-        <f>Q9+0.2*(V9-Q9)</f>
+        <f t="shared" si="7"/>
         <v>5988.8</v>
       </c>
       <c r="S9">
-        <f>Q9+0.4*(V9-Q9)</f>
+        <f t="shared" si="8"/>
         <v>6994.6</v>
       </c>
       <c r="T9">
-        <f>Q9+0.6*(V9-Q9)</f>
+        <f t="shared" si="9"/>
         <v>8000.4</v>
       </c>
       <c r="U9">
-        <f>Q9+0.8*(V9-Q9)</f>
+        <f t="shared" si="10"/>
         <v>9006.2000000000007</v>
       </c>
       <c r="V9">
-        <f>L9</f>
+        <f t="shared" si="11"/>
         <v>10012</v>
       </c>
       <c r="W9">
-        <f>V9+0.2*(AA9-V9)</f>
+        <f t="shared" si="12"/>
         <v>11658.8</v>
       </c>
       <c r="X9">
-        <f>V9+0.4*(AA9-V9)</f>
+        <f t="shared" si="13"/>
         <v>13305.6</v>
       </c>
       <c r="Y9">
-        <f>V9+0.6*(AA9-V9)</f>
+        <f t="shared" si="14"/>
         <v>14952.4</v>
       </c>
       <c r="Z9">
-        <f>V9+0.8*(AA9-V9)</f>
+        <f t="shared" si="15"/>
         <v>16599.2</v>
       </c>
       <c r="AA9">
-        <f>M9</f>
+        <f t="shared" si="16"/>
         <v>18246</v>
       </c>
       <c r="AB9">
-        <f>AA9+0.2*(AF9-AA9)</f>
+        <f t="shared" si="17"/>
         <v>23100.6</v>
       </c>
       <c r="AC9">
-        <f>AA9+0.4*(AF9-AA9)</f>
+        <f t="shared" si="18"/>
         <v>27955.200000000001</v>
       </c>
       <c r="AD9">
-        <f>AA9+0.6*(AF9-AA9)</f>
+        <f t="shared" si="19"/>
         <v>32809.800000000003</v>
       </c>
       <c r="AE9">
-        <f>AA9+0.8*(AF9-AA9)</f>
+        <f t="shared" si="20"/>
         <v>37664.400000000001</v>
       </c>
       <c r="AF9">
-        <f>N9</f>
+        <f t="shared" si="21"/>
         <v>42519</v>
       </c>
       <c r="AG9">
-        <f>AF9+0.2*(AK9-AF9)</f>
+        <f t="shared" si="22"/>
         <v>55073.2</v>
       </c>
       <c r="AH9">
-        <f>AF9+0.4*(AK9-AF9)</f>
+        <f t="shared" si="23"/>
         <v>67627.399999999994</v>
       </c>
       <c r="AI9">
-        <f>AF9+0.6*(AK9-AF9)</f>
+        <f t="shared" si="24"/>
         <v>80181.600000000006</v>
       </c>
       <c r="AJ9">
-        <f>AF9+0.8*(AK9-AF9)</f>
+        <f t="shared" si="25"/>
         <v>92735.8</v>
       </c>
       <c r="AK9">
-        <f>O9</f>
+        <f t="shared" si="26"/>
         <v>105290</v>
       </c>
       <c r="AL9">
-        <f>AK9+0.2*(AP9-AK9)</f>
+        <f t="shared" si="27"/>
         <v>142223.4</v>
       </c>
       <c r="AM9">
-        <f>AK9+0.4*(AP9-AK9)</f>
+        <f t="shared" si="28"/>
         <v>179156.8</v>
       </c>
       <c r="AN9">
-        <f>AK9+0.6*(AP9-AK9)</f>
+        <f t="shared" si="29"/>
         <v>216090.2</v>
       </c>
       <c r="AO9">
-        <f>AK9+0.8*(AP9-AK9)</f>
+        <f t="shared" si="30"/>
         <v>253023.6</v>
       </c>
       <c r="AP9">
-        <f>P9</f>
+        <f t="shared" si="31"/>
         <v>289957</v>
       </c>
     </row>
@@ -3714,15 +3707,15 @@
         <v>24</v>
       </c>
       <c r="B10" s="3">
-        <f>E$4</f>
+        <f t="shared" si="0"/>
         <v>709776.91212891659</v>
       </c>
       <c r="C10" s="3">
-        <f>F$4</f>
+        <f t="shared" si="1"/>
         <v>219041.54431546232</v>
       </c>
       <c r="D10" s="3">
-        <f>G$4</f>
+        <f t="shared" si="2"/>
         <v>79692.853169511349</v>
       </c>
       <c r="E10" s="3">
@@ -3738,15 +3731,15 @@
         <v>72905.393296508759</v>
       </c>
       <c r="H10" s="3">
-        <f>E10-$B10</f>
+        <f t="shared" si="3"/>
         <v>-27865.668002608116</v>
       </c>
       <c r="I10" s="3">
-        <f>F10-$C10</f>
+        <f t="shared" si="4"/>
         <v>-12631.054123761802</v>
       </c>
       <c r="J10" s="3">
-        <f>G10-$D10</f>
+        <f t="shared" si="5"/>
         <v>-6787.45987300259</v>
       </c>
       <c r="K10">
@@ -3768,107 +3761,107 @@
         <v>308210</v>
       </c>
       <c r="Q10">
-        <f>K10</f>
+        <f t="shared" si="6"/>
         <v>4760</v>
       </c>
       <c r="R10">
-        <f>Q10+0.2*(V10-Q10)</f>
+        <f t="shared" si="7"/>
         <v>5307.4</v>
       </c>
       <c r="S10">
-        <f>Q10+0.4*(V10-Q10)</f>
+        <f t="shared" si="8"/>
         <v>5854.8</v>
       </c>
       <c r="T10">
-        <f>Q10+0.6*(V10-Q10)</f>
+        <f t="shared" si="9"/>
         <v>6402.2</v>
       </c>
       <c r="U10">
-        <f>Q10+0.8*(V10-Q10)</f>
+        <f t="shared" si="10"/>
         <v>6949.6</v>
       </c>
       <c r="V10">
-        <f>L10</f>
+        <f t="shared" si="11"/>
         <v>7497</v>
       </c>
       <c r="W10">
-        <f>V10+0.2*(AA10-V10)</f>
+        <f t="shared" si="12"/>
         <v>9569.2000000000007</v>
       </c>
       <c r="X10">
-        <f>V10+0.4*(AA10-V10)</f>
+        <f t="shared" si="13"/>
         <v>11641.400000000001</v>
       </c>
       <c r="Y10">
-        <f>V10+0.6*(AA10-V10)</f>
+        <f t="shared" si="14"/>
         <v>13713.599999999999</v>
       </c>
       <c r="Z10">
-        <f>V10+0.8*(AA10-V10)</f>
+        <f t="shared" si="15"/>
         <v>15785.800000000001</v>
       </c>
       <c r="AA10">
-        <f>M10</f>
+        <f t="shared" si="16"/>
         <v>17858</v>
       </c>
       <c r="AB10">
-        <f>AA10+0.2*(AF10-AA10)</f>
+        <f t="shared" si="17"/>
         <v>23551.4</v>
       </c>
       <c r="AC10">
-        <f>AA10+0.4*(AF10-AA10)</f>
+        <f t="shared" si="18"/>
         <v>29244.800000000003</v>
       </c>
       <c r="AD10">
-        <f>AA10+0.6*(AF10-AA10)</f>
+        <f t="shared" si="19"/>
         <v>34938.199999999997</v>
       </c>
       <c r="AE10">
-        <f>AA10+0.8*(AF10-AA10)</f>
+        <f t="shared" si="20"/>
         <v>40631.600000000006</v>
       </c>
       <c r="AF10">
-        <f>N10</f>
+        <f t="shared" si="21"/>
         <v>46325</v>
       </c>
       <c r="AG10">
-        <f>AF10+0.2*(AK10-AF10)</f>
+        <f t="shared" si="22"/>
         <v>59677.2</v>
       </c>
       <c r="AH10">
-        <f>AF10+0.4*(AK10-AF10)</f>
+        <f t="shared" si="23"/>
         <v>73029.399999999994</v>
       </c>
       <c r="AI10">
-        <f>AF10+0.6*(AK10-AF10)</f>
+        <f t="shared" si="24"/>
         <v>86381.6</v>
       </c>
       <c r="AJ10">
-        <f>AF10+0.8*(AK10-AF10)</f>
+        <f t="shared" si="25"/>
         <v>99733.8</v>
       </c>
       <c r="AK10">
-        <f>O10</f>
+        <f t="shared" si="26"/>
         <v>113086</v>
       </c>
       <c r="AL10">
-        <f>AK10+0.2*(AP10-AK10)</f>
+        <f t="shared" si="27"/>
         <v>152110.79999999999</v>
       </c>
       <c r="AM10">
-        <f>AK10+0.4*(AP10-AK10)</f>
+        <f t="shared" si="28"/>
         <v>191135.6</v>
       </c>
       <c r="AN10">
-        <f>AK10+0.6*(AP10-AK10)</f>
+        <f t="shared" si="29"/>
         <v>230160.4</v>
       </c>
       <c r="AO10">
-        <f>AK10+0.8*(AP10-AK10)</f>
+        <f t="shared" si="30"/>
         <v>269185.2</v>
       </c>
       <c r="AP10">
-        <f>P10</f>
+        <f t="shared" si="31"/>
         <v>308210</v>
       </c>
     </row>
@@ -3877,15 +3870,15 @@
         <v>25</v>
       </c>
       <c r="B11" s="3">
-        <f>E$4</f>
+        <f t="shared" si="0"/>
         <v>709776.91212891659</v>
       </c>
       <c r="C11" s="3">
-        <f>F$4</f>
+        <f t="shared" si="1"/>
         <v>219041.54431546232</v>
       </c>
       <c r="D11" s="3">
-        <f>G$4</f>
+        <f t="shared" si="2"/>
         <v>79692.853169511349</v>
       </c>
       <c r="E11" s="3">
@@ -3901,15 +3894,15 @@
         <v>96722.886654337548</v>
       </c>
       <c r="H11" s="3">
-        <f>E11-$B11</f>
+        <f t="shared" si="3"/>
         <v>24232.50337599928</v>
       </c>
       <c r="I11" s="3">
-        <f>F11-$C11</f>
+        <f t="shared" si="4"/>
         <v>22181.596266089822</v>
       </c>
       <c r="J11" s="3">
-        <f>G11-$D11</f>
+        <f t="shared" si="5"/>
         <v>17030.033484826199</v>
       </c>
       <c r="K11">
@@ -3931,107 +3924,107 @@
         <v>308253</v>
       </c>
       <c r="Q11">
-        <f>K11</f>
+        <f t="shared" si="6"/>
         <v>8076</v>
       </c>
       <c r="R11">
-        <f>Q11+0.2*(V11-Q11)</f>
+        <f t="shared" si="7"/>
         <v>9471.2000000000007</v>
       </c>
       <c r="S11">
-        <f>Q11+0.4*(V11-Q11)</f>
+        <f t="shared" si="8"/>
         <v>10866.4</v>
       </c>
       <c r="T11">
-        <f>Q11+0.6*(V11-Q11)</f>
+        <f t="shared" si="9"/>
         <v>12261.599999999999</v>
       </c>
       <c r="U11">
-        <f>Q11+0.8*(V11-Q11)</f>
+        <f t="shared" si="10"/>
         <v>13656.8</v>
       </c>
       <c r="V11">
-        <f>L11</f>
+        <f t="shared" si="11"/>
         <v>15052</v>
       </c>
       <c r="W11">
-        <f>V11+0.2*(AA11-V11)</f>
+        <f t="shared" si="12"/>
         <v>16627.400000000001</v>
       </c>
       <c r="X11">
-        <f>V11+0.4*(AA11-V11)</f>
+        <f t="shared" si="13"/>
         <v>18202.8</v>
       </c>
       <c r="Y11">
-        <f>V11+0.6*(AA11-V11)</f>
+        <f t="shared" si="14"/>
         <v>19778.2</v>
       </c>
       <c r="Z11">
-        <f>V11+0.8*(AA11-V11)</f>
+        <f t="shared" si="15"/>
         <v>21353.599999999999</v>
       </c>
       <c r="AA11">
-        <f>M11</f>
+        <f t="shared" si="16"/>
         <v>22929</v>
       </c>
       <c r="AB11">
-        <f>AA11+0.2*(AF11-AA11)</f>
+        <f t="shared" si="17"/>
         <v>27603.8</v>
       </c>
       <c r="AC11">
-        <f>AA11+0.4*(AF11-AA11)</f>
+        <f t="shared" si="18"/>
         <v>32278.6</v>
       </c>
       <c r="AD11">
-        <f>AA11+0.6*(AF11-AA11)</f>
+        <f t="shared" si="19"/>
         <v>36953.4</v>
       </c>
       <c r="AE11">
-        <f>AA11+0.8*(AF11-AA11)</f>
+        <f t="shared" si="20"/>
         <v>41628.199999999997</v>
       </c>
       <c r="AF11">
-        <f>N11</f>
+        <f t="shared" si="21"/>
         <v>46303</v>
       </c>
       <c r="AG11">
-        <f>AF11+0.2*(AK11-AF11)</f>
+        <f t="shared" si="22"/>
         <v>59659.4</v>
       </c>
       <c r="AH11">
-        <f>AF11+0.4*(AK11-AF11)</f>
+        <f t="shared" si="23"/>
         <v>73015.8</v>
       </c>
       <c r="AI11">
-        <f>AF11+0.6*(AK11-AF11)</f>
+        <f t="shared" si="24"/>
         <v>86372.2</v>
       </c>
       <c r="AJ11">
-        <f>AF11+0.8*(AK11-AF11)</f>
+        <f t="shared" si="25"/>
         <v>99728.6</v>
       </c>
       <c r="AK11">
-        <f>O11</f>
+        <f t="shared" si="26"/>
         <v>113085</v>
       </c>
       <c r="AL11">
-        <f>AK11+0.2*(AP11-AK11)</f>
+        <f t="shared" si="27"/>
         <v>152118.6</v>
       </c>
       <c r="AM11">
-        <f>AK11+0.4*(AP11-AK11)</f>
+        <f t="shared" si="28"/>
         <v>191152.2</v>
       </c>
       <c r="AN11">
-        <f>AK11+0.6*(AP11-AK11)</f>
+        <f t="shared" si="29"/>
         <v>230185.8</v>
       </c>
       <c r="AO11">
-        <f>AK11+0.8*(AP11-AK11)</f>
+        <f t="shared" si="30"/>
         <v>269219.40000000002</v>
       </c>
       <c r="AP11">
-        <f>P11</f>
+        <f t="shared" si="31"/>
         <v>308253</v>
       </c>
     </row>
@@ -4040,15 +4033,15 @@
         <v>26</v>
       </c>
       <c r="B12" s="3">
-        <f>E$4</f>
+        <f t="shared" si="0"/>
         <v>709776.91212891659</v>
       </c>
       <c r="C12" s="3">
-        <f>F$4</f>
+        <f t="shared" si="1"/>
         <v>219041.54431546232</v>
       </c>
       <c r="D12" s="3">
-        <f>G$4</f>
+        <f t="shared" si="2"/>
         <v>79692.853169511349</v>
       </c>
       <c r="E12" s="3">
@@ -4064,15 +4057,15 @@
         <v>172113.39439421654</v>
       </c>
       <c r="H12" s="3">
-        <f>E12-$B12</f>
+        <f t="shared" si="3"/>
         <v>569096.86274592637</v>
       </c>
       <c r="I12" s="3">
-        <f>F12-$C12</f>
+        <f t="shared" si="4"/>
         <v>215061.28634846405</v>
       </c>
       <c r="J12" s="3">
-        <f>G12-$D12</f>
+        <f t="shared" si="5"/>
         <v>92420.541224705186</v>
       </c>
       <c r="K12">
@@ -4094,107 +4087,107 @@
         <v>427156</v>
       </c>
       <c r="Q12">
-        <f>K12</f>
+        <f t="shared" si="6"/>
         <v>4760</v>
       </c>
       <c r="R12">
-        <f>Q12+0.2*(V12-Q12)</f>
+        <f t="shared" si="7"/>
         <v>9872</v>
       </c>
       <c r="S12">
-        <f>Q12+0.4*(V12-Q12)</f>
+        <f t="shared" si="8"/>
         <v>14984</v>
       </c>
       <c r="T12">
-        <f>Q12+0.6*(V12-Q12)</f>
+        <f t="shared" si="9"/>
         <v>20096</v>
       </c>
       <c r="U12">
-        <f>Q12+0.8*(V12-Q12)</f>
+        <f t="shared" si="10"/>
         <v>25208</v>
       </c>
       <c r="V12">
-        <f>L12</f>
+        <f t="shared" si="11"/>
         <v>30320</v>
       </c>
       <c r="W12">
-        <f>V12+0.2*(AA12-V12)</f>
+        <f t="shared" si="12"/>
         <v>35504</v>
       </c>
       <c r="X12">
-        <f>V12+0.4*(AA12-V12)</f>
+        <f t="shared" si="13"/>
         <v>40688</v>
       </c>
       <c r="Y12">
-        <f>V12+0.6*(AA12-V12)</f>
+        <f t="shared" si="14"/>
         <v>45872</v>
       </c>
       <c r="Z12">
-        <f>V12+0.8*(AA12-V12)</f>
+        <f t="shared" si="15"/>
         <v>51056</v>
       </c>
       <c r="AA12">
-        <f>M12</f>
+        <f t="shared" si="16"/>
         <v>56240</v>
       </c>
       <c r="AB12">
-        <f>AA12+0.2*(AF12-AA12)</f>
+        <f t="shared" si="17"/>
         <v>65556.600000000006</v>
       </c>
       <c r="AC12">
-        <f>AA12+0.4*(AF12-AA12)</f>
+        <f t="shared" si="18"/>
         <v>74873.2</v>
       </c>
       <c r="AD12">
-        <f>AA12+0.6*(AF12-AA12)</f>
+        <f t="shared" si="19"/>
         <v>84189.8</v>
       </c>
       <c r="AE12">
-        <f>AA12+0.8*(AF12-AA12)</f>
+        <f t="shared" si="20"/>
         <v>93506.4</v>
       </c>
       <c r="AF12">
-        <f>N12</f>
+        <f t="shared" si="21"/>
         <v>102823</v>
       </c>
       <c r="AG12">
-        <f>AF12+0.2*(AK12-AF12)</f>
+        <f t="shared" si="22"/>
         <v>122768.4</v>
       </c>
       <c r="AH12">
-        <f>AF12+0.4*(AK12-AF12)</f>
+        <f t="shared" si="23"/>
         <v>142713.79999999999</v>
       </c>
       <c r="AI12">
-        <f>AF12+0.6*(AK12-AF12)</f>
+        <f t="shared" si="24"/>
         <v>162659.20000000001</v>
       </c>
       <c r="AJ12">
-        <f>AF12+0.8*(AK12-AF12)</f>
+        <f t="shared" si="25"/>
         <v>182604.6</v>
       </c>
       <c r="AK12">
-        <f>O12</f>
+        <f t="shared" si="26"/>
         <v>202550</v>
       </c>
       <c r="AL12">
-        <f>AK12+0.2*(AP12-AK12)</f>
+        <f t="shared" si="27"/>
         <v>247471.2</v>
       </c>
       <c r="AM12">
-        <f>AK12+0.4*(AP12-AK12)</f>
+        <f t="shared" si="28"/>
         <v>292392.40000000002</v>
       </c>
       <c r="AN12">
-        <f>AK12+0.6*(AP12-AK12)</f>
+        <f t="shared" si="29"/>
         <v>337313.6</v>
       </c>
       <c r="AO12">
-        <f>AK12+0.8*(AP12-AK12)</f>
+        <f t="shared" si="30"/>
         <v>382234.80000000005</v>
       </c>
       <c r="AP12">
-        <f>P12</f>
+        <f t="shared" si="31"/>
         <v>427156</v>
       </c>
     </row>
@@ -4203,15 +4196,15 @@
         <v>27</v>
       </c>
       <c r="B13" s="3">
-        <f>E$4</f>
+        <f t="shared" si="0"/>
         <v>709776.91212891659</v>
       </c>
       <c r="C13" s="3">
-        <f>F$4</f>
+        <f t="shared" si="1"/>
         <v>219041.54431546232</v>
       </c>
       <c r="D13" s="3">
-        <f>G$4</f>
+        <f t="shared" si="2"/>
         <v>79692.853169511349</v>
       </c>
       <c r="E13" s="3">
@@ -4227,15 +4220,15 @@
         <v>83232.990658578477</v>
       </c>
       <c r="H13" s="3">
-        <f>E13-$B13</f>
+        <f t="shared" si="3"/>
         <v>-720.7966358284466</v>
       </c>
       <c r="I13" s="3">
-        <f>F13-$C13</f>
+        <f t="shared" si="4"/>
         <v>4045.3140468056954</v>
       </c>
       <c r="J13" s="3">
-        <f>G13-$D13</f>
+        <f t="shared" si="5"/>
         <v>3540.1374890671286</v>
       </c>
       <c r="K13">
@@ -4257,107 +4250,107 @@
         <v>308117</v>
       </c>
       <c r="Q13">
-        <f>K13</f>
+        <f t="shared" si="6"/>
         <v>4778</v>
       </c>
       <c r="R13">
-        <f>Q13+0.2*(V13-Q13)</f>
+        <f t="shared" si="7"/>
         <v>6153.4</v>
       </c>
       <c r="S13">
-        <f>Q13+0.4*(V13-Q13)</f>
+        <f t="shared" si="8"/>
         <v>7528.8</v>
       </c>
       <c r="T13">
-        <f>Q13+0.6*(V13-Q13)</f>
+        <f t="shared" si="9"/>
         <v>8904.2000000000007</v>
       </c>
       <c r="U13">
-        <f>Q13+0.8*(V13-Q13)</f>
+        <f t="shared" si="10"/>
         <v>10279.6</v>
       </c>
       <c r="V13">
-        <f>L13</f>
+        <f t="shared" si="11"/>
         <v>11655</v>
       </c>
       <c r="W13">
-        <f>V13+0.2*(AA13-V13)</f>
+        <f t="shared" si="12"/>
         <v>13693.4</v>
       </c>
       <c r="X13">
-        <f>V13+0.4*(AA13-V13)</f>
+        <f t="shared" si="13"/>
         <v>15731.8</v>
       </c>
       <c r="Y13">
-        <f>V13+0.6*(AA13-V13)</f>
+        <f t="shared" si="14"/>
         <v>17770.2</v>
       </c>
       <c r="Z13">
-        <f>V13+0.8*(AA13-V13)</f>
+        <f t="shared" si="15"/>
         <v>19808.599999999999</v>
       </c>
       <c r="AA13">
-        <f>M13</f>
+        <f t="shared" si="16"/>
         <v>21847</v>
       </c>
       <c r="AB13">
-        <f>AA13+0.2*(AF13-AA13)</f>
+        <f t="shared" si="17"/>
         <v>26739</v>
       </c>
       <c r="AC13">
-        <f>AA13+0.4*(AF13-AA13)</f>
+        <f t="shared" si="18"/>
         <v>31631</v>
       </c>
       <c r="AD13">
-        <f>AA13+0.6*(AF13-AA13)</f>
+        <f t="shared" si="19"/>
         <v>36523</v>
       </c>
       <c r="AE13">
-        <f>AA13+0.8*(AF13-AA13)</f>
+        <f t="shared" si="20"/>
         <v>41415</v>
       </c>
       <c r="AF13">
-        <f>N13</f>
+        <f t="shared" si="21"/>
         <v>46307</v>
       </c>
       <c r="AG13">
-        <f>AF13+0.2*(AK13-AF13)</f>
+        <f t="shared" si="22"/>
         <v>59653.599999999999</v>
       </c>
       <c r="AH13">
-        <f>AF13+0.4*(AK13-AF13)</f>
+        <f t="shared" si="23"/>
         <v>73000.2</v>
       </c>
       <c r="AI13">
-        <f>AF13+0.6*(AK13-AF13)</f>
+        <f t="shared" si="24"/>
         <v>86346.799999999988</v>
       </c>
       <c r="AJ13">
-        <f>AF13+0.8*(AK13-AF13)</f>
+        <f t="shared" si="25"/>
         <v>99693.4</v>
       </c>
       <c r="AK13">
-        <f>O13</f>
+        <f t="shared" si="26"/>
         <v>113040</v>
       </c>
       <c r="AL13">
-        <f>AK13+0.2*(AP13-AK13)</f>
+        <f t="shared" si="27"/>
         <v>152055.4</v>
       </c>
       <c r="AM13">
-        <f>AK13+0.4*(AP13-AK13)</f>
+        <f t="shared" si="28"/>
         <v>191070.8</v>
       </c>
       <c r="AN13">
-        <f>AK13+0.6*(AP13-AK13)</f>
+        <f t="shared" si="29"/>
         <v>230086.2</v>
       </c>
       <c r="AO13">
-        <f>AK13+0.8*(AP13-AK13)</f>
+        <f t="shared" si="30"/>
         <v>269101.59999999998</v>
       </c>
       <c r="AP13">
-        <f>P13</f>
+        <f t="shared" si="31"/>
         <v>308117</v>
       </c>
     </row>

</xml_diff>

<commit_message>
CDRIA finally has a working scenario
</commit_message>
<xml_diff>
--- a/data/data_analysis/policy_effectiveness.xlsx
+++ b/data/data_analysis/policy_effectiveness.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\data\data_analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AC797D2-DFC3-4EE8-AEC1-47CFAC79D6A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36493C2A-6E2E-4AED-A124-E0C304B7480F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{5B094011-67C9-461D-BBBF-A6D3FE50B4AB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{5B094011-67C9-461D-BBBF-A6D3FE50B4AB}"/>
   </bookViews>
   <sheets>
     <sheet name="Low" sheetId="1" r:id="rId1"/>
@@ -19,10 +19,28 @@
     <sheet name="Counterproductive Intervention" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Counterproductive Intervention'!$A$1:$F$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Counterproductive Intervention'!$A$1:$H$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">High!$A$1:$N$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Low!$A$1:$N$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Net-Zero Mandate'!$A$1:$H$26</definedName>
+    <definedName name="_xlchart.v1.0" hidden="1">'Net-Zero Mandate'!$A$2:$B$26</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">'Net-Zero Mandate'!$D$1</definedName>
+    <definedName name="_xlchart.v1.10" hidden="1">'Net-Zero Mandate'!$D$1</definedName>
+    <definedName name="_xlchart.v1.11" hidden="1">'Net-Zero Mandate'!$D$2:$D$26</definedName>
+    <definedName name="_xlchart.v1.12" hidden="1">'Net-Zero Mandate'!$F$1</definedName>
+    <definedName name="_xlchart.v1.13" hidden="1">'Net-Zero Mandate'!$F$2:$F$26</definedName>
+    <definedName name="_xlchart.v1.14" hidden="1">'Net-Zero Mandate'!$H$1</definedName>
+    <definedName name="_xlchart.v1.15" hidden="1">'Net-Zero Mandate'!$H$2:$H$26</definedName>
+    <definedName name="_xlchart.v1.16" hidden="1">'Net-Zero Mandate'!$I$1</definedName>
+    <definedName name="_xlchart.v1.17" hidden="1">'Net-Zero Mandate'!$I$2:$I$26</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">'Net-Zero Mandate'!$D$2:$D$26</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">'Net-Zero Mandate'!$F$1</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">'Net-Zero Mandate'!$F$2:$F$26</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">'Net-Zero Mandate'!$H$1</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">'Net-Zero Mandate'!$H$2:$H$26</definedName>
+    <definedName name="_xlchart.v1.7" hidden="1">'Net-Zero Mandate'!$I$1</definedName>
+    <definedName name="_xlchart.v1.8" hidden="1">'Net-Zero Mandate'!$I$2:$I$26</definedName>
+    <definedName name="_xlchart.v1.9" hidden="1">'Net-Zero Mandate'!$A$2:$B$26</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="58">
   <si>
     <t>Scenario</t>
   </si>
@@ -161,46 +179,72 @@
     <t>4.1 Gt</t>
   </si>
   <si>
-    <t>NPV of Net Zero Mandate | 3.0% | Trillion $USD</t>
-  </si>
-  <si>
-    <t>Cost Decrease necessary in CDR market | 3.0% | % of CDR market</t>
-  </si>
-  <si>
     <t>NPV of Net Zero Mandate | 12.0% | Trillion $USD</t>
   </si>
   <si>
-    <t>Cost Decrease necessary in CDR market | 12.0% | % of CDR market</t>
-  </si>
-  <si>
     <t>NPV of Net Zero Mandate | 20.0% | Trillion $USD</t>
   </si>
   <si>
-    <t>Cost Decrease necessary in CDR market | 20.0% | % of CDR market</t>
-  </si>
-  <si>
     <t>B/C</t>
   </si>
   <si>
-    <t>NPV</t>
-  </si>
-  <si>
     <t>B/C Ranking</t>
   </si>
   <si>
-    <t>NPV Ranking</t>
-  </si>
-  <si>
-    <t>Correlation</t>
+    <t>Benefits | 2.0%</t>
+  </si>
+  <si>
+    <t>Costs | 2.0%</t>
+  </si>
+  <si>
+    <t>Benefits/Costs | 2.0%</t>
+  </si>
+  <si>
+    <t>Benefits-Costs | 2.0%</t>
+  </si>
+  <si>
+    <t>NPV of Net Zero Mandate | 2.0% | Trillion $USD</t>
+  </si>
+  <si>
+    <t>Abatement size in 2050</t>
+  </si>
+  <si>
+    <t>Correlation - NPV - Long</t>
+  </si>
+  <si>
+    <t>Correlation - NPV - Medium</t>
+  </si>
+  <si>
+    <t>NPV - Medium Term</t>
+  </si>
+  <si>
+    <t>NPV - Medium Term Ranking</t>
+  </si>
+  <si>
+    <t>NPV - Long Term</t>
+  </si>
+  <si>
+    <t>NPV - Long Term Ranking</t>
+  </si>
+  <si>
+    <t>Cost Decrease necessary in size of the CDR market in 2050</t>
+  </si>
+  <si>
+    <t>Cost Decrease necessary in NPV of CDR market | 12.0% discount rate</t>
+  </si>
+  <si>
+    <t>Cost Decrease necessary in NPV of CDR market | 2.0% discount rate</t>
+  </si>
+  <si>
+    <t>Cost Decrease necessary in NPV of CDR market | 20.0% discount rate</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
-    <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -253,12 +297,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -274,6 +317,808 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chartEx1.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:strDim type="cat">
+        <cx:f>_xlchart.v1.0</cx:f>
+      </cx:strDim>
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.2</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="1">
+      <cx:strDim type="cat">
+        <cx:f>_xlchart.v1.0</cx:f>
+      </cx:strDim>
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.4</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="2">
+      <cx:strDim type="cat">
+        <cx:f>_xlchart.v1.0</cx:f>
+      </cx:strDim>
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.6</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="3">
+      <cx:strDim type="cat">
+        <cx:f>_xlchart.v1.0</cx:f>
+      </cx:strDim>
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.8</cx:f>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0"/>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="boxWhisker" uniqueId="{DE0C5B9F-0FE7-4992-B189-22212844EA67}" formatIdx="1">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.1</cx:f>
+              <cx:v>Cost Decrease necessary in NPV of CDR market | 2.0% discount rate</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:visibility meanLine="0" meanMarker="1" nonoutliers="0" outliers="1"/>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{7B086B9F-0854-4B42-B6BE-2AD7B2DD934D}" formatIdx="3">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.3</cx:f>
+              <cx:v>Cost Decrease necessary in NPV of CDR market | 12.0% discount rate</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="1"/>
+          <cx:layoutPr>
+            <cx:visibility meanLine="0" meanMarker="1" nonoutliers="0" outliers="1"/>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{784F1E4D-A9F0-40BE-84B5-F799BC8E7E1C}" formatIdx="5">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.5</cx:f>
+              <cx:v>Cost Decrease necessary in NPV of CDR market | 20.0% discount rate</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="2"/>
+          <cx:layoutPr>
+            <cx:visibility meanLine="0" meanMarker="1" nonoutliers="0" outliers="1"/>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{30BC8885-0D0D-4EF2-A56D-0275F6A414C4}" formatIdx="6">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.7</cx:f>
+              <cx:v>Cost Decrease necessary in size of the CDR market in 2050</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="3"/>
+          <cx:layoutPr>
+            <cx:visibility meanLine="0" meanMarker="1" nonoutliers="0" outliers="1"/>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0">
+        <cx:catScaling gapWidth="1"/>
+        <cx:title>
+          <cx:tx>
+            <cx:txData>
+              <cx:v>CDR supply in 2050</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:txPr>
+            <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr" rtl="0">
+                <a:defRPr/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:sysClr>
+                  </a:solidFill>
+                  <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+                </a:rPr>
+                <a:t>CDR supply in 2050</a:t>
+              </a:r>
+            </a:p>
+          </cx:txPr>
+        </cx:title>
+        <cx:tickLabels/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+        <cx:title>
+          <cx:tx>
+            <cx:txData>
+              <cx:v>% of the size of the CDR market</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:txPr>
+            <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr" rtl="0">
+                <a:defRPr/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:sysClr>
+                  </a:solidFill>
+                  <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+                </a:rPr>
+                <a:t>% of the size of the CDR market</a:t>
+              </a:r>
+            </a:p>
+          </cx:txPr>
+        </cx:title>
+        <cx:majorGridlines/>
+        <cx:tickLabels/>
+      </cx:axis>
+    </cx:plotArea>
+    <cx:legend pos="t" align="ctr" overlay="0"/>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="406">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat">
+        <a:solidFill>
+          <a:srgbClr val="D9D9D9"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>495300</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>100011</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>47624</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="2" name="Chart 1">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{98AEC7E0-D0A5-1096-0DCB-A2DB2DA06286}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2014/chartex">
+              <cx:chart xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="8191500" y="290511"/>
+              <a:ext cx="4572000" cy="5662613"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100"/>
+                <a:t>This chart isn't available in your version of Excel.
+Editing this shape or saving this workbook into a different file format will permanently break the chart.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -614,16 +1459,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>15</v>
+        <v>42</v>
       </c>
       <c r="C1" t="s">
-        <v>16</v>
+        <v>43</v>
       </c>
       <c r="D1" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="E1" t="s">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="F1" t="s">
         <v>19</v>
@@ -686,16 +1531,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="1">
-        <v>-35712.763948744301</v>
+        <v>-40991.392169844003</v>
       </c>
       <c r="C2" s="1">
-        <v>67308.485298308602</v>
-      </c>
-      <c r="D2" s="4">
-        <v>-0.53058338470204403</v>
+        <v>73964.863896627197</v>
+      </c>
+      <c r="D2">
+        <v>-0.55420087336513202</v>
       </c>
       <c r="E2" s="1">
-        <v>-103021.249247053</v>
+        <v>-114956.256066471</v>
       </c>
       <c r="F2" s="1">
         <v>-11644.658803537901</v>
@@ -703,7 +1548,7 @@
       <c r="G2" s="1">
         <v>32506.920082813402</v>
       </c>
-      <c r="H2" s="4">
+      <c r="H2">
         <v>-0.358220919541823</v>
       </c>
       <c r="I2" s="1">
@@ -715,7 +1560,7 @@
       <c r="K2" s="1">
         <v>20078.072923277199</v>
       </c>
-      <c r="L2" s="4">
+      <c r="L2">
         <v>-0.24913278949754</v>
       </c>
       <c r="M2" s="1">
@@ -758,40 +1603,40 @@
         <v>2</v>
       </c>
       <c r="B3" s="1">
-        <v>-155964.89309999999</v>
+        <v>-190307.317572267</v>
       </c>
       <c r="C3" s="1">
-        <v>284005.84899999999</v>
-      </c>
-      <c r="D3" s="4">
-        <v>-0.54916084899999995</v>
+        <v>341722.55580809899</v>
+      </c>
+      <c r="D3">
+        <v>-0.55690592949661299</v>
       </c>
       <c r="E3" s="1">
-        <v>-439970.74209999997</v>
+        <v>-532029.87338036601</v>
       </c>
       <c r="F3" s="1">
-        <v>-30848.809229999999</v>
+        <v>-30848.8092279228</v>
       </c>
       <c r="G3" s="1">
-        <v>68806.729019999999</v>
-      </c>
-      <c r="H3" s="4">
-        <v>-0.44834000499999999</v>
+        <v>68806.729018270402</v>
+      </c>
+      <c r="H3">
+        <v>-0.44834000493950898</v>
       </c>
       <c r="I3" s="1">
-        <v>-99655.538249999998</v>
+        <v>-99655.538246193304</v>
       </c>
       <c r="J3" s="1">
-        <v>-9394.0921610000005</v>
+        <v>-9394.0921605190797</v>
       </c>
       <c r="K3" s="1">
-        <v>28774.34908</v>
-      </c>
-      <c r="L3" s="4">
-        <v>-0.32647453199999998</v>
+        <v>28774.349079517</v>
+      </c>
+      <c r="L3">
+        <v>-0.32647453238850899</v>
       </c>
       <c r="M3" s="1">
-        <v>-38168.44124</v>
+        <v>-38168.441240036103</v>
       </c>
       <c r="N3" t="s">
         <v>28</v>
@@ -830,40 +1675,40 @@
         <v>3</v>
       </c>
       <c r="B4" s="1">
-        <v>-101866.4703</v>
+        <v>-111896.814259928</v>
       </c>
       <c r="C4" s="1">
-        <v>53255.489130000002</v>
-      </c>
-      <c r="D4" s="4">
-        <v>-1.9127881819999999</v>
+        <v>57301.611772837801</v>
+      </c>
+      <c r="D4">
+        <v>-1.95276905479594</v>
       </c>
       <c r="E4" s="1">
-        <v>-155121.95939999999</v>
+        <v>-169198.426032766</v>
       </c>
       <c r="F4" s="1">
-        <v>-48616.163950000002</v>
+        <v>-48616.163952201903</v>
       </c>
       <c r="G4" s="1">
-        <v>29022.260190000001</v>
-      </c>
-      <c r="H4" s="4">
-        <v>-1.675133626</v>
+        <v>29022.260186042298</v>
+      </c>
+      <c r="H4">
+        <v>-1.6751336264148999</v>
       </c>
       <c r="I4" s="1">
-        <v>-77638.424140000003</v>
+        <v>-77638.4241382443</v>
       </c>
       <c r="J4" s="1">
-        <v>-28740.526330000001</v>
+        <v>-28740.526331305198</v>
       </c>
       <c r="K4" s="1">
-        <v>18227.87427</v>
-      </c>
-      <c r="L4" s="4">
-        <v>-1.5767349450000001</v>
+        <v>18227.874266083199</v>
+      </c>
+      <c r="L4">
+        <v>-1.5767349451593899</v>
       </c>
       <c r="M4" s="1">
-        <v>-46968.400600000001</v>
+        <v>-46968.400597388398</v>
       </c>
       <c r="N4" t="s">
         <v>28</v>
@@ -902,40 +1747,40 @@
         <v>4</v>
       </c>
       <c r="B5" s="1">
-        <v>-509105.55219999998</v>
+        <v>-610364.29686758004</v>
       </c>
       <c r="C5" s="1">
-        <v>520350.64659999998</v>
-      </c>
-      <c r="D5" s="4">
-        <v>-0.978389391</v>
+        <v>625628.34973158105</v>
+      </c>
+      <c r="D5">
+        <v>-0.97560204413602802</v>
       </c>
       <c r="E5" s="1">
-        <v>-1029456.199</v>
+        <v>-1235992.64659916</v>
       </c>
       <c r="F5" s="1">
-        <v>-123972.1329</v>
+        <v>-123972.132911298</v>
       </c>
       <c r="G5" s="1">
-        <v>121689.4575</v>
-      </c>
-      <c r="H5" s="4">
-        <v>-1.0187582019999999</v>
+        <v>121689.457472546</v>
+      </c>
+      <c r="H5">
+        <v>-1.01875820211678</v>
       </c>
       <c r="I5" s="1">
-        <v>-245661.59039999999</v>
+        <v>-245661.590383845</v>
       </c>
       <c r="J5" s="1">
-        <v>-48875.479590000003</v>
+        <v>-48875.479587231799</v>
       </c>
       <c r="K5" s="1">
-        <v>45154.745640000001</v>
-      </c>
-      <c r="L5" s="4">
-        <v>-1.082399621</v>
+        <v>45154.7456426149</v>
+      </c>
+      <c r="L5">
+        <v>-1.0823996213834299</v>
       </c>
       <c r="M5" s="1">
-        <v>-94030.225229999996</v>
+        <v>-94030.225229846794</v>
       </c>
       <c r="N5" t="s">
         <v>28</v>
@@ -946,40 +1791,40 @@
         <v>6</v>
       </c>
       <c r="B6" s="1">
-        <v>-19940.231660000001</v>
+        <v>-23639.052484741402</v>
       </c>
       <c r="C6" s="1">
-        <v>15897.22961</v>
-      </c>
-      <c r="D6" s="4">
-        <v>-1.254321171</v>
+        <v>19682.8288777735</v>
+      </c>
+      <c r="D6">
+        <v>-1.20099872998618</v>
       </c>
       <c r="E6" s="1">
-        <v>-35837.461259999996</v>
+        <v>-43321.881362514898</v>
       </c>
       <c r="F6" s="1">
-        <v>-5718.2312860000002</v>
+        <v>-5718.2312864800897</v>
       </c>
       <c r="G6" s="1">
-        <v>12851.378199999999</v>
-      </c>
-      <c r="H6" s="4">
-        <v>-0.44495082200000002</v>
+        <v>15677.5227380697</v>
+      </c>
+      <c r="H6">
+        <v>-0.36474074265537498</v>
       </c>
       <c r="I6" s="1">
-        <v>-18569.609479999999</v>
+        <v>-21395.754024549798</v>
       </c>
       <c r="J6" s="1">
-        <v>-2790.366364</v>
+        <v>-2790.36636372676</v>
       </c>
       <c r="K6" s="1">
-        <v>10951.605100000001</v>
-      </c>
-      <c r="L6" s="4">
-        <v>-0.25479063000000002</v>
+        <v>13463.719299594801</v>
+      </c>
+      <c r="L6">
+        <v>-0.207250782761842</v>
       </c>
       <c r="M6" s="1">
-        <v>-13741.97147</v>
+        <v>-16254.085663321601</v>
       </c>
       <c r="N6" t="s">
         <v>28</v>
@@ -990,40 +1835,40 @@
         <v>5</v>
       </c>
       <c r="B7" s="1">
-        <v>-25551.220799999999</v>
+        <v>-30682.746255407401</v>
       </c>
       <c r="C7" s="1">
-        <v>14303.578229999999</v>
-      </c>
-      <c r="D7" s="4">
-        <v>-1.7863516660000001</v>
+        <v>17090.916249983798</v>
+      </c>
+      <c r="D7">
+        <v>-1.7952663161307201</v>
       </c>
       <c r="E7" s="1">
-        <v>-39854.799030000002</v>
+        <v>-47773.662505391199</v>
       </c>
       <c r="F7" s="1">
-        <v>-6100.398029</v>
+        <v>-6100.3980291768003</v>
       </c>
       <c r="G7" s="1">
-        <v>11648.73883</v>
-      </c>
-      <c r="H7" s="4">
-        <v>-0.52369600900000002</v>
+        <v>12692.2292408466</v>
+      </c>
+      <c r="H7">
+        <v>-0.48064039133048803</v>
       </c>
       <c r="I7" s="1">
-        <v>-17749.136849999999</v>
+        <v>-18792.6272700234</v>
       </c>
       <c r="J7" s="1">
-        <v>-2360.7973050000001</v>
+        <v>-2360.7973050558699</v>
       </c>
       <c r="K7" s="1">
-        <v>9987.3194139999996</v>
-      </c>
-      <c r="L7" s="4">
-        <v>-0.23637947400000001</v>
+        <v>10689.1346820868</v>
+      </c>
+      <c r="L7">
+        <v>-0.220859534028715</v>
       </c>
       <c r="M7" s="1">
-        <v>-12348.11672</v>
+        <v>-13049.9319871426</v>
       </c>
       <c r="N7" t="s">
         <v>28</v>
@@ -1034,40 +1879,40 @@
         <v>8</v>
       </c>
       <c r="B8" s="1">
-        <v>-81560.515498519802</v>
+        <v>-97079.650583780895</v>
       </c>
       <c r="C8" s="1">
-        <v>14661.522330296701</v>
-      </c>
-      <c r="D8" s="4">
-        <v>-5.5628954252575902</v>
+        <v>29977.691435656099</v>
+      </c>
+      <c r="D8">
+        <v>-3.2383964853381602</v>
       </c>
       <c r="E8" s="1">
-        <v>-96222.037828816494</v>
+        <v>-127057.342019437</v>
       </c>
       <c r="F8" s="1">
         <v>-20972.403124771499</v>
       </c>
       <c r="G8" s="1">
-        <v>11912.037176166101</v>
-      </c>
-      <c r="H8" s="4">
-        <v>-1.76060591606728</v>
+        <v>18375.511162999999</v>
+      </c>
+      <c r="H8">
+        <v>-1.14132352230834</v>
       </c>
       <c r="I8" s="1">
-        <v>-32884.440300937698</v>
+        <v>-39347.9142877716</v>
       </c>
       <c r="J8" s="1">
         <v>-8406.4334333911793</v>
       </c>
       <c r="K8" s="1">
-        <v>10193.2673365766</v>
-      </c>
-      <c r="L8" s="4">
-        <v>-0.82470449913799904</v>
+        <v>13832.566021950501</v>
+      </c>
+      <c r="L8">
+        <v>-0.60772769275427296</v>
       </c>
       <c r="M8" s="1">
-        <v>-18599.7007699678</v>
+        <v>-22238.999455341698</v>
       </c>
       <c r="N8" t="s">
         <v>28</v>
@@ -1078,40 +1923,40 @@
         <v>7</v>
       </c>
       <c r="B9" s="1">
-        <v>-36596.431331457497</v>
+        <v>-43683.1580178394</v>
       </c>
       <c r="C9" s="1">
-        <v>14354.7341723564</v>
-      </c>
-      <c r="D9" s="4">
-        <v>-2.5494328833990401</v>
+        <v>19701.6259138606</v>
+      </c>
+      <c r="D9">
+        <v>-2.2172361920194099</v>
       </c>
       <c r="E9" s="1">
-        <v>-50951.165503814002</v>
+        <v>-63384.783931700098</v>
       </c>
       <c r="F9" s="1">
         <v>-9175.9801601351992</v>
       </c>
       <c r="G9" s="1">
-        <v>11684.215094699301</v>
-      </c>
-      <c r="H9" s="4">
-        <v>-0.78533132827192897</v>
+        <v>13838.706423644</v>
+      </c>
+      <c r="H9">
+        <v>-0.66306632131870602</v>
       </c>
       <c r="I9" s="1">
-        <v>-20860.195254834602</v>
+        <v>-23014.686583779199</v>
       </c>
       <c r="J9" s="1">
         <v>-3610.0129557775899</v>
       </c>
       <c r="K9" s="1">
-        <v>10013.395327025401</v>
-      </c>
-      <c r="L9" s="4">
-        <v>-0.36051836943203802</v>
+        <v>11226.4948888167</v>
+      </c>
+      <c r="L9">
+        <v>-0.32156189367473098</v>
       </c>
       <c r="M9" s="1">
-        <v>-13623.4082828029</v>
+        <v>-14836.5078445943</v>
       </c>
       <c r="N9" t="s">
         <v>28</v>
@@ -1122,40 +1967,40 @@
         <v>9</v>
       </c>
       <c r="B10" s="1">
-        <v>-42183.564330000001</v>
+        <v>-50470.5551048856</v>
       </c>
       <c r="C10" s="1">
-        <v>14413.47406</v>
-      </c>
-      <c r="D10" s="4">
-        <v>-2.9266757019999998</v>
+        <v>22047.6456426271</v>
+      </c>
+      <c r="D10">
+        <v>-2.2891584853534401</v>
       </c>
       <c r="E10" s="1">
-        <v>-56597.038390000002</v>
+        <v>-72518.200747512703</v>
       </c>
       <c r="F10" s="1">
-        <v>-10472.884529999999</v>
+        <v>-10472.8845316388</v>
       </c>
       <c r="G10" s="1">
-        <v>11734.88387</v>
-      </c>
-      <c r="H10" s="4">
-        <v>-0.89245744999999999</v>
+        <v>14865.3551125206</v>
+      </c>
+      <c r="H10">
+        <v>-0.70451626970000103</v>
       </c>
       <c r="I10" s="1">
-        <v>-22207.768400000001</v>
+        <v>-25338.239644159399</v>
       </c>
       <c r="J10" s="1">
-        <v>-4213.4803810000003</v>
+        <v>-4213.4803805597603</v>
       </c>
       <c r="K10" s="1">
-        <v>10058.82447</v>
-      </c>
-      <c r="L10" s="4">
-        <v>-0.41888397500000002</v>
+        <v>12164.270271887701</v>
+      </c>
+      <c r="L10">
+        <v>-0.346381680641979</v>
       </c>
       <c r="M10" s="1">
-        <v>-14272.30485</v>
+        <v>-16377.750652447499</v>
       </c>
       <c r="N10" t="s">
         <v>28</v>
@@ -1169,13 +2014,13 @@
         <v>0</v>
       </c>
       <c r="C11" s="1">
-        <v>14126.162917527599</v>
-      </c>
-      <c r="D11" s="4">
+        <v>14486.1268858849</v>
+      </c>
+      <c r="D11">
         <v>0</v>
       </c>
       <c r="E11" s="1">
-        <v>-14126.162917527599</v>
+        <v>-14486.1268858849</v>
       </c>
       <c r="F11" s="1">
         <v>0</v>
@@ -1183,7 +2028,7 @@
       <c r="G11" s="1">
         <v>11511.601320002699</v>
       </c>
-      <c r="H11" s="4">
+      <c r="H11">
         <v>0</v>
       </c>
       <c r="I11" s="1">
@@ -1195,7 +2040,7 @@
       <c r="K11" s="1">
         <v>9874.8984398431494</v>
       </c>
-      <c r="L11" s="4">
+      <c r="L11">
         <v>0</v>
       </c>
       <c r="M11" s="1">
@@ -1210,16 +2055,16 @@
         <v>10</v>
       </c>
       <c r="B12" s="1">
-        <v>-952.55022205237697</v>
+        <v>-1404.5679010868701</v>
       </c>
       <c r="C12" s="1">
-        <v>43434.528384603</v>
-      </c>
-      <c r="D12" s="4">
-        <v>-2.1930714053523401E-2</v>
+        <v>45132.0836071905</v>
+      </c>
+      <c r="D12">
+        <v>-3.1121273134907899E-2</v>
       </c>
       <c r="E12" s="1">
-        <v>-44387.078606655399</v>
+        <v>-46536.651508277399</v>
       </c>
       <c r="F12" s="1">
         <v>-32.085743248811902</v>
@@ -1227,7 +2072,7 @@
       <c r="G12" s="1">
         <v>32278.589396815001</v>
       </c>
-      <c r="H12" s="4">
+      <c r="H12">
         <v>-9.9402557076976408E-4</v>
       </c>
       <c r="I12" s="1">
@@ -1239,7 +2084,7 @@
       <c r="K12" s="1">
         <v>26285.648960687002</v>
       </c>
-      <c r="L12" s="4">
+      <c r="L12">
         <v>-8.6525474766389696E-3</v>
       </c>
       <c r="M12" s="1">
@@ -1253,41 +2098,41 @@
       <c r="A13" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="1">
-        <v>33227.843509999999</v>
+      <c r="B13">
+        <v>40603.4193094004</v>
       </c>
       <c r="C13" s="1">
-        <v>708723.9375</v>
-      </c>
-      <c r="D13" s="4">
-        <v>4.6884043E-2</v>
+        <v>828169.20249635505</v>
+      </c>
+      <c r="D13">
+        <v>4.9027927127704499E-2</v>
       </c>
       <c r="E13" s="1">
-        <v>-675496.09400000004</v>
+        <v>-787565.78318695503</v>
       </c>
       <c r="F13" s="1">
-        <v>4460.6170439999996</v>
+        <v>4460.6170443716501</v>
       </c>
       <c r="G13" s="1">
-        <v>222303.6073</v>
-      </c>
-      <c r="H13" s="4">
-        <v>2.0065428E-2</v>
+        <v>222303.607323328</v>
+      </c>
+      <c r="H13">
+        <v>2.0065428078654302E-2</v>
       </c>
       <c r="I13" s="1">
-        <v>-217842.9903</v>
+        <v>-217842.99027895599</v>
       </c>
       <c r="J13" s="1">
-        <v>-1031.071105</v>
+        <v>-1031.07110519603</v>
       </c>
       <c r="K13" s="1">
-        <v>108783.8031</v>
-      </c>
-      <c r="L13" s="4">
-        <v>-9.4781669999999991E-3</v>
+        <v>108783.803081255</v>
+      </c>
+      <c r="L13">
+        <v>-9.4781674844175191E-3</v>
       </c>
       <c r="M13" s="1">
-        <v>-109814.87420000001</v>
+        <v>-109814.87418645099</v>
       </c>
       <c r="N13" t="s">
         <v>28</v>
@@ -1297,17 +2142,17 @@
       <c r="A14" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="1">
-        <v>-1993.91561208246</v>
+      <c r="B14">
+        <v>-2626.77829541446</v>
       </c>
       <c r="C14" s="1">
-        <v>24714.8821550674</v>
-      </c>
-      <c r="D14" s="4">
-        <v>-8.0676719377908795E-2</v>
+        <v>25767.324754375601</v>
+      </c>
+      <c r="D14">
+        <v>-0.10194222025196401</v>
       </c>
       <c r="E14" s="1">
-        <v>-26708.797767149899</v>
+        <v>-28394.103049790101</v>
       </c>
       <c r="F14" s="1">
         <v>-184.162683612303</v>
@@ -1315,7 +2160,7 @@
       <c r="G14" s="1">
         <v>17829.693968081301</v>
       </c>
-      <c r="H14" s="4">
+      <c r="H14">
         <v>-1.0328987359064601E-2</v>
       </c>
       <c r="I14" s="1">
@@ -1327,7 +2172,7 @@
       <c r="K14" s="1">
         <v>14163.2689710182</v>
       </c>
-      <c r="L14" s="4">
+      <c r="L14">
         <v>-8.84242966642553E-3</v>
       </c>
       <c r="M14" s="1">
@@ -1457,40 +2302,40 @@
         <v>1</v>
       </c>
       <c r="B2" s="1">
-        <v>-81497.373680000004</v>
+        <v>-94864.731470308194</v>
       </c>
       <c r="C2" s="1">
-        <v>109656.8652</v>
-      </c>
-      <c r="D2" s="4">
-        <v>-0.74320357000000004</v>
-      </c>
-      <c r="E2">
-        <v>-191154.2389</v>
-      </c>
-      <c r="F2">
-        <v>-24012.40149</v>
+        <v>121535.566517909</v>
+      </c>
+      <c r="D2">
+        <v>-0.78055119327006905</v>
+      </c>
+      <c r="E2" s="1">
+        <v>-216400.297988217</v>
+      </c>
+      <c r="F2" s="1">
+        <v>-24012.4014868552</v>
       </c>
       <c r="G2" s="1">
-        <v>48730.788209999999</v>
-      </c>
-      <c r="H2" s="4">
-        <v>-0.49275627100000002</v>
+        <v>48730.788212699401</v>
+      </c>
+      <c r="H2">
+        <v>-0.49275627108772002</v>
       </c>
       <c r="I2" s="1">
-        <v>-72743.189700000003</v>
+        <v>-72743.189699554699</v>
       </c>
       <c r="J2" s="1">
-        <v>-9686.1108139999997</v>
+        <v>-9686.1108143464007</v>
       </c>
       <c r="K2" s="1">
-        <v>27914.545330000001</v>
-      </c>
-      <c r="L2" s="4">
-        <v>-0.34699153100000002</v>
+        <v>27914.545327342599</v>
+      </c>
+      <c r="L2">
+        <v>-0.346991530786594</v>
       </c>
       <c r="M2" s="1">
-        <v>-37600.656139999999</v>
+        <v>-37600.656141689004</v>
       </c>
       <c r="N2" t="s">
         <v>28</v>
@@ -1529,24 +2374,24 @@
         <v>2</v>
       </c>
       <c r="B3" s="1">
-        <v>-466401.91596012301</v>
+        <v>-573819.81405192497</v>
       </c>
       <c r="C3" s="1">
-        <v>669973.28975875594</v>
-      </c>
-      <c r="D3" s="4">
-        <v>-0.69615001536563403</v>
-      </c>
-      <c r="E3">
-        <v>-1136375.2057188801</v>
-      </c>
-      <c r="F3">
+        <v>815193.62386759603</v>
+      </c>
+      <c r="D3">
+        <v>-0.70390616075908496</v>
+      </c>
+      <c r="E3" s="1">
+        <v>-1389013.4379195201</v>
+      </c>
+      <c r="F3" s="1">
         <v>-84257.525916830593</v>
       </c>
       <c r="G3" s="1">
         <v>140944.522706794</v>
       </c>
-      <c r="H3" s="4">
+      <c r="H3">
         <v>-0.59780631626324898</v>
       </c>
       <c r="I3" s="1">
@@ -1558,7 +2403,7 @@
       <c r="K3" s="1">
         <v>49651.190773092399</v>
       </c>
-      <c r="L3" s="4">
+      <c r="L3">
         <v>-0.46735729927019298</v>
       </c>
       <c r="M3" s="1">
@@ -1573,40 +2418,40 @@
         <v>3</v>
       </c>
       <c r="B4" s="1">
-        <v>-170840.76010000001</v>
+        <v>-190209.27119441601</v>
       </c>
       <c r="C4" s="1">
-        <v>81431.476880000002</v>
-      </c>
-      <c r="D4" s="4">
-        <v>-2.0979695650000001</v>
+        <v>87711.441262196604</v>
+      </c>
+      <c r="D4">
+        <v>-2.1685799304770401</v>
       </c>
       <c r="E4" s="1">
-        <v>-252272.23699999999</v>
+        <v>-277920.71245661197</v>
       </c>
       <c r="F4" s="1">
-        <v>-74587.047070000001</v>
+        <v>-74587.047067286199</v>
       </c>
       <c r="G4" s="1">
-        <v>43819.217380000002</v>
-      </c>
-      <c r="H4" s="4">
-        <v>-1.7021537929999999</v>
+        <v>43819.217383484502</v>
+      </c>
+      <c r="H4">
+        <v>-1.7021537928104999</v>
       </c>
       <c r="I4" s="1">
-        <v>-118406.2645</v>
+        <v>-118406.26445077</v>
       </c>
       <c r="J4" s="1">
-        <v>-41848.541729999997</v>
+        <v>-41848.541730477998</v>
       </c>
       <c r="K4" s="1">
-        <v>27065.3112</v>
-      </c>
-      <c r="L4" s="4">
-        <v>-1.546205821</v>
+        <v>27065.311199394699</v>
+      </c>
+      <c r="L4">
+        <v>-1.54620582125114</v>
       </c>
       <c r="M4" s="1">
-        <v>-68913.852929999994</v>
+        <v>-68913.852929872693</v>
       </c>
       <c r="N4" t="s">
         <v>28</v>
@@ -1617,40 +2462,40 @@
         <v>4</v>
       </c>
       <c r="B5" s="1">
-        <v>-1258784.9040000001</v>
+        <v>-1529208.4767719801</v>
       </c>
       <c r="C5" s="1">
-        <v>1260175.575</v>
-      </c>
-      <c r="D5" s="4">
-        <v>-0.99889644700000002</v>
+        <v>1530788.13776271</v>
+      </c>
+      <c r="D5">
+        <v>-0.99896807340495397</v>
       </c>
       <c r="E5" s="1">
-        <v>-2518960.4789999998</v>
+        <v>-3059996.6145346998</v>
       </c>
       <c r="F5" s="1">
-        <v>-265869.2219</v>
+        <v>-265869.22186544299</v>
       </c>
       <c r="G5" s="1">
-        <v>264137.73710000003</v>
-      </c>
-      <c r="H5" s="4">
-        <v>-1.0065552339999999</v>
+        <v>264137.73711263499</v>
+      </c>
+      <c r="H5">
+        <v>-1.0065552342945601</v>
       </c>
       <c r="I5" s="1">
-        <v>-530006.95900000003</v>
+        <v>-530006.95897807798</v>
       </c>
       <c r="J5" s="1">
-        <v>-90716.728929999997</v>
+        <v>-90716.728933609906</v>
       </c>
       <c r="K5" s="1">
-        <v>87679.742610000001</v>
-      </c>
-      <c r="L5" s="4">
-        <v>-1.034637263</v>
+        <v>87679.742607520398</v>
+      </c>
+      <c r="L5">
+        <v>-1.0346372632465799</v>
       </c>
       <c r="M5" s="1">
-        <v>-178396.47150000001</v>
+        <v>-178396.47154113001</v>
       </c>
       <c r="N5" t="s">
         <v>28</v>
@@ -1664,21 +2509,21 @@
         <v>0</v>
       </c>
       <c r="C6" s="1">
-        <v>16026.1779279129</v>
-      </c>
-      <c r="D6" s="4">
+        <v>16454.604553368801</v>
+      </c>
+      <c r="D6">
         <v>0</v>
       </c>
-      <c r="E6">
-        <v>-16026.1779279129</v>
-      </c>
-      <c r="F6">
+      <c r="E6" s="1">
+        <v>-16454.604553368801</v>
+      </c>
+      <c r="F6" s="1">
         <v>0</v>
       </c>
       <c r="G6" s="1">
         <v>12922.5120645157</v>
       </c>
-      <c r="H6" s="4">
+      <c r="H6">
         <v>0</v>
       </c>
       <c r="I6" s="1">
@@ -1690,7 +2535,7 @@
       <c r="K6" s="1">
         <v>10988.815786839299</v>
       </c>
-      <c r="L6" s="4">
+      <c r="L6">
         <v>0</v>
       </c>
       <c r="M6" s="1">
@@ -1705,40 +2550,40 @@
         <v>6</v>
       </c>
       <c r="B7" s="1">
-        <v>-67025.524609999993</v>
+        <v>-81711.783899172602</v>
       </c>
       <c r="C7" s="1">
-        <v>18191.474730000002</v>
-      </c>
-      <c r="D7" s="4">
-        <v>-3.6844470060000001</v>
+        <v>22059.733037833099</v>
+      </c>
+      <c r="D7">
+        <v>-3.7041148122252601</v>
       </c>
       <c r="E7" s="1">
-        <v>-85216.999349999998</v>
+        <v>-103771.516937005</v>
       </c>
       <c r="F7" s="1">
-        <v>-14041.80701</v>
+        <v>-14041.807010664401</v>
       </c>
       <c r="G7" s="1">
-        <v>14555.096159999999</v>
-      </c>
-      <c r="H7" s="4">
-        <v>-0.96473474699999995</v>
+        <v>17381.240704187301</v>
+      </c>
+      <c r="H7">
+        <v>-0.8078713855727</v>
       </c>
       <c r="I7" s="1">
-        <v>-28596.903170000001</v>
+        <v>-31423.0477148518</v>
       </c>
       <c r="J7" s="1">
-        <v>-5067.3328270000002</v>
+        <v>-5067.3328268512496</v>
       </c>
       <c r="K7" s="1">
-        <v>12296.74086</v>
-      </c>
-      <c r="L7" s="4">
-        <v>-0.41208747000000001</v>
+        <v>14808.855061788299</v>
+      </c>
+      <c r="L7">
+        <v>-0.34218262017612899</v>
       </c>
       <c r="M7" s="1">
-        <v>-17364.073690000001</v>
+        <v>-19876.187888639499</v>
       </c>
       <c r="N7" t="s">
         <v>28</v>
@@ -1749,40 +2594,40 @@
         <v>5</v>
       </c>
       <c r="B8" s="1">
-        <v>-61496.951390000002</v>
+        <v>-74787.623200904796</v>
       </c>
       <c r="C8" s="1">
-        <v>16237.943450000001</v>
-      </c>
-      <c r="D8" s="4">
-        <v>-3.7872376870000002</v>
+        <v>19094.971222653399</v>
+      </c>
+      <c r="D8">
+        <v>-3.9166135590809201</v>
       </c>
       <c r="E8" s="1">
-        <v>-77734.894839999994</v>
+        <v>-93882.594423558301</v>
       </c>
       <c r="F8" s="1">
-        <v>-12795.920630000001</v>
+        <v>-12795.920628411601</v>
       </c>
       <c r="G8" s="1">
-        <v>13085.23021</v>
-      </c>
-      <c r="H8" s="4">
-        <v>-0.97789037099999998</v>
+        <v>14128.7206300791</v>
+      </c>
+      <c r="H8">
+        <v>-0.90566732568623198</v>
       </c>
       <c r="I8" s="1">
-        <v>-25881.150839999998</v>
+        <v>-26924.641258490799</v>
       </c>
       <c r="J8" s="1">
-        <v>-4277.3243689999999</v>
+        <v>-4277.3243685469497</v>
       </c>
       <c r="K8" s="1">
-        <v>11121.488859999999</v>
-      </c>
-      <c r="L8" s="4">
-        <v>-0.38459997800000001</v>
+        <v>11823.3041249241</v>
+      </c>
+      <c r="L8">
+        <v>-0.361770645781675</v>
       </c>
       <c r="M8" s="1">
-        <v>-15398.81323</v>
+        <v>-16100.628493471</v>
       </c>
       <c r="N8" t="s">
         <v>28</v>
@@ -1793,40 +2638,40 @@
         <v>8</v>
       </c>
       <c r="B9" s="1">
-        <v>-167293.31460000001</v>
+        <v>-201382.40255214801</v>
       </c>
       <c r="C9" s="1">
-        <v>16682.334579999999</v>
-      </c>
-      <c r="D9" s="4">
-        <v>-10.028171650000001</v>
+        <v>32071.308412600101</v>
+      </c>
+      <c r="D9">
+        <v>-6.2792075696240897</v>
       </c>
       <c r="E9" s="1">
-        <v>-183975.64920000001</v>
+        <v>-233453.710964748</v>
       </c>
       <c r="F9" s="1">
-        <v>-38626.101040000001</v>
+        <v>-38626.101035459098</v>
       </c>
       <c r="G9" s="1">
-        <v>13412.72192</v>
-      </c>
-      <c r="H9" s="4">
-        <v>-2.8798107700000002</v>
+        <v>19876.195905398199</v>
+      </c>
+      <c r="H9">
+        <v>-1.9433346913716201</v>
       </c>
       <c r="I9" s="1">
-        <v>-52038.822950000002</v>
+        <v>-58502.296940857297</v>
       </c>
       <c r="J9" s="1">
-        <v>-14104.874299999999</v>
+        <v>-14104.8743016727</v>
       </c>
       <c r="K9" s="1">
-        <v>11378.1173</v>
-      </c>
-      <c r="L9" s="4">
-        <v>-1.239649226</v>
+        <v>15017.4159804518</v>
+      </c>
+      <c r="L9">
+        <v>-0.93923444086739505</v>
       </c>
       <c r="M9" s="1">
-        <v>-25482.991600000001</v>
+        <v>-29122.290282124501</v>
       </c>
       <c r="N9" t="s">
         <v>28</v>
@@ -1837,40 +2682,40 @@
         <v>7</v>
       </c>
       <c r="B10" s="1">
-        <v>-81354.279490000001</v>
+        <v>-98338.675448048598</v>
       </c>
       <c r="C10" s="1">
-        <v>16305.1145</v>
-      </c>
-      <c r="D10" s="4">
-        <v>-4.9894945230000003</v>
+        <v>21722.272439247401</v>
+      </c>
+      <c r="D10">
+        <v>-4.5270896828626404</v>
       </c>
       <c r="E10" s="1">
-        <v>-97659.393979999993</v>
+        <v>-120060.947887296</v>
       </c>
       <c r="F10" s="1">
-        <v>-17986.986789999999</v>
+        <v>-17986.986790839499</v>
       </c>
       <c r="G10" s="1">
-        <v>13132.603209999999</v>
-      </c>
-      <c r="H10" s="4">
-        <v>-1.3696436649999999</v>
+        <v>15287.094538355101</v>
+      </c>
+      <c r="H10">
+        <v>-1.1766125175526601</v>
       </c>
       <c r="I10" s="1">
-        <v>-31119.59</v>
+        <v>-33274.081329194603</v>
       </c>
       <c r="J10" s="1">
-        <v>-6302.0903449999996</v>
+        <v>-6302.0903447309802</v>
       </c>
       <c r="K10" s="1">
-        <v>11156.96053</v>
-      </c>
-      <c r="L10" s="4">
-        <v>-0.56485727699999999</v>
+        <v>12370.0600946878</v>
+      </c>
+      <c r="L10">
+        <v>-0.50946319552944896</v>
       </c>
       <c r="M10" s="1">
-        <v>-17459.050879999999</v>
+        <v>-18672.1504394187</v>
       </c>
       <c r="N10" t="s">
         <v>28</v>
@@ -1881,40 +2726,40 @@
         <v>9</v>
       </c>
       <c r="B11" s="1">
-        <v>-92931.793090000006</v>
+        <v>-112560.083841115</v>
       </c>
       <c r="C11" s="1">
-        <v>16367.139950000001</v>
-      </c>
-      <c r="D11" s="4">
-        <v>-5.6779494389999998</v>
+        <v>24071.699131444799</v>
+      </c>
+      <c r="D11">
+        <v>-4.6760340109967</v>
       </c>
       <c r="E11" s="1">
-        <v>-109298.933</v>
+        <v>-136631.78297256</v>
       </c>
       <c r="F11" s="1">
-        <v>-20252.154009999998</v>
+        <v>-20252.154009836198</v>
       </c>
       <c r="G11" s="1">
-        <v>13185.69109</v>
-      </c>
-      <c r="H11" s="4">
-        <v>-1.5359190410000001</v>
+        <v>16316.162333554499</v>
+      </c>
+      <c r="H11">
+        <v>-1.2412326866954</v>
       </c>
       <c r="I11" s="1">
-        <v>-33437.845099999999</v>
+        <v>-36568.316343390703</v>
       </c>
       <c r="J11" s="1">
-        <v>-7133.5598010000003</v>
+        <v>-7133.5598014398502</v>
       </c>
       <c r="K11" s="1">
-        <v>11204.283649999999</v>
-      </c>
-      <c r="L11" s="4">
-        <v>-0.63668147200000003</v>
+        <v>13309.729450819899</v>
+      </c>
+      <c r="L11">
+        <v>-0.535965800642205</v>
       </c>
       <c r="M11" s="1">
-        <v>-18337.84345</v>
+        <v>-20443.289252259801</v>
       </c>
       <c r="N11" t="s">
         <v>28</v>
@@ -1925,40 +2770,40 @@
         <v>10</v>
       </c>
       <c r="B12" s="1">
-        <v>-44390.982504673499</v>
+        <v>-20612.841126253501</v>
       </c>
       <c r="C12" s="1">
-        <v>50120.450696353699</v>
-      </c>
-      <c r="D12" s="4">
-        <v>-0.88568602013594699</v>
-      </c>
-      <c r="E12">
-        <v>-94511.433201027306</v>
-      </c>
-      <c r="F12">
-        <v>-17986.197270025001</v>
+        <v>47147.659759674803</v>
+      </c>
+      <c r="D12">
+        <v>-0.43719754556903001</v>
+      </c>
+      <c r="E12" s="1">
+        <v>-67760.500885928399</v>
+      </c>
+      <c r="F12" s="1">
+        <v>-2555.2191726661399</v>
       </c>
       <c r="G12" s="1">
-        <v>36363.512184802501</v>
-      </c>
-      <c r="H12" s="4">
-        <v>-0.49462211401961598</v>
+        <v>33709.460372616202</v>
+      </c>
+      <c r="H12">
+        <v>-7.58012482081101E-2</v>
       </c>
       <c r="I12" s="1">
-        <v>-54349.7094548276</v>
+        <v>-36264.679545282401</v>
       </c>
       <c r="J12" s="1">
-        <v>-10413.617036727001</v>
+        <v>-817.00285092435604</v>
       </c>
       <c r="K12" s="1">
-        <v>29063.638202340098</v>
-      </c>
-      <c r="L12" s="4">
-        <v>-0.35830397296538602</v>
+        <v>27410.213109250599</v>
+      </c>
+      <c r="L12">
+        <v>-2.9806512180987999E-2</v>
       </c>
       <c r="M12" s="1">
-        <v>-39477.255239067199</v>
+        <v>-28227.215960174901</v>
       </c>
       <c r="N12" t="s">
         <v>28</v>
@@ -1969,40 +2814,40 @@
         <v>11</v>
       </c>
       <c r="B13" s="1">
-        <v>28435.070199999998</v>
+        <v>33750.559282223403</v>
       </c>
       <c r="C13" s="1">
-        <v>778616.07140000002</v>
-      </c>
-      <c r="D13" s="4">
-        <v>3.6520014000000003E-2</v>
+        <v>913639.44245667802</v>
+      </c>
+      <c r="D13">
+        <v>3.6940786172137897E-2</v>
       </c>
       <c r="E13" s="1">
-        <v>-750181.00120000006</v>
+        <v>-879888.88317445503</v>
       </c>
       <c r="F13" s="1">
-        <v>5157.5221170000004</v>
+        <v>5157.5221174354301</v>
       </c>
       <c r="G13" s="1">
-        <v>235929.4785</v>
-      </c>
-      <c r="H13" s="4">
-        <v>2.1860439999999998E-2</v>
+        <v>235929.47854249101</v>
+      </c>
+      <c r="H13">
+        <v>2.1860439608043899E-2</v>
       </c>
       <c r="I13" s="1">
-        <v>-230771.9564</v>
+        <v>-230771.95642505601</v>
       </c>
       <c r="J13" s="1">
-        <v>-354.46081329999998</v>
+        <v>-354.46081332431601</v>
       </c>
       <c r="K13" s="1">
-        <v>113106.55809999999</v>
-      </c>
-      <c r="L13" s="4">
-        <v>-3.1338659999999999E-3</v>
+        <v>113106.55812487499</v>
+      </c>
+      <c r="L13">
+        <v>-3.1338661453474098E-3</v>
       </c>
       <c r="M13" s="1">
-        <v>-113461.0189</v>
+        <v>-113461.01893819901</v>
       </c>
       <c r="N13" t="s">
         <v>28</v>
@@ -2013,24 +2858,24 @@
         <v>12</v>
       </c>
       <c r="B14" s="1">
-        <v>-17689.664092087602</v>
+        <v>-22101.075343330998</v>
       </c>
       <c r="C14" s="1">
-        <v>26639.461793662798</v>
-      </c>
-      <c r="D14" s="4">
-        <v>-0.66403984544071204</v>
-      </c>
-      <c r="E14">
-        <v>-44329.125885750502</v>
-      </c>
-      <c r="F14">
+        <v>27762.780358668701</v>
+      </c>
+      <c r="D14">
+        <v>-0.79606851539385404</v>
+      </c>
+      <c r="E14" s="1">
+        <v>-49863.855701999797</v>
+      </c>
+      <c r="F14" s="1">
         <v>-2707.91448460225</v>
       </c>
       <c r="G14" s="1">
         <v>19251.584572950102</v>
       </c>
-      <c r="H14" s="4">
+      <c r="H14">
         <v>-0.140659303879175</v>
       </c>
       <c r="I14" s="1">
@@ -2042,7 +2887,7 @@
       <c r="K14" s="1">
         <v>15282.8414246461</v>
       </c>
-      <c r="L14" s="4">
+      <c r="L14">
         <v>-4.5280302139073698E-2</v>
       </c>
       <c r="M14" s="1">
@@ -2108,14 +2953,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66EF8D6B-AAC7-4D47-8A22-E3B6AC50568B}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2123,25 +2968,31 @@
         <v>32</v>
       </c>
       <c r="C1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E1" t="s">
         <v>38</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
+        <v>55</v>
+      </c>
+      <c r="G1" t="s">
         <v>39</v>
       </c>
-      <c r="E1" t="s">
-        <v>40</v>
-      </c>
-      <c r="F1" t="s">
-        <v>41</v>
-      </c>
-      <c r="G1" t="s">
-        <v>42</v>
-      </c>
       <c r="H1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>57</v>
+      </c>
+      <c r="I1" t="s">
+        <v>54</v>
+      </c>
+      <c r="J1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>31</v>
       </c>
@@ -2149,25 +3000,31 @@
         <v>33</v>
       </c>
       <c r="C2">
-        <v>11.6714641925513</v>
+        <v>5.4175769899473796</v>
       </c>
       <c r="D2">
         <v>0</v>
       </c>
       <c r="E2">
-        <v>4.0170113230740796</v>
+        <v>1.21462324059764</v>
       </c>
       <c r="F2">
         <v>0</v>
       </c>
       <c r="G2">
-        <v>1.95023254692459</v>
+        <v>0.50517645710506498</v>
       </c>
       <c r="H2">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0.84290901691641495</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -2175,25 +3032,31 @@
         <v>34</v>
       </c>
       <c r="C3">
-        <v>11.8429645489643</v>
+        <v>5.4526751392889503</v>
       </c>
       <c r="D3">
-        <v>46.648999763436599</v>
+        <v>7.9722193986204699</v>
       </c>
       <c r="E3">
-        <v>4.0359766571962803</v>
+        <v>1.2265993616247699</v>
       </c>
       <c r="F3">
-        <v>20.498026403063999</v>
+        <v>12.943976807287701</v>
       </c>
       <c r="G3">
-        <v>1.9519792491260499</v>
+        <v>0.51196546571708901</v>
       </c>
       <c r="H3">
-        <v>4.4576105335652398</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+        <v>17.3256530369916</v>
+      </c>
+      <c r="I3">
+        <v>2.1065459229826602</v>
+      </c>
+      <c r="J3">
+        <v>0.84470017355869997</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -2201,25 +3064,31 @@
         <v>34</v>
       </c>
       <c r="C4">
-        <v>11.864365629027301</v>
+        <v>5.4176986655229298</v>
       </c>
       <c r="D4">
-        <v>77.975318603618106</v>
+        <v>4.18215697221197E-2</v>
       </c>
       <c r="E4">
-        <v>4.0201810500522601</v>
+        <v>1.2200220480936199</v>
       </c>
       <c r="F4">
-        <v>4.3232246062359998</v>
+        <v>7.3634914210611901</v>
       </c>
       <c r="G4">
-        <v>1.94080995822802</v>
+        <v>0.50945647219154799</v>
       </c>
       <c r="H4">
-        <v>-27.082058811239101</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+        <v>12.3014623706724</v>
+      </c>
+      <c r="I4">
+        <v>-32.193007747667103</v>
+      </c>
+      <c r="J4">
+        <v>0.83139861124438796</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -2227,25 +3096,31 @@
         <v>34</v>
       </c>
       <c r="C5">
-        <v>11.8492873032673</v>
+        <v>5.4325606637280597</v>
       </c>
       <c r="D5">
-        <v>46.379062212209298</v>
+        <v>3.27434679522118</v>
       </c>
       <c r="E5">
-        <v>4.0355326064168597</v>
+        <v>1.2224848613141599</v>
       </c>
       <c r="F5">
-        <v>18.813043557568299</v>
+        <v>7.9854624669163199</v>
       </c>
       <c r="G5">
-        <v>1.9512772139851899</v>
+        <v>0.51069933585084104</v>
       </c>
       <c r="H5">
-        <v>2.5235661806703602</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+        <v>13.341427664723501</v>
+      </c>
+      <c r="I5">
+        <v>-4.7661224787360901</v>
+      </c>
+      <c r="J5">
+        <v>0.83899992545385804</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -2253,25 +3128,31 @@
         <v>34</v>
       </c>
       <c r="C6">
-        <v>11.923951512722301</v>
+        <v>5.4675026820248398</v>
       </c>
       <c r="D6">
-        <v>66.830684641143094</v>
+        <v>11.080702210154501</v>
       </c>
       <c r="E6">
-        <v>4.06937919676413</v>
+        <v>1.23111451544623</v>
       </c>
       <c r="F6">
-        <v>53.400101276959496</v>
+        <v>16.816335761750899</v>
       </c>
       <c r="G6">
-        <v>1.9689061406836099</v>
+        <v>0.513737215902481</v>
       </c>
       <c r="H6">
-        <v>44.645868252751001</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+        <v>20.4675390471334</v>
+      </c>
+      <c r="I6">
+        <v>-1.6578001841819501</v>
+      </c>
+      <c r="J6">
+        <v>0.84157377260607302</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -2279,25 +3160,31 @@
         <v>34</v>
       </c>
       <c r="C7">
-        <v>12.1201777868246</v>
+        <v>5.4690262916548296</v>
       </c>
       <c r="D7">
-        <v>139.44203911104401</v>
+        <v>13.3924163736789</v>
       </c>
       <c r="E7">
-        <v>4.1666434691336596</v>
+        <v>1.24274587562168</v>
       </c>
       <c r="F7">
-        <v>179.857163829526</v>
+        <v>33.8032802979519</v>
       </c>
       <c r="G7">
-        <v>2.0235870922189201</v>
+        <v>0.52159577509564503</v>
       </c>
       <c r="H7">
-        <v>205.01324778073999</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+        <v>45.889149664641799</v>
+      </c>
+      <c r="I7">
+        <v>-17.610796138934401</v>
+      </c>
+      <c r="J7">
+        <v>0.83026724806194996</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -2305,25 +3192,31 @@
         <v>34</v>
       </c>
       <c r="C8">
-        <v>11.978026074055</v>
+        <v>5.4704807351999003</v>
       </c>
       <c r="D8">
-        <v>83.5873579802481</v>
+        <v>12.090518117610101</v>
       </c>
       <c r="E8">
-        <v>4.0952437698930897</v>
+        <v>1.2344805645724799</v>
       </c>
       <c r="F8">
-        <v>82.357389931911399</v>
+        <v>20.904336245338801</v>
       </c>
       <c r="G8">
-        <v>1.9832089280410501</v>
+        <v>0.51580994167138305</v>
       </c>
       <c r="H8">
-        <v>81.269026505650601</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+        <v>26.205814883550801</v>
+      </c>
+      <c r="I8">
+        <v>-4.2330036189303399</v>
+      </c>
+      <c r="J8">
+        <v>0.83955683086218402</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -2331,25 +3224,31 @@
         <v>34</v>
       </c>
       <c r="C9">
-        <v>11.9783780590988</v>
+        <v>5.4684294412951697</v>
       </c>
       <c r="D9">
-        <v>84.977875967937194</v>
+        <v>11.804833462263</v>
       </c>
       <c r="E9">
-        <v>4.0969123769269702</v>
+        <v>1.23469984643818</v>
       </c>
       <c r="F9">
-        <v>85.278269416212396</v>
+        <v>21.4277299143567</v>
       </c>
       <c r="G9">
-        <v>1.98468952931547</v>
+        <v>0.51633662594582996</v>
       </c>
       <c r="H9">
-        <v>86.199895651216806</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+        <v>27.919026065915698</v>
+      </c>
+      <c r="I9">
+        <v>-5.6982743163725003</v>
+      </c>
+      <c r="J9">
+        <v>0.83849573801586097</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -2357,25 +3256,31 @@
         <v>34</v>
       </c>
       <c r="C10">
-        <v>11.911226021002999</v>
+        <v>5.5007324623894398</v>
       </c>
       <c r="D10">
-        <v>59.442226114714899</v>
+        <v>17.279164053851499</v>
       </c>
       <c r="E10">
-        <v>4.0538802198026396</v>
+        <v>1.2333937815064</v>
       </c>
       <c r="F10">
-        <v>35.393894665297204</v>
+        <v>18.019593931069998</v>
       </c>
       <c r="G10">
-        <v>1.95853077165749</v>
+        <v>0.513172389200656</v>
       </c>
       <c r="H10">
-        <v>18.779861431983999</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+        <v>18.0957375351921</v>
+      </c>
+      <c r="I10">
+        <v>10.550045036612699</v>
+      </c>
+      <c r="J10">
+        <v>0.85202798348279696</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -2383,25 +3288,31 @@
         <v>34</v>
       </c>
       <c r="C11">
-        <v>11.8908294673068</v>
+        <v>5.4984718932521197</v>
       </c>
       <c r="D11">
-        <v>54.514211977778203</v>
+        <v>16.858636173362701</v>
       </c>
       <c r="E11">
-        <v>4.0557526757695896</v>
+        <v>1.2461970757383001</v>
       </c>
       <c r="F11">
-        <v>37.202899164071297</v>
+        <v>30.32001009859</v>
       </c>
       <c r="G11">
-        <v>1.96485522697099</v>
+        <v>0.52572239246154995</v>
       </c>
       <c r="H11">
-        <v>33.264066186409202</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+        <v>46.738446809391498</v>
+      </c>
+      <c r="I11">
+        <v>3.6313721464693201</v>
+      </c>
+      <c r="J11">
+        <v>0.84599726777568296</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -2409,25 +3320,31 @@
         <v>34</v>
       </c>
       <c r="C12">
-        <v>12.236527303614601</v>
+        <v>5.7243968175114803</v>
       </c>
       <c r="D12">
-        <v>129.429290816709</v>
+        <v>58.794583510587898</v>
       </c>
       <c r="E12">
-        <v>4.1027265788317999</v>
+        <v>1.3160625148040399</v>
       </c>
       <c r="F12">
-        <v>78.907141092873204</v>
+        <v>93.382246268824602</v>
       </c>
       <c r="G12">
-        <v>1.9735796206688301</v>
+        <v>0.56052492044233604</v>
       </c>
       <c r="H12">
-        <v>54.099560276592101</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+        <v>128.25279781669599</v>
+      </c>
+      <c r="I12">
+        <v>11.060630810043</v>
+      </c>
+      <c r="J12">
+        <v>0.85298997575326196</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -2435,25 +3352,31 @@
         <v>34</v>
       </c>
       <c r="C13">
-        <v>11.875310269400501</v>
+        <v>5.4812879541932098</v>
       </c>
       <c r="D13">
-        <v>50.788990038952299</v>
+        <v>13.3113794026041</v>
       </c>
       <c r="E13">
-        <v>4.0440175944995902</v>
+        <v>1.2334114219814001</v>
       </c>
       <c r="F13">
-        <v>25.9717569864757</v>
+        <v>18.068472816125901</v>
       </c>
       <c r="G13">
-        <v>1.95475015347694</v>
+        <v>0.51482952026028495</v>
       </c>
       <c r="H13">
-        <v>10.2529361886546</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>21.908114265485199</v>
+      </c>
+      <c r="I13">
+        <v>3.6008171018680599</v>
+      </c>
+      <c r="J13">
+        <v>0.84597114411709196</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>1</v>
       </c>
@@ -2461,25 +3384,31 @@
         <v>36</v>
       </c>
       <c r="C14">
-        <v>12.3829778439019</v>
+        <v>5.5417657965940101</v>
       </c>
       <c r="D14">
-        <v>73.687970804576906</v>
+        <v>10.5657233468163</v>
       </c>
       <c r="E14">
-        <v>4.1061101086294602</v>
+        <v>1.2457635282608599</v>
       </c>
       <c r="F14">
-        <v>44.141849009060799</v>
+        <v>15.427706085558601</v>
       </c>
       <c r="G14">
-        <v>1.9630318924891701</v>
+        <v>0.51994929271492896</v>
       </c>
       <c r="H14">
-        <v>18.2262669057897</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>21.036516548608301</v>
+      </c>
+      <c r="I14">
+        <v>2.9193308209991198</v>
+      </c>
+      <c r="J14">
+        <v>0.85190822649338904</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>2</v>
       </c>
@@ -2487,25 +3416,31 @@
         <v>36</v>
       </c>
       <c r="C15">
-        <v>12.5900485095412</v>
+        <v>5.5469377878581998</v>
       </c>
       <c r="D15">
-        <v>158.19336070381399</v>
+        <v>18.574625943324801</v>
       </c>
       <c r="E15">
-        <v>4.1427045613212297</v>
+        <v>1.24906589704301</v>
       </c>
       <c r="F15">
-        <v>88.765537100189803</v>
+        <v>24.3236703991907</v>
       </c>
       <c r="G15">
-        <v>1.97226029495764</v>
+        <v>0.52138261081502402</v>
       </c>
       <c r="H15">
-        <v>38.845541358940103</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>28.5792634483009</v>
+      </c>
+      <c r="I15">
+        <v>2.9106502559085001</v>
+      </c>
+      <c r="J15">
+        <v>0.84685936766477898</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -2513,25 +3448,31 @@
         <v>36</v>
       </c>
       <c r="C16">
-        <v>12.5386826547015</v>
+        <v>5.6382572848615498</v>
       </c>
       <c r="D16">
-        <v>82.823053052219606</v>
+        <v>17.3728711500404</v>
       </c>
       <c r="E16">
-        <v>4.1526147790860204</v>
+        <v>1.26406672926263</v>
       </c>
       <c r="F16">
-        <v>60.039008352776797</v>
+        <v>21.891315429941098</v>
       </c>
       <c r="G16">
-        <v>1.9819425484725299</v>
+        <v>0.52557117328980196</v>
       </c>
       <c r="H16">
-        <v>39.681729973460101</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>25.521841091825902</v>
+      </c>
+      <c r="I16">
+        <v>6.3225799064404198</v>
+      </c>
+      <c r="J16">
+        <v>0.86290930411762501</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>6</v>
       </c>
@@ -2539,25 +3480,31 @@
         <v>36</v>
       </c>
       <c r="C17">
-        <v>12.4124638387233</v>
+        <v>5.4997560593119497</v>
       </c>
       <c r="D17">
-        <v>75.608486762679703</v>
+        <v>6.9142507501659596</v>
       </c>
       <c r="E17">
-        <v>4.1185187728864197</v>
+        <v>1.2403987076644101</v>
       </c>
       <c r="F17">
-        <v>47.922213765437903</v>
+        <v>12.1687368263228</v>
       </c>
       <c r="G17">
-        <v>1.96872763712804</v>
+        <v>0.51878134271989196</v>
       </c>
       <c r="H17">
-        <v>24.711684783752499</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>18.177778055381498</v>
+      </c>
+      <c r="I17">
+        <v>-3.1562896930530902</v>
+      </c>
+      <c r="J17">
+        <v>0.83367092671279197</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>5</v>
       </c>
@@ -2565,25 +3512,31 @@
         <v>36</v>
       </c>
       <c r="C18">
-        <v>12.510377009198001</v>
+        <v>5.54833513221618</v>
       </c>
       <c r="D18">
-        <v>85.118968174572501</v>
+        <v>10.9377981211906</v>
       </c>
       <c r="E18">
-        <v>4.1582064783472701</v>
+        <v>1.2520633936749701</v>
       </c>
       <c r="F18">
-        <v>66.269204650542093</v>
+        <v>17.572339232378901</v>
       </c>
       <c r="G18">
-        <v>1.9885654697995501</v>
+        <v>0.52294039663778702</v>
       </c>
       <c r="H18">
-        <v>50.682459178720002</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>23.486863841748999</v>
+      </c>
+      <c r="I18">
+        <v>-1.91250657480905</v>
+      </c>
+      <c r="J18">
+        <v>0.83722312530660403</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>8</v>
       </c>
@@ -2591,25 +3544,31 @@
         <v>36</v>
       </c>
       <c r="C19">
-        <v>12.6670735192263</v>
+        <v>5.4635976264752202</v>
       </c>
       <c r="D19">
-        <v>113.16565662919101</v>
+        <v>4.3055182785194903</v>
       </c>
       <c r="E19">
-        <v>4.2474793439328602</v>
+        <v>1.24990611993794</v>
       </c>
       <c r="F19">
-        <v>123.091679006717</v>
+        <v>18.844388223606401</v>
       </c>
       <c r="G19">
-        <v>2.0407414068473302</v>
+        <v>0.52663439663696598</v>
       </c>
       <c r="H19">
-        <v>137.53900058894601</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>32.607896734475098</v>
+      </c>
+      <c r="I19">
+        <v>-14.256171407604199</v>
+      </c>
+      <c r="J19">
+        <v>0.803877527412028</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>7</v>
       </c>
@@ -2617,25 +3576,31 @@
         <v>36</v>
       </c>
       <c r="C20">
-        <v>12.5564537726205</v>
+        <v>5.5358720502600303</v>
       </c>
       <c r="D20">
-        <v>91.640439158138193</v>
+        <v>10.094129555691</v>
       </c>
       <c r="E20">
-        <v>4.1822037789523101</v>
+        <v>1.2527627412573199</v>
       </c>
       <c r="F20">
-        <v>79.468378970673896</v>
+        <v>18.347595088783098</v>
       </c>
       <c r="G20">
-        <v>2.0022065572862999</v>
+        <v>0.52415207638914296</v>
       </c>
       <c r="H20">
-        <v>70.608473205183699</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>25.7790287192941</v>
+      </c>
+      <c r="I20">
+        <v>-3.7834628368867498</v>
+      </c>
+      <c r="J20">
+        <v>0.83178761107612398</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>9</v>
       </c>
@@ -2643,25 +3608,31 @@
         <v>36</v>
       </c>
       <c r="C21">
-        <v>12.5517544923092</v>
+        <v>5.5232699771311804</v>
       </c>
       <c r="D21">
-        <v>92.259886174847793</v>
+        <v>9.1295821492606297</v>
       </c>
       <c r="E21">
-        <v>4.1829475885494798</v>
+        <v>1.2516020094135401</v>
       </c>
       <c r="F21">
-        <v>80.705644316190003</v>
+        <v>17.985190607705601</v>
       </c>
       <c r="G21">
-        <v>2.0034139009629501</v>
+        <v>0.52434373084310903</v>
       </c>
       <c r="H21">
-        <v>73.074121408882405</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>26.336894077588902</v>
+      </c>
+      <c r="I21">
+        <v>-5.5231217389472302</v>
+      </c>
+      <c r="J21">
+        <v>0.82691386934122102</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>10</v>
       </c>
@@ -2669,25 +3640,31 @@
         <v>36</v>
       </c>
       <c r="C22">
-        <v>12.490226515314699</v>
+        <v>5.6119825340455902</v>
       </c>
       <c r="D22">
-        <v>79.442827948923096</v>
+        <v>15.5568590322536</v>
       </c>
       <c r="E22">
-        <v>4.1463358566009196</v>
+        <v>1.2719189458234801</v>
       </c>
       <c r="F22">
-        <v>57.914191697663703</v>
+        <v>25.6581977557504</v>
       </c>
       <c r="G22">
-        <v>1.9847209886939701</v>
+        <v>0.53623613968750194</v>
       </c>
       <c r="H22">
-        <v>43.604464558063803</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>39.269411978856098</v>
+      </c>
+      <c r="I22">
+        <v>2.8341151029912499</v>
+      </c>
+      <c r="J22">
+        <v>0.851644293857301</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>11</v>
       </c>
@@ -2695,25 +3672,31 @@
         <v>36</v>
       </c>
       <c r="C23">
-        <v>12.7047580260835</v>
+        <v>5.8166522657457698</v>
       </c>
       <c r="D23">
-        <v>96.074880752610099</v>
+        <v>30.603730057832198</v>
       </c>
       <c r="E23">
-        <v>4.1591923180979897</v>
+        <v>1.3364385232365401</v>
       </c>
       <c r="F23">
-        <v>61.545833512479902</v>
+        <v>52.730135299082299</v>
       </c>
       <c r="G23">
-        <v>1.98106841799883</v>
+        <v>0.56914999220891305</v>
       </c>
       <c r="H23">
-        <v>38.759774563325102</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>80.412834541766998</v>
+      </c>
+      <c r="I23">
+        <v>7.8453238562851402</v>
+      </c>
+      <c r="J23">
+        <v>0.86755067881605097</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>12</v>
       </c>
@@ -2721,25 +3704,31 @@
         <v>36</v>
       </c>
       <c r="C24">
-        <v>12.482889268767099</v>
+        <v>5.5985806170975803</v>
       </c>
       <c r="D24">
-        <v>78.826268381373893</v>
+        <v>14.5016716897262</v>
       </c>
       <c r="E24">
-        <v>4.1401076200791396</v>
+        <v>1.2617380288169799</v>
       </c>
       <c r="F24">
-        <v>55.162779377454299</v>
+        <v>21.1134106483448</v>
       </c>
       <c r="G24">
-        <v>1.9778511666876</v>
+        <v>0.52686850022717402</v>
       </c>
       <c r="H24">
-        <v>34.863708894695797</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+        <v>27.382435589819298</v>
+      </c>
+      <c r="I24">
+        <v>2.51401455023696</v>
+      </c>
+      <c r="J24">
+        <v>0.850655130555378</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>29</v>
       </c>
@@ -2747,7 +3736,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>30</v>
       </c>
@@ -2755,37 +3744,50 @@
         <v>37</v>
       </c>
       <c r="C26">
-        <v>11.4383450056322</v>
+        <v>5.6764675158573299</v>
       </c>
       <c r="D26">
-        <v>-8.2907480192294294</v>
+        <v>7.5077860222692498</v>
       </c>
       <c r="E26">
-        <v>3.9717488860538102</v>
+        <v>1.2753904629780699</v>
       </c>
       <c r="F26">
-        <v>-8.4827721199104893</v>
+        <v>11.388571489914501</v>
       </c>
       <c r="G26">
-        <v>1.93944630809244</v>
+        <v>0.53294102312719405</v>
       </c>
       <c r="H26">
-        <v>-6.6784586301151698</v>
+        <v>17.1908399626004</v>
+      </c>
+      <c r="I26">
+        <v>18.9014044107759</v>
+      </c>
+      <c r="J26">
+        <v>1.03936327231345</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H26" xr:uid="{66EF8D6B-AAC7-4D47-8A22-E3B6AC50568B}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="500 Mt"/>
-      </filters>
-    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A14:H24">
       <sortCondition ref="A1:A26"/>
     </sortState>
   </autoFilter>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="B35:Z35">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="num" val="0"/>
+        <cfvo type="max"/>
+        <color rgb="FF00B050"/>
+        <color theme="0"/>
+        <color rgb="FFC00000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:D26 F2:F26 H2:I26">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -2797,7 +3799,688 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F26">
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6EDCC38-97F2-44B2-A211-84A041F26FA0}">
+  <dimension ref="A1:O23"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F1" t="s">
+        <v>53</v>
+      </c>
+      <c r="G1" t="s">
+        <v>50</v>
+      </c>
+      <c r="H1" t="s">
+        <v>51</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="L1">
+        <f>CORREL(D2:D23,F2:F23)</f>
+        <v>0.67272727272727262</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="O1">
+        <f>CORREL(C2:C23,H2:H23)</f>
+        <v>3.8878507412835051E-2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2">
+        <v>-0.70390616075908496</v>
+      </c>
+      <c r="D2">
+        <v>8</v>
+      </c>
+      <c r="E2">
+        <v>18.574625943324801</v>
+      </c>
+      <c r="F2">
+        <v>10</v>
+      </c>
+      <c r="G2">
+        <v>7.3634914210611901</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>10</v>
+      </c>
+      <c r="E3">
+        <v>17.3728711500404</v>
+      </c>
+      <c r="F3">
+        <v>9</v>
+      </c>
+      <c r="G3">
+        <v>7.9854624669163199</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4">
+        <v>-0.78055119327006905</v>
+      </c>
+      <c r="D4">
+        <v>7</v>
+      </c>
+      <c r="E4">
+        <v>10.5657233468163</v>
+      </c>
+      <c r="F4">
+        <v>5</v>
+      </c>
+      <c r="G4">
+        <v>12.943976807287701</v>
+      </c>
+      <c r="H4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5">
+        <v>-3.7041148122252601</v>
+      </c>
+      <c r="D5">
+        <v>5</v>
+      </c>
+      <c r="E5">
+        <v>6.9142507501659596</v>
+      </c>
+      <c r="F5">
+        <v>2</v>
+      </c>
+      <c r="G5">
+        <v>16.816335761750899</v>
+      </c>
+      <c r="H5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6">
+        <v>-4.6760340109967</v>
+      </c>
+      <c r="D6">
+        <v>2</v>
+      </c>
+      <c r="E6">
+        <v>9.1295821492606297</v>
+      </c>
+      <c r="F6">
+        <v>3</v>
+      </c>
+      <c r="G6">
+        <v>18.019593931069998</v>
+      </c>
+      <c r="H6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7">
+        <v>-0.79606851539385404</v>
+      </c>
+      <c r="D7">
+        <v>6</v>
+      </c>
+      <c r="E7">
+        <v>14.5016716897262</v>
+      </c>
+      <c r="F7">
+        <v>7</v>
+      </c>
+      <c r="G7">
+        <v>18.068472816125901</v>
+      </c>
+      <c r="H7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8">
+        <v>-6.2792075696240897</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>4.3055182785194903</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <v>20.904336245338801</v>
+      </c>
+      <c r="H8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9">
+        <v>-4.5270896828626404</v>
+      </c>
+      <c r="D9">
+        <v>3</v>
+      </c>
+      <c r="E9">
+        <v>10.094129555691</v>
+      </c>
+      <c r="F9">
+        <v>4</v>
+      </c>
+      <c r="G9">
+        <v>21.4277299143567</v>
+      </c>
+      <c r="H9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10">
+        <v>-0.43719754556903001</v>
+      </c>
+      <c r="D10">
+        <v>9</v>
+      </c>
+      <c r="E10">
+        <v>15.5568590322536</v>
+      </c>
+      <c r="F10">
+        <v>8</v>
+      </c>
+      <c r="G10">
+        <v>30.32001009859</v>
+      </c>
+      <c r="H10">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11">
+        <v>-3.9166135590809201</v>
+      </c>
+      <c r="D11">
+        <v>4</v>
+      </c>
+      <c r="E11">
+        <v>10.9377981211906</v>
+      </c>
+      <c r="F11">
+        <v>6</v>
+      </c>
+      <c r="G11">
+        <v>33.8032802979519</v>
+      </c>
+      <c r="H11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12">
+        <v>3.6940786172137897E-2</v>
+      </c>
+      <c r="D12">
+        <v>11</v>
+      </c>
+      <c r="E12">
+        <v>30.603730057832198</v>
+      </c>
+      <c r="F12">
+        <v>11</v>
+      </c>
+      <c r="G12">
+        <v>93.382246268824602</v>
+      </c>
+      <c r="H12">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" t="s">
+        <v>34</v>
+      </c>
+      <c r="C13">
+        <v>-1.7952663161307201</v>
+      </c>
+      <c r="D13">
+        <v>4</v>
+      </c>
+      <c r="E13">
+        <v>11.080702210154501</v>
+      </c>
+      <c r="F13">
+        <v>4</v>
+      </c>
+      <c r="G13">
+        <v>12.1687368263228</v>
+      </c>
+      <c r="H13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>1</v>
+      </c>
+      <c r="B14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14">
+        <v>-0.55420087336513202</v>
+      </c>
+      <c r="D14">
+        <v>7</v>
+      </c>
+      <c r="E14">
+        <v>7.9722193986204699</v>
+      </c>
+      <c r="F14">
+        <v>3</v>
+      </c>
+      <c r="G14">
+        <v>15.427706085558601</v>
+      </c>
+      <c r="H14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15">
+        <v>-3.2383964853381602</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15">
+        <v>13.3924163736789</v>
+      </c>
+      <c r="F15">
+        <v>8</v>
+      </c>
+      <c r="G15">
+        <v>17.572339232378901</v>
+      </c>
+      <c r="H15">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16">
+        <v>0</v>
+      </c>
+      <c r="D16">
+        <v>10</v>
+      </c>
+      <c r="E16">
+        <v>17.279164053851499</v>
+      </c>
+      <c r="F16">
+        <v>10</v>
+      </c>
+      <c r="G16">
+        <v>17.985190607705601</v>
+      </c>
+      <c r="H16">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17">
+        <v>-2.2891584853534401</v>
+      </c>
+      <c r="D17">
+        <v>2</v>
+      </c>
+      <c r="E17">
+        <v>11.804833462263</v>
+      </c>
+      <c r="F17">
+        <v>5</v>
+      </c>
+      <c r="G17">
+        <v>18.347595088783098</v>
+      </c>
+      <c r="H17">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B18" t="s">
+        <v>34</v>
+      </c>
+      <c r="C18">
+        <v>-2.2172361920194099</v>
+      </c>
+      <c r="D18">
+        <v>3</v>
+      </c>
+      <c r="E18">
+        <v>12.090518117610101</v>
+      </c>
+      <c r="F18">
+        <v>6</v>
+      </c>
+      <c r="G18">
+        <v>18.844388223606401</v>
+      </c>
+      <c r="H18">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" t="s">
+        <v>34</v>
+      </c>
+      <c r="C19">
+        <v>-0.10194222025196401</v>
+      </c>
+      <c r="D19">
+        <v>8</v>
+      </c>
+      <c r="E19">
+        <v>13.3113794026041</v>
+      </c>
+      <c r="F19">
+        <v>7</v>
+      </c>
+      <c r="G19">
+        <v>21.1134106483448</v>
+      </c>
+      <c r="H19">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>6</v>
+      </c>
+      <c r="B20" t="s">
+        <v>34</v>
+      </c>
+      <c r="C20">
+        <v>-1.20099872998618</v>
+      </c>
+      <c r="D20">
+        <v>5</v>
+      </c>
+      <c r="E20">
+        <v>3.27434679522118</v>
+      </c>
+      <c r="F20">
+        <v>2</v>
+      </c>
+      <c r="G20">
+        <v>21.891315429941098</v>
+      </c>
+      <c r="H20">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>2</v>
+      </c>
+      <c r="B21" t="s">
+        <v>34</v>
+      </c>
+      <c r="C21">
+        <v>-0.55690592949661299</v>
+      </c>
+      <c r="D21">
+        <v>6</v>
+      </c>
+      <c r="E21">
+        <v>4.18215697221197E-2</v>
+      </c>
+      <c r="F21">
+        <v>1</v>
+      </c>
+      <c r="G21">
+        <v>24.3236703991907</v>
+      </c>
+      <c r="H21">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>10</v>
+      </c>
+      <c r="B22" t="s">
+        <v>34</v>
+      </c>
+      <c r="C22">
+        <v>-3.1121273134907899E-2</v>
+      </c>
+      <c r="D22">
+        <v>9</v>
+      </c>
+      <c r="E22">
+        <v>16.858636173362701</v>
+      </c>
+      <c r="F22">
+        <v>9</v>
+      </c>
+      <c r="G22">
+        <v>25.6581977557504</v>
+      </c>
+      <c r="H22">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>11</v>
+      </c>
+      <c r="B23" t="s">
+        <v>34</v>
+      </c>
+      <c r="C23">
+        <v>4.9027927127704499E-2</v>
+      </c>
+      <c r="D23">
+        <v>11</v>
+      </c>
+      <c r="E23">
+        <v>58.794583510587898</v>
+      </c>
+      <c r="F23">
+        <v>11</v>
+      </c>
+      <c r="G23">
+        <v>52.730135299082299</v>
+      </c>
+      <c r="H23">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H23" xr:uid="{C6EDCC38-97F2-44B2-A211-84A041F26FA0}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H12">
+      <sortCondition ref="G1:G23"/>
+    </sortState>
+  </autoFilter>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="C2:C12">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="num" val="-1"/>
+        <cfvo type="max"/>
+        <color theme="6"/>
+        <color theme="0"/>
+        <color rgb="FFC00000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C13:C23">
+    <cfRule type="colorScale" priority="26">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="num" val="-1"/>
+        <cfvo type="max"/>
+        <color theme="6"/>
+        <color theme="0"/>
+        <color rgb="FFC00000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2:E12">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="num" val="0"/>
+        <cfvo type="max"/>
+        <color rgb="FF00B050"/>
+        <color theme="0"/>
+        <color rgb="FFC00000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E13:E23">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="num" val="0"/>
+        <cfvo type="max"/>
+        <color rgb="FF00B050"/>
+        <color theme="0"/>
+        <color rgb="FFC00000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G12">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -2809,505 +4492,20 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6EDCC38-97F2-44B2-A211-84A041F26FA0}">
-  <dimension ref="A1:J23"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.5703125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D1" t="s">
-        <v>46</v>
-      </c>
-      <c r="E1" t="s">
-        <v>45</v>
-      </c>
-      <c r="F1" t="s">
-        <v>47</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="J1">
-        <f>CORREL(D2:D23,F2:F23)</f>
-        <v>-0.51818181818181808</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C2" s="4">
-        <v>-0.49275627100000002</v>
-      </c>
-      <c r="D2">
-        <v>8</v>
-      </c>
-      <c r="E2">
-        <v>44.141849009060799</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>34</v>
-      </c>
-      <c r="C3" s="4">
-        <v>-0.44834000499999999</v>
-      </c>
-      <c r="D3">
-        <v>5</v>
-      </c>
-      <c r="E3">
-        <v>4.3232246062359998</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>36</v>
-      </c>
-      <c r="C4" s="4">
-        <v>-0.96473474699999995</v>
-      </c>
-      <c r="D4">
-        <v>5</v>
-      </c>
-      <c r="E4">
-        <v>47.922213765437903</v>
-      </c>
-      <c r="F4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" t="s">
-        <v>36</v>
-      </c>
-      <c r="C5" s="4">
-        <v>-0.140659303879175</v>
-      </c>
-      <c r="D5">
-        <v>9</v>
-      </c>
-      <c r="E5">
-        <v>55.162779377454299</v>
-      </c>
-      <c r="F5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C6" s="4">
-        <v>-0.49462211401961598</v>
-      </c>
-      <c r="D6">
-        <v>7</v>
-      </c>
-      <c r="E6">
-        <v>57.914191697663703</v>
-      </c>
-      <c r="F6">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" t="s">
-        <v>36</v>
-      </c>
-      <c r="C7" s="4">
-        <v>0</v>
-      </c>
-      <c r="D7">
-        <v>10</v>
-      </c>
-      <c r="E7">
-        <v>60.039008352776797</v>
-      </c>
-      <c r="F7">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" t="s">
-        <v>34</v>
-      </c>
-      <c r="C8" s="4">
-        <v>-0.44495082200000002</v>
-      </c>
-      <c r="D8">
-        <v>6</v>
-      </c>
-      <c r="E8">
-        <v>18.813043557568299</v>
-      </c>
-      <c r="F8">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>1</v>
-      </c>
-      <c r="B9" t="s">
-        <v>34</v>
-      </c>
-      <c r="C9" s="4">
-        <v>-0.358220919541823</v>
-      </c>
-      <c r="D9">
-        <v>7</v>
-      </c>
-      <c r="E9">
-        <v>20.498026403063999</v>
-      </c>
-      <c r="F9">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10" t="s">
-        <v>36</v>
-      </c>
-      <c r="C10" s="4">
-        <v>2.1860439999999998E-2</v>
-      </c>
-      <c r="D10">
-        <v>11</v>
-      </c>
-      <c r="E10">
-        <v>61.545833512479902</v>
-      </c>
-      <c r="F10">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" s="4">
-        <v>-1.0328987359064601E-2</v>
-      </c>
-      <c r="D11">
-        <v>8</v>
-      </c>
-      <c r="E11">
-        <v>25.9717569864757</v>
-      </c>
-      <c r="F11">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" t="s">
-        <v>36</v>
-      </c>
-      <c r="C12" s="4">
-        <v>-0.97789037099999998</v>
-      </c>
-      <c r="D12">
-        <v>4</v>
-      </c>
-      <c r="E12">
-        <v>66.269204650542093</v>
-      </c>
-      <c r="F12">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>7</v>
-      </c>
-      <c r="B13" t="s">
-        <v>36</v>
-      </c>
-      <c r="C13" s="4">
-        <v>-1.3696436649999999</v>
-      </c>
-      <c r="D13">
-        <v>3</v>
-      </c>
-      <c r="E13">
-        <v>79.468378970673896</v>
-      </c>
-      <c r="F13">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" t="s">
-        <v>34</v>
-      </c>
-      <c r="C14" s="4">
-        <v>0</v>
-      </c>
-      <c r="D14">
-        <v>10</v>
-      </c>
-      <c r="E14">
-        <v>35.393894665297204</v>
-      </c>
-      <c r="F14">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>10</v>
-      </c>
-      <c r="B15" t="s">
-        <v>34</v>
-      </c>
-      <c r="C15" s="4">
-        <v>-9.9402557076976408E-4</v>
-      </c>
-      <c r="D15">
-        <v>9</v>
-      </c>
-      <c r="E15">
-        <v>37.202899164071297</v>
-      </c>
-      <c r="F15">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>5</v>
-      </c>
-      <c r="B16" t="s">
-        <v>34</v>
-      </c>
-      <c r="C16" s="4">
-        <v>-0.52369600900000002</v>
-      </c>
-      <c r="D16">
-        <v>4</v>
-      </c>
-      <c r="E16">
-        <v>53.400101276959496</v>
-      </c>
-      <c r="F16">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>9</v>
-      </c>
-      <c r="B17" t="s">
-        <v>36</v>
-      </c>
-      <c r="C17" s="4">
-        <v>-1.5359190410000001</v>
-      </c>
-      <c r="D17">
-        <v>2</v>
-      </c>
-      <c r="E17">
-        <v>80.705644316190003</v>
-      </c>
-      <c r="F17">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>11</v>
-      </c>
-      <c r="B18" t="s">
-        <v>34</v>
-      </c>
-      <c r="C18" s="4">
-        <v>2.0065428E-2</v>
-      </c>
-      <c r="D18">
-        <v>11</v>
-      </c>
-      <c r="E18">
-        <v>78.907141092873204</v>
-      </c>
-      <c r="F18">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>7</v>
-      </c>
-      <c r="B19" t="s">
-        <v>34</v>
-      </c>
-      <c r="C19" s="4">
-        <v>-0.78533132827192897</v>
-      </c>
-      <c r="D19">
-        <v>3</v>
-      </c>
-      <c r="E19">
-        <v>82.357389931911399</v>
-      </c>
-      <c r="F19">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>9</v>
-      </c>
-      <c r="B20" t="s">
-        <v>34</v>
-      </c>
-      <c r="C20" s="4">
-        <v>-0.89245744999999999</v>
-      </c>
-      <c r="D20">
-        <v>2</v>
-      </c>
-      <c r="E20">
-        <v>85.278269416212396</v>
-      </c>
-      <c r="F20">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>2</v>
-      </c>
-      <c r="B21" t="s">
-        <v>36</v>
-      </c>
-      <c r="C21" s="4">
-        <v>-0.59780631626324898</v>
-      </c>
-      <c r="D21">
-        <v>6</v>
-      </c>
-      <c r="E21">
-        <v>88.765537100189803</v>
-      </c>
-      <c r="F21">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>8</v>
-      </c>
-      <c r="B22" t="s">
-        <v>34</v>
-      </c>
-      <c r="C22" s="4">
-        <v>-1.76060591606728</v>
-      </c>
-      <c r="D22">
-        <v>1</v>
-      </c>
-      <c r="E22">
-        <v>179.857163829526</v>
-      </c>
-      <c r="F22">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>8</v>
-      </c>
-      <c r="B23" t="s">
-        <v>36</v>
-      </c>
-      <c r="C23" s="4">
-        <v>-2.8798107700000002</v>
-      </c>
-      <c r="D23">
-        <v>1</v>
-      </c>
-      <c r="E23">
-        <v>123.091679006717</v>
-      </c>
-      <c r="F23">
-        <v>11</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:F23" xr:uid="{C6EDCC38-97F2-44B2-A211-84A041F26FA0}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:F22">
-      <sortCondition ref="E1:E23"/>
-    </sortState>
-  </autoFilter>
-  <phoneticPr fontId="3" type="noConversion"/>
-  <conditionalFormatting sqref="C13:C23">
-    <cfRule type="colorScale" priority="7">
+  <conditionalFormatting sqref="G13:G23">
+    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
+        <cfvo type="num" val="0"/>
         <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
+        <color rgb="FF00B050"/>
+        <color theme="0"/>
+        <color rgb="FFC00000"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C11:C23">
-    <cfRule type="colorScale" priority="6">
+  <conditionalFormatting sqref="J3:J13">
+    <cfRule type="colorScale" priority="27">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="num" val="-1"/>
@@ -3318,40 +4516,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C10">
-    <cfRule type="colorScale" priority="15">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="num" val="-1"/>
-        <cfvo type="max"/>
-        <color theme="6"/>
-        <color theme="0"/>
-        <color rgb="FFC00000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C4:C10">
-    <cfRule type="colorScale" priority="17">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E23">
-    <cfRule type="colorScale" priority="18">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="num" val="0"/>
-        <cfvo type="max"/>
-        <color rgb="FF00B050"/>
-        <color theme="0"/>
-        <color rgb="FFC00000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update procurement data analysis
</commit_message>
<xml_diff>
--- a/data/data_analysis/policy_effectiveness.xlsx
+++ b/data/data_analysis/policy_effectiveness.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\data\data_analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99BCAFAF-FC8C-4A8E-A96D-D06598DE66D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4876D8D1-E0E9-48E5-8ABD-177D1C1E9261}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{5B094011-67C9-461D-BBBF-A6D3FE50B4AB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{5B094011-67C9-461D-BBBF-A6D3FE50B4AB}"/>
   </bookViews>
   <sheets>
     <sheet name="Low" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="67">
   <si>
     <t>Scenario</t>
   </si>
@@ -100,18 +100,6 @@
   </si>
   <si>
     <t>High Baseline</t>
-  </si>
-  <si>
-    <t>Benefits | 3.0%</t>
-  </si>
-  <si>
-    <t>Costs | 3.0%</t>
-  </si>
-  <si>
-    <t>Benefits/Costs | 3.0%</t>
-  </si>
-  <si>
-    <t>Benefits-Costs | 3.0%</t>
   </si>
   <si>
     <t>Benefits | 12.0%</t>
@@ -248,13 +236,37 @@
   <si>
     <t>500Mt</t>
   </si>
+  <si>
+    <t>Marginal</t>
+  </si>
+  <si>
+    <t>2% Benefits</t>
+  </si>
+  <si>
+    <t>2% Costs</t>
+  </si>
+  <si>
+    <t>12% Benefits</t>
+  </si>
+  <si>
+    <t>12% Costs</t>
+  </si>
+  <si>
+    <t>20% Benefits</t>
+  </si>
+  <si>
+    <t>20% Costs</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="4">
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -307,11 +319,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5616,7 +5631,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="8191500" y="290511"/>
+              <a:off x="10096500" y="290511"/>
               <a:ext cx="4572000" cy="5662613"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -6331,19 +6346,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1B4DBF1-F2D7-44F8-977D-1BE3C41C10B1}">
-  <dimension ref="A1:AP16"/>
+  <dimension ref="A1:AP34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="21" style="5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="21" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="22.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6352,43 +6370,43 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D1" t="s">
-        <v>44</v>
+        <v>39</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>40</v>
       </c>
       <c r="E1" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="F1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J1" t="s">
         <v>19</v>
       </c>
-      <c r="G1" t="s">
+      <c r="K1" t="s">
         <v>20</v>
       </c>
-      <c r="H1" t="s">
+      <c r="L1" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="I1" t="s">
+      <c r="M1" t="s">
         <v>22</v>
       </c>
-      <c r="J1" t="s">
+      <c r="N1" t="s">
         <v>23</v>
-      </c>
-      <c r="K1" t="s">
-        <v>24</v>
-      </c>
-      <c r="L1" t="s">
-        <v>25</v>
-      </c>
-      <c r="M1" t="s">
-        <v>26</v>
-      </c>
-      <c r="N1" t="s">
-        <v>27</v>
       </c>
       <c r="O1" s="3"/>
       <c r="P1" s="3"/>
@@ -6423,47 +6441,50 @@
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="6">
         <v>-40991.392169844003</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="6">
         <v>73964.863896627197</v>
       </c>
-      <c r="D2">
-        <v>-0.55420087336513202</v>
-      </c>
-      <c r="E2" s="1">
+      <c r="D2" s="5">
+        <f>B2/C2</f>
+        <v>-0.55420087336513324</v>
+      </c>
+      <c r="E2" s="6">
         <f>B2+C2</f>
         <v>32973.471726783195</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F2" s="6">
         <v>-11644.658803537901</v>
       </c>
-      <c r="G2" s="1">
+      <c r="G2" s="6">
         <v>32506.920082813402</v>
       </c>
-      <c r="H2">
-        <v>-0.358220919541823</v>
-      </c>
-      <c r="I2" s="1">
+      <c r="H2" s="5">
+        <f>F2/G2</f>
+        <v>-0.35822091954182089</v>
+      </c>
+      <c r="I2" s="6">
         <f>F2+G2</f>
         <v>20862.261279275503</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="6">
         <v>-5002.1063151110802</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="6">
         <v>20078.072923277199</v>
       </c>
-      <c r="L2">
-        <v>-0.24913278949754</v>
-      </c>
-      <c r="M2" s="1">
+      <c r="L2" s="5">
+        <f>J2/K2</f>
+        <v>-0.2491327894975402</v>
+      </c>
+      <c r="M2" s="6">
         <f>J2+K2</f>
         <v>15075.96660816612</v>
       </c>
       <c r="N2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="O2" s="3"/>
       <c r="P2" s="3"/>
@@ -6498,47 +6519,50 @@
       <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="6">
         <v>-190307.317572267</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="6">
         <v>341722.55580809899</v>
       </c>
-      <c r="D3">
-        <v>-0.55690592949661299</v>
-      </c>
-      <c r="E3" s="1">
-        <f t="shared" ref="E3:E15" si="0">B3+C3</f>
+      <c r="D3" s="5">
+        <f t="shared" ref="D3:D15" si="0">B3/C3</f>
+        <v>-0.55690592949661133</v>
+      </c>
+      <c r="E3" s="6">
+        <f t="shared" ref="E3:E15" si="1">B3+C3</f>
         <v>151415.23823583199</v>
       </c>
-      <c r="F3" s="1">
+      <c r="F3" s="6">
         <v>-30848.8092279228</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G3" s="6">
         <v>68806.729018270402</v>
       </c>
-      <c r="H3">
-        <v>-0.44834000493950898</v>
-      </c>
-      <c r="I3" s="1">
-        <f t="shared" ref="I3:I15" si="1">F3+G3</f>
+      <c r="H3" s="5">
+        <f t="shared" ref="H3:H15" si="2">F3/G3</f>
+        <v>-0.44834000493950887</v>
+      </c>
+      <c r="I3" s="6">
+        <f t="shared" ref="I3:I15" si="3">F3+G3</f>
         <v>37957.919790347602</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="6">
         <v>-9394.0921605190797</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="6">
         <v>28774.349079517</v>
       </c>
-      <c r="L3">
-        <v>-0.32647453238850899</v>
-      </c>
-      <c r="M3" s="1">
-        <f t="shared" ref="M3:M15" si="2">J3+K3</f>
+      <c r="L3" s="5">
+        <f t="shared" ref="L3:L15" si="4">J3/K3</f>
+        <v>-0.32647453238851049</v>
+      </c>
+      <c r="M3" s="6">
+        <f t="shared" ref="M3:M15" si="5">J3+K3</f>
         <v>19380.256918997919</v>
       </c>
       <c r="N3" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="O3" s="3"/>
       <c r="P3" s="3"/>
@@ -6573,47 +6597,50 @@
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="6">
         <v>-112322.040618713</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="6">
         <v>56741.484497939098</v>
       </c>
-      <c r="D4">
-        <v>-1.9795400422206499</v>
-      </c>
-      <c r="E4" s="1">
+      <c r="D4" s="5">
         <f t="shared" si="0"/>
+        <v>-1.9795400422206548</v>
+      </c>
+      <c r="E4" s="6">
+        <f t="shared" si="1"/>
         <v>-55580.556120773901</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F4" s="6">
         <v>-48889.259790475502</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G4" s="6">
         <v>28709.564463483799</v>
       </c>
-      <c r="H4">
-        <v>-1.7028910296656901</v>
-      </c>
-      <c r="I4" s="1">
-        <f t="shared" si="1"/>
+      <c r="H4" s="5">
+        <f t="shared" si="2"/>
+        <v>-1.7028910296656925</v>
+      </c>
+      <c r="I4" s="6">
+        <f t="shared" si="3"/>
         <v>-20179.695326991703</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="6">
         <v>-28941.9181735079</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="6">
         <v>18022.833509243501</v>
       </c>
-      <c r="L4">
-        <v>-1.6058472802661199</v>
-      </c>
-      <c r="M4" s="1">
-        <f t="shared" si="2"/>
+      <c r="L4" s="5">
+        <f t="shared" si="4"/>
+        <v>-1.6058472802661274</v>
+      </c>
+      <c r="M4" s="6">
+        <f t="shared" si="5"/>
         <v>-10919.084664264399</v>
       </c>
       <c r="N4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
@@ -6648,529 +6675,1433 @@
       <c r="A5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="6">
         <v>-611711.12191152503</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="6">
         <v>632967.09479468397</v>
       </c>
-      <c r="D5">
-        <v>-0.96641851834327297</v>
-      </c>
-      <c r="E5" s="1">
+      <c r="D5" s="5">
         <f t="shared" si="0"/>
+        <v>-0.96641851834327386</v>
+      </c>
+      <c r="E5" s="6">
+        <f t="shared" si="1"/>
         <v>21255.972883158945</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5" s="6">
         <v>-124837.11295495099</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G5" s="6">
         <v>125786.37310764899</v>
       </c>
-      <c r="H5">
-        <v>-0.99245339436025104</v>
-      </c>
-      <c r="I5" s="1">
-        <f t="shared" si="1"/>
+      <c r="H5" s="5">
+        <f t="shared" si="2"/>
+        <v>-0.99245339436024904</v>
+      </c>
+      <c r="I5" s="6">
+        <f t="shared" si="3"/>
         <v>949.26015269799973</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="6">
         <v>-49513.350620204001</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="6">
         <v>47841.174083838101</v>
       </c>
-      <c r="L5">
-        <v>-1.0349526651130101</v>
-      </c>
-      <c r="M5" s="1">
-        <f t="shared" si="2"/>
+      <c r="L5" s="5">
+        <f t="shared" si="4"/>
+        <v>-1.0349526651130161</v>
+      </c>
+      <c r="M5" s="6">
+        <f t="shared" si="5"/>
         <v>-1672.1765363658997</v>
       </c>
       <c r="N5" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="6">
         <v>-23639.052484741402</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="6">
         <v>19682.8288777735</v>
       </c>
-      <c r="D6">
-        <v>-1.20099872998618</v>
-      </c>
-      <c r="E6" s="1">
+      <c r="D6" s="5">
         <f t="shared" si="0"/>
+        <v>-1.2009987299861862</v>
+      </c>
+      <c r="E6" s="6">
+        <f t="shared" si="1"/>
         <v>-3956.223606967902</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F6" s="6">
         <v>-5718.2312864800897</v>
       </c>
-      <c r="G6" s="1">
+      <c r="G6" s="6">
         <v>15677.5227380697</v>
       </c>
-      <c r="H6">
-        <v>-0.36474074265537498</v>
-      </c>
-      <c r="I6" s="1">
-        <f t="shared" si="1"/>
+      <c r="H6" s="5">
+        <f t="shared" si="2"/>
+        <v>-0.3647407426553762</v>
+      </c>
+      <c r="I6" s="6">
+        <f t="shared" si="3"/>
         <v>9959.29145158961</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="6">
         <v>-2790.36636372676</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="6">
         <v>13463.719299594801</v>
       </c>
-      <c r="L6">
-        <v>-0.207250782761842</v>
-      </c>
-      <c r="M6" s="1">
-        <f t="shared" si="2"/>
+      <c r="L6" s="5">
+        <f t="shared" si="4"/>
+        <v>-0.20725078276184336</v>
+      </c>
+      <c r="M6" s="6">
+        <f t="shared" si="5"/>
         <v>10673.352935868041</v>
       </c>
       <c r="N6" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="1">
+      <c r="B7" s="6">
         <v>-30682.746255407401</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7" s="6">
         <v>17090.916249983798</v>
       </c>
-      <c r="D7">
-        <v>-1.7952663161307201</v>
-      </c>
-      <c r="E7" s="1">
+      <c r="D7" s="5">
         <f t="shared" si="0"/>
+        <v>-1.7952663161307392</v>
+      </c>
+      <c r="E7" s="6">
+        <f t="shared" si="1"/>
         <v>-13591.830005423602</v>
       </c>
-      <c r="F7" s="1">
+      <c r="F7" s="6">
         <v>-6100.3980291768003</v>
       </c>
-      <c r="G7" s="1">
+      <c r="G7" s="6">
         <v>12692.2292408466</v>
       </c>
-      <c r="H7">
-        <v>-0.48064039133048803</v>
-      </c>
-      <c r="I7" s="1">
-        <f t="shared" si="1"/>
+      <c r="H7" s="5">
+        <f t="shared" si="2"/>
+        <v>-0.48064039133049019</v>
+      </c>
+      <c r="I7" s="6">
+        <f t="shared" si="3"/>
         <v>6591.8312116697998</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="6">
         <v>-2360.7973050558699</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="6">
         <v>10689.1346820868</v>
       </c>
-      <c r="L7">
-        <v>-0.220859534028715</v>
-      </c>
-      <c r="M7" s="1">
-        <f t="shared" si="2"/>
+      <c r="L7" s="5">
+        <f t="shared" si="4"/>
+        <v>-0.22085953402871522</v>
+      </c>
+      <c r="M7" s="6">
+        <f t="shared" si="5"/>
         <v>8328.3373770309299</v>
       </c>
       <c r="N7" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="1">
+      <c r="B8" s="6">
         <v>-97079.650583780895</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="6">
         <v>29977.691435656099</v>
       </c>
-      <c r="D8">
-        <v>-3.2383964853381602</v>
-      </c>
-      <c r="E8" s="1">
+      <c r="D8" s="5">
         <f t="shared" si="0"/>
+        <v>-3.2383964853381708</v>
+      </c>
+      <c r="E8" s="6">
+        <f t="shared" si="1"/>
         <v>-67101.959148124792</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F8" s="6">
         <v>-20972.403124771499</v>
       </c>
-      <c r="G8" s="1">
+      <c r="G8" s="6">
         <v>18375.511162999999</v>
       </c>
-      <c r="H8">
-        <v>-1.14132352230834</v>
-      </c>
-      <c r="I8" s="1">
-        <f t="shared" si="1"/>
+      <c r="H8" s="5">
+        <f t="shared" si="2"/>
+        <v>-1.1413235223083464</v>
+      </c>
+      <c r="I8" s="6">
+        <f t="shared" si="3"/>
         <v>-2596.8919617715001</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="6">
         <v>-8406.4334333911793</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="6">
         <v>13832.566021950501</v>
       </c>
-      <c r="L8">
-        <v>-0.60772769275427296</v>
-      </c>
-      <c r="M8" s="1">
-        <f t="shared" si="2"/>
+      <c r="L8" s="5">
+        <f t="shared" si="4"/>
+        <v>-0.60772769275427652</v>
+      </c>
+      <c r="M8" s="6">
+        <f t="shared" si="5"/>
         <v>5426.1325885593214</v>
       </c>
       <c r="N8" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="1">
+      <c r="B9" s="6">
         <v>-43683.1580178394</v>
       </c>
-      <c r="C9" s="1">
+      <c r="C9" s="6">
         <v>19701.6259138606</v>
       </c>
-      <c r="D9">
-        <v>-2.2172361920194099</v>
-      </c>
-      <c r="E9" s="1">
+      <c r="D9" s="5">
         <f t="shared" si="0"/>
+        <v>-2.2172361920194197</v>
+      </c>
+      <c r="E9" s="6">
+        <f t="shared" si="1"/>
         <v>-23981.5321039788</v>
       </c>
-      <c r="F9" s="1">
+      <c r="F9" s="6">
         <v>-9175.9801601351992</v>
       </c>
-      <c r="G9" s="1">
+      <c r="G9" s="6">
         <v>13838.706423644</v>
       </c>
-      <c r="H9">
-        <v>-0.66306632131870602</v>
-      </c>
-      <c r="I9" s="1">
-        <f t="shared" si="1"/>
+      <c r="H9" s="5">
+        <f t="shared" si="2"/>
+        <v>-0.66306632131870791</v>
+      </c>
+      <c r="I9" s="6">
+        <f t="shared" si="3"/>
         <v>4662.7262635088009</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="6">
         <v>-3610.0129557775899</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="6">
         <v>11226.4948888167</v>
       </c>
-      <c r="L9">
-        <v>-0.32156189367473098</v>
-      </c>
-      <c r="M9" s="1">
-        <f t="shared" si="2"/>
+      <c r="L9" s="5">
+        <f t="shared" si="4"/>
+        <v>-0.32156189367473126</v>
+      </c>
+      <c r="M9" s="6">
+        <f t="shared" si="5"/>
         <v>7616.4819330391101</v>
       </c>
       <c r="N9" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="1">
+      <c r="B10" s="6">
         <v>-50470.5551048856</v>
       </c>
-      <c r="C10" s="1">
+      <c r="C10" s="6">
         <v>22047.6456426271</v>
       </c>
-      <c r="D10">
-        <v>-2.2891584853534401</v>
-      </c>
-      <c r="E10" s="1">
+      <c r="D10" s="5">
         <f t="shared" si="0"/>
+        <v>-2.2891584853534388</v>
+      </c>
+      <c r="E10" s="6">
+        <f t="shared" si="1"/>
         <v>-28422.9094622585</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F10" s="6">
         <v>-10472.8845316388</v>
       </c>
-      <c r="G10" s="1">
+      <c r="G10" s="6">
         <v>14865.3551125206</v>
       </c>
-      <c r="H10">
-        <v>-0.70451626970000103</v>
-      </c>
-      <c r="I10" s="1">
-        <f t="shared" si="1"/>
+      <c r="H10" s="5">
+        <f t="shared" si="2"/>
+        <v>-0.70451626969999748</v>
+      </c>
+      <c r="I10" s="6">
+        <f t="shared" si="3"/>
         <v>4392.4705808817998</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="6">
         <v>-4213.4803805597603</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="6">
         <v>12164.270271887701</v>
       </c>
-      <c r="L10">
-        <v>-0.346381680641979</v>
-      </c>
-      <c r="M10" s="1">
-        <f t="shared" si="2"/>
+      <c r="L10" s="5">
+        <f t="shared" si="4"/>
+        <v>-0.34638168064198194</v>
+      </c>
+      <c r="M10" s="6">
+        <f t="shared" si="5"/>
         <v>7950.7898913279405</v>
       </c>
       <c r="N10" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="1">
+      <c r="B11" s="6">
         <v>0</v>
       </c>
-      <c r="C11" s="1">
+      <c r="C11" s="6">
         <v>14486.1268858849</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="5">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="E11" s="1">
-        <f t="shared" si="0"/>
+      <c r="E11" s="6">
+        <f t="shared" si="1"/>
         <v>14486.1268858849</v>
       </c>
-      <c r="F11" s="1">
+      <c r="F11" s="6">
         <v>0</v>
       </c>
-      <c r="G11" s="1">
+      <c r="G11" s="6">
         <v>11511.601320002699</v>
       </c>
-      <c r="H11">
+      <c r="H11" s="5">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="I11" s="1">
-        <f t="shared" si="1"/>
+      <c r="I11" s="6">
+        <f t="shared" si="3"/>
         <v>11511.601320002699</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="6">
         <v>0</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="6">
         <v>9874.8984398431494</v>
       </c>
-      <c r="L11">
+      <c r="L11" s="5">
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="M11" s="1">
-        <f t="shared" si="2"/>
+      <c r="M11" s="6">
+        <f t="shared" si="5"/>
         <v>9874.8984398431494</v>
       </c>
       <c r="N11" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="1">
+      <c r="B12" s="6">
         <v>-1404.5679010868701</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12" s="6">
         <v>45132.0836071905</v>
       </c>
-      <c r="D12">
-        <v>-3.1121273134907899E-2</v>
-      </c>
-      <c r="E12" s="1">
+      <c r="D12" s="5">
         <f t="shared" si="0"/>
+        <v>-3.1121273134907791E-2</v>
+      </c>
+      <c r="E12" s="6">
+        <f t="shared" si="1"/>
         <v>43727.51570610363</v>
       </c>
-      <c r="F12" s="1">
+      <c r="F12" s="6">
         <v>-32.085743248811902</v>
       </c>
-      <c r="G12" s="1">
+      <c r="G12" s="6">
         <v>32278.589396815001</v>
       </c>
-      <c r="H12">
-        <v>-9.9402557076976408E-4</v>
-      </c>
-      <c r="I12" s="1">
-        <f t="shared" si="1"/>
+      <c r="H12" s="5">
+        <f t="shared" si="2"/>
+        <v>-9.9402557076976451E-4</v>
+      </c>
+      <c r="I12" s="6">
+        <f t="shared" si="3"/>
         <v>32246.503653566189</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="6">
         <v>-227.43782558660999</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="6">
         <v>26285.648960687002</v>
       </c>
-      <c r="L12">
-        <v>-8.6525474766389696E-3</v>
-      </c>
-      <c r="M12" s="1">
-        <f t="shared" si="2"/>
+      <c r="L12" s="5">
+        <f t="shared" si="4"/>
+        <v>-8.6525474766389662E-3</v>
+      </c>
+      <c r="M12" s="6">
+        <f t="shared" si="5"/>
         <v>26058.211135100391</v>
       </c>
       <c r="N12" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="1">
+      <c r="B13" s="6">
         <v>40603.4193094004</v>
       </c>
-      <c r="C13" s="1">
+      <c r="C13" s="6">
         <v>828169.20249635505</v>
       </c>
-      <c r="D13">
-        <v>4.9027927127704499E-2</v>
-      </c>
-      <c r="E13" s="1">
+      <c r="D13" s="5">
         <f t="shared" si="0"/>
+        <v>4.9027927127704443E-2</v>
+      </c>
+      <c r="E13" s="6">
+        <f t="shared" si="1"/>
         <v>868772.62180575542</v>
       </c>
-      <c r="F13" s="1">
+      <c r="F13" s="6">
         <v>4460.6170443716501</v>
       </c>
-      <c r="G13" s="1">
+      <c r="G13" s="6">
         <v>222303.607323328</v>
       </c>
-      <c r="H13">
-        <v>2.0065428078654302E-2</v>
-      </c>
-      <c r="I13" s="1">
-        <f t="shared" si="1"/>
+      <c r="H13" s="5">
+        <f t="shared" si="2"/>
+        <v>2.0065428078654322E-2</v>
+      </c>
+      <c r="I13" s="6">
+        <f t="shared" si="3"/>
         <v>226764.22436769964</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="6">
         <v>-1031.07110519603</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="6">
         <v>108783.803081255</v>
       </c>
-      <c r="L13">
-        <v>-9.4781674844175191E-3</v>
-      </c>
-      <c r="M13" s="1">
-        <f t="shared" si="2"/>
+      <c r="L13" s="5">
+        <f t="shared" si="4"/>
+        <v>-9.4781674844175243E-3</v>
+      </c>
+      <c r="M13" s="6">
+        <f t="shared" si="5"/>
         <v>107752.73197605897</v>
       </c>
       <c r="N13" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="1">
+      <c r="B14" s="6">
         <v>-2626.77829541446</v>
       </c>
-      <c r="C14" s="1">
+      <c r="C14" s="6">
         <v>25767.324754375601</v>
       </c>
-      <c r="D14">
-        <v>-0.10194222025196401</v>
-      </c>
-      <c r="E14" s="1">
+      <c r="D14" s="5">
         <f t="shared" si="0"/>
+        <v>-0.10194222025196471</v>
+      </c>
+      <c r="E14" s="6">
+        <f t="shared" si="1"/>
         <v>23140.54645896114</v>
       </c>
-      <c r="F14" s="1">
+      <c r="F14" s="6">
         <v>-184.162683612303</v>
       </c>
-      <c r="G14" s="1">
+      <c r="G14" s="6">
         <v>17829.693968081301</v>
       </c>
-      <c r="H14">
-        <v>-1.0328987359064601E-2</v>
-      </c>
-      <c r="I14" s="1">
-        <f t="shared" si="1"/>
+      <c r="H14" s="5">
+        <f t="shared" si="2"/>
+        <v>-1.0328987359064651E-2</v>
+      </c>
+      <c r="I14" s="6">
+        <f t="shared" si="3"/>
         <v>17645.531284468998</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="6">
         <v>-125.237709722896</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="6">
         <v>14163.2689710182</v>
       </c>
-      <c r="L14">
-        <v>-8.84242966642553E-3</v>
-      </c>
-      <c r="M14" s="1">
-        <f t="shared" si="2"/>
+      <c r="L14" s="5">
+        <f t="shared" si="4"/>
+        <v>-8.8424296664255629E-3</v>
+      </c>
+      <c r="M14" s="6">
+        <f t="shared" si="5"/>
         <v>14038.031261295304</v>
       </c>
       <c r="N14" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>59</v>
-      </c>
-      <c r="B15" s="1">
+        <v>55</v>
+      </c>
+      <c r="B15" s="6">
         <v>-177560.27976733001</v>
       </c>
-      <c r="C15" s="1">
+      <c r="C15" s="6">
         <v>84648.601837562499</v>
       </c>
-      <c r="D15">
-        <v>-2.0976162147138702</v>
-      </c>
-      <c r="E15" s="1">
+      <c r="D15" s="5">
         <f t="shared" si="0"/>
+        <v>-2.0976162147138773</v>
+      </c>
+      <c r="E15" s="6">
+        <f t="shared" si="1"/>
         <v>-92911.677929767509</v>
       </c>
-      <c r="F15" s="1">
+      <c r="F15" s="6">
         <v>-55394.240300793303</v>
       </c>
-      <c r="G15" s="1">
+      <c r="G15" s="6">
         <v>44328.768128424897</v>
       </c>
-      <c r="H15">
-        <v>-1.2496228214668701</v>
-      </c>
-      <c r="I15" s="1">
-        <f t="shared" si="1"/>
+      <c r="H15" s="5">
+        <f t="shared" si="2"/>
+        <v>-1.2496228214668772</v>
+      </c>
+      <c r="I15" s="6">
+        <f t="shared" si="3"/>
         <v>-11065.472172368405</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="6">
         <v>-27847.218892906101</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="6">
         <v>28922.694502216698</v>
       </c>
-      <c r="L15">
-        <v>-0.96281551121635001</v>
-      </c>
-      <c r="M15" s="1">
-        <f t="shared" si="2"/>
+      <c r="L15" s="5">
+        <f t="shared" si="4"/>
+        <v>-0.96281551121635056</v>
+      </c>
+      <c r="M15" s="6">
+        <f t="shared" si="5"/>
         <v>1075.4756093105971</v>
       </c>
       <c r="N15" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" spans="1:42" x14ac:dyDescent="0.25">
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
-      <c r="J16" s="1"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6"/>
+      <c r="I16" s="6"/>
+      <c r="J16" s="6"/>
+      <c r="K16" s="6"/>
+      <c r="M16" s="6"/>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I17" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J17" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="K17" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="L17" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="M17" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="N17" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B18" s="6">
+        <f>B2-B$34</f>
+        <v>-40991.392169844003</v>
+      </c>
+      <c r="C18" s="6">
+        <f>C2-C$34</f>
+        <v>59478.737010742298</v>
+      </c>
+      <c r="D18" s="5">
+        <f>B18/C18</f>
+        <v>-0.68917724602055108</v>
+      </c>
+      <c r="E18" s="6">
+        <f>B18+C18</f>
+        <v>18487.344840898295</v>
+      </c>
+      <c r="F18" s="6">
+        <f>F2-F$34</f>
+        <v>-11644.658803537901</v>
+      </c>
+      <c r="G18" s="6">
+        <f>G2-G$34</f>
+        <v>20995.318762810704</v>
+      </c>
+      <c r="H18" s="5">
+        <f>F18/G18</f>
+        <v>-0.55463119827283802</v>
+      </c>
+      <c r="I18" s="6">
+        <f>F18+G18</f>
+        <v>9350.6599592728035</v>
+      </c>
+      <c r="J18" s="6">
+        <f>J2-J$34</f>
+        <v>-5002.1063151110802</v>
+      </c>
+      <c r="K18" s="6">
+        <f>K2-K$34</f>
+        <v>10203.17448343405</v>
+      </c>
+      <c r="L18" s="5">
+        <f>J18/K18</f>
+        <v>-0.49025000241175304</v>
+      </c>
+      <c r="M18" s="6">
+        <f>J18+K18</f>
+        <v>5201.0681683229695</v>
+      </c>
+      <c r="N18" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>2</v>
+      </c>
+      <c r="B19" s="6">
+        <f t="shared" ref="B19:C19" si="6">B3-B$34</f>
+        <v>-190307.317572267</v>
+      </c>
+      <c r="C19" s="6">
+        <f t="shared" si="6"/>
+        <v>327236.42892221408</v>
+      </c>
+      <c r="D19" s="5">
+        <f t="shared" ref="D19:D31" si="7">B19/C19</f>
+        <v>-0.58155908313467175</v>
+      </c>
+      <c r="E19" s="6">
+        <f t="shared" ref="E19:E31" si="8">B19+C19</f>
+        <v>136929.11134994708</v>
+      </c>
+      <c r="F19" s="6">
+        <f t="shared" ref="F19:G19" si="9">F3-F$34</f>
+        <v>-30848.8092279228</v>
+      </c>
+      <c r="G19" s="6">
+        <f t="shared" si="9"/>
+        <v>57295.127698267701</v>
+      </c>
+      <c r="H19" s="5">
+        <f t="shared" ref="H19:H31" si="10">F19/G19</f>
+        <v>-0.5384194165755477</v>
+      </c>
+      <c r="I19" s="6">
+        <f t="shared" ref="I19:I31" si="11">F19+G19</f>
+        <v>26446.318470344901</v>
+      </c>
+      <c r="J19" s="6">
+        <f t="shared" ref="J19:K19" si="12">J3-J$34</f>
+        <v>-9394.0921605190797</v>
+      </c>
+      <c r="K19" s="6">
+        <f t="shared" si="12"/>
+        <v>18899.450639673851</v>
+      </c>
+      <c r="L19" s="5">
+        <f t="shared" ref="L19:L31" si="13">J19/K19</f>
+        <v>-0.49705636103511602</v>
+      </c>
+      <c r="M19" s="6">
+        <f t="shared" ref="M19:M31" si="14">J19+K19</f>
+        <v>9505.358479154771</v>
+      </c>
+      <c r="N19" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>3</v>
+      </c>
+      <c r="B20" s="6">
+        <f t="shared" ref="B20:C20" si="15">B4-B$34</f>
+        <v>-112322.040618713</v>
+      </c>
+      <c r="C20" s="6">
+        <f t="shared" si="15"/>
+        <v>42255.357612054198</v>
+      </c>
+      <c r="D20" s="5">
+        <f t="shared" si="7"/>
+        <v>-2.6581727611901895</v>
+      </c>
+      <c r="E20" s="6">
+        <f t="shared" si="8"/>
+        <v>-70066.683006658801</v>
+      </c>
+      <c r="F20" s="6">
+        <f t="shared" ref="F20:G20" si="16">F4-F$34</f>
+        <v>-48889.259790475502</v>
+      </c>
+      <c r="G20" s="6">
+        <f t="shared" si="16"/>
+        <v>17197.963143481102</v>
+      </c>
+      <c r="H20" s="5">
+        <f t="shared" si="10"/>
+        <v>-2.8427354671362348</v>
+      </c>
+      <c r="I20" s="6">
+        <f t="shared" si="11"/>
+        <v>-31691.2966469944</v>
+      </c>
+      <c r="J20" s="6">
+        <f t="shared" ref="J20:K20" si="17">J4-J$34</f>
+        <v>-28941.9181735079</v>
+      </c>
+      <c r="K20" s="6">
+        <f t="shared" si="17"/>
+        <v>8147.9350694003515</v>
+      </c>
+      <c r="L20" s="5">
+        <f t="shared" si="13"/>
+        <v>-3.5520555732211898</v>
+      </c>
+      <c r="M20" s="6">
+        <f t="shared" si="14"/>
+        <v>-20793.983104107549</v>
+      </c>
+      <c r="N20" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>4</v>
+      </c>
+      <c r="B21" s="6">
+        <f t="shared" ref="B21:C21" si="18">B5-B$34</f>
+        <v>-611711.12191152503</v>
+      </c>
+      <c r="C21" s="6">
+        <f t="shared" si="18"/>
+        <v>618480.96790879907</v>
+      </c>
+      <c r="D21" s="5">
+        <f t="shared" si="7"/>
+        <v>-0.989054075471127</v>
+      </c>
+      <c r="E21" s="6">
+        <f t="shared" si="8"/>
+        <v>6769.8459972740384</v>
+      </c>
+      <c r="F21" s="6">
+        <f t="shared" ref="F21:G21" si="19">F5-F$34</f>
+        <v>-124837.11295495099</v>
+      </c>
+      <c r="G21" s="6">
+        <f t="shared" si="19"/>
+        <v>114274.7717876463</v>
+      </c>
+      <c r="H21" s="5">
+        <f t="shared" si="10"/>
+        <v>-1.0924293350323413</v>
+      </c>
+      <c r="I21" s="6">
+        <f t="shared" si="11"/>
+        <v>-10562.341167304694</v>
+      </c>
+      <c r="J21" s="6">
+        <f t="shared" ref="J21:K21" si="20">J5-J$34</f>
+        <v>-49513.350620204001</v>
+      </c>
+      <c r="K21" s="6">
+        <f t="shared" si="20"/>
+        <v>37966.275643994952</v>
+      </c>
+      <c r="L21" s="5">
+        <f t="shared" si="13"/>
+        <v>-1.3041403134846445</v>
+      </c>
+      <c r="M21" s="6">
+        <f t="shared" si="14"/>
+        <v>-11547.074976209049</v>
+      </c>
+      <c r="N21" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>6</v>
+      </c>
+      <c r="B22" s="6">
+        <f t="shared" ref="B22:C22" si="21">B6-B$34</f>
+        <v>-23639.052484741402</v>
+      </c>
+      <c r="C22" s="6">
+        <f t="shared" si="21"/>
+        <v>5196.7019918885999</v>
+      </c>
+      <c r="D22" s="5">
+        <f t="shared" si="7"/>
+        <v>-4.54885666363763</v>
+      </c>
+      <c r="E22" s="6">
+        <f t="shared" si="8"/>
+        <v>-18442.350492852802</v>
+      </c>
+      <c r="F22" s="6">
+        <f t="shared" ref="F22:G22" si="22">F6-F$34</f>
+        <v>-5718.2312864800897</v>
+      </c>
+      <c r="G22" s="6">
+        <f t="shared" si="22"/>
+        <v>4165.9214180670006</v>
+      </c>
+      <c r="H22" s="5">
+        <f t="shared" si="10"/>
+        <v>-1.3726210152887055</v>
+      </c>
+      <c r="I22" s="6">
+        <f t="shared" si="11"/>
+        <v>-1552.3098684130891</v>
+      </c>
+      <c r="J22" s="6">
+        <f t="shared" ref="J22:K22" si="23">J6-J$34</f>
+        <v>-2790.36636372676</v>
+      </c>
+      <c r="K22" s="6">
+        <f t="shared" si="23"/>
+        <v>3588.8208597516514</v>
+      </c>
+      <c r="L22" s="5">
+        <f t="shared" si="13"/>
+        <v>-0.77751620177549208</v>
+      </c>
+      <c r="M22" s="6">
+        <f t="shared" si="14"/>
+        <v>798.45449602489134</v>
+      </c>
+      <c r="N22" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>5</v>
+      </c>
+      <c r="B23" s="6">
+        <f t="shared" ref="B23:C23" si="24">B7-B$34</f>
+        <v>-30682.746255407401</v>
+      </c>
+      <c r="C23" s="6">
+        <f t="shared" si="24"/>
+        <v>2604.7893640988987</v>
+      </c>
+      <c r="D23" s="5">
+        <f t="shared" si="7"/>
+        <v>-11.779357931316568</v>
+      </c>
+      <c r="E23" s="6">
+        <f t="shared" si="8"/>
+        <v>-28077.956891308502</v>
+      </c>
+      <c r="F23" s="6">
+        <f t="shared" ref="F23:G23" si="25">F7-F$34</f>
+        <v>-6100.3980291768003</v>
+      </c>
+      <c r="G23" s="6">
+        <f t="shared" si="25"/>
+        <v>1180.6279208439009</v>
+      </c>
+      <c r="H23" s="5">
+        <f t="shared" si="10"/>
+        <v>-5.1670792478093333</v>
+      </c>
+      <c r="I23" s="6">
+        <f t="shared" si="11"/>
+        <v>-4919.7701083328993</v>
+      </c>
+      <c r="J23" s="6">
+        <f t="shared" ref="J23:K23" si="26">J7-J$34</f>
+        <v>-2360.7973050558699</v>
+      </c>
+      <c r="K23" s="6">
+        <f t="shared" si="26"/>
+        <v>814.23624224365085</v>
+      </c>
+      <c r="L23" s="5">
+        <f t="shared" si="13"/>
+        <v>-2.8994009141015713</v>
+      </c>
+      <c r="M23" s="6">
+        <f t="shared" si="14"/>
+        <v>-1546.561062812219</v>
+      </c>
+      <c r="N23" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B24" s="6">
+        <f t="shared" ref="B24:C24" si="27">B8-B$34</f>
+        <v>-97079.650583780895</v>
+      </c>
+      <c r="C24" s="6">
+        <f t="shared" si="27"/>
+        <v>15491.564549771199</v>
+      </c>
+      <c r="D24" s="5">
+        <f t="shared" si="7"/>
+        <v>-6.2666136962399124</v>
+      </c>
+      <c r="E24" s="6">
+        <f t="shared" si="8"/>
+        <v>-81588.086034009699</v>
+      </c>
+      <c r="F24" s="6">
+        <f t="shared" ref="F24:G24" si="28">F8-F$34</f>
+        <v>-20972.403124771499</v>
+      </c>
+      <c r="G24" s="6">
+        <f t="shared" si="28"/>
+        <v>6863.9098429973001</v>
+      </c>
+      <c r="H24" s="5">
+        <f t="shared" si="10"/>
+        <v>-3.0554601684006633</v>
+      </c>
+      <c r="I24" s="6">
+        <f t="shared" si="11"/>
+        <v>-14108.493281774199</v>
+      </c>
+      <c r="J24" s="6">
+        <f t="shared" ref="J24:K24" si="29">J8-J$34</f>
+        <v>-8406.4334333911793</v>
+      </c>
+      <c r="K24" s="6">
+        <f t="shared" si="29"/>
+        <v>3957.6675821073513</v>
+      </c>
+      <c r="L24" s="5">
+        <f t="shared" si="13"/>
+        <v>-2.1240878014608242</v>
+      </c>
+      <c r="M24" s="6">
+        <f t="shared" si="14"/>
+        <v>-4448.7658512838279</v>
+      </c>
+      <c r="N24" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>7</v>
+      </c>
+      <c r="B25" s="6">
+        <f t="shared" ref="B25:C25" si="30">B9-B$34</f>
+        <v>-43683.1580178394</v>
+      </c>
+      <c r="C25" s="6">
+        <f t="shared" si="30"/>
+        <v>5215.4990279757003</v>
+      </c>
+      <c r="D25" s="5">
+        <f t="shared" si="7"/>
+        <v>-8.3756430177677963</v>
+      </c>
+      <c r="E25" s="6">
+        <f t="shared" si="8"/>
+        <v>-38467.658989863703</v>
+      </c>
+      <c r="F25" s="6">
+        <f t="shared" ref="F25:G25" si="31">F9-F$34</f>
+        <v>-9175.9801601351992</v>
+      </c>
+      <c r="G25" s="6">
+        <f t="shared" si="31"/>
+        <v>2327.105103641301</v>
+      </c>
+      <c r="H25" s="5">
+        <f t="shared" si="10"/>
+        <v>-3.9430879790419562</v>
+      </c>
+      <c r="I25" s="6">
+        <f t="shared" si="11"/>
+        <v>-6848.8750564938982</v>
+      </c>
+      <c r="J25" s="6">
+        <f t="shared" ref="J25:K25" si="32">J9-J$34</f>
+        <v>-3610.0129557775899</v>
+      </c>
+      <c r="K25" s="6">
+        <f t="shared" si="32"/>
+        <v>1351.5964489735507</v>
+      </c>
+      <c r="L25" s="5">
+        <f t="shared" si="13"/>
+        <v>-2.6709251555959321</v>
+      </c>
+      <c r="M25" s="6">
+        <f t="shared" si="14"/>
+        <v>-2258.4165068040393</v>
+      </c>
+      <c r="N25" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>9</v>
+      </c>
+      <c r="B26" s="6">
+        <f t="shared" ref="B26:C26" si="33">B10-B$34</f>
+        <v>-50470.5551048856</v>
+      </c>
+      <c r="C26" s="6">
+        <f t="shared" si="33"/>
+        <v>7561.5187567421999</v>
+      </c>
+      <c r="D26" s="5">
+        <f t="shared" si="7"/>
+        <v>-6.6746584553379193</v>
+      </c>
+      <c r="E26" s="6">
+        <f t="shared" si="8"/>
+        <v>-42909.036348143403</v>
+      </c>
+      <c r="F26" s="6">
+        <f t="shared" ref="F26:G26" si="34">F10-F$34</f>
+        <v>-10472.8845316388</v>
+      </c>
+      <c r="G26" s="6">
+        <f t="shared" si="34"/>
+        <v>3353.7537925179004</v>
+      </c>
+      <c r="H26" s="5">
+        <f t="shared" si="10"/>
+        <v>-3.1227350543750152</v>
+      </c>
+      <c r="I26" s="6">
+        <f t="shared" si="11"/>
+        <v>-7119.1307391208993</v>
+      </c>
+      <c r="J26" s="6">
+        <f t="shared" ref="J26:K26" si="35">J10-J$34</f>
+        <v>-4213.4803805597603</v>
+      </c>
+      <c r="K26" s="6">
+        <f t="shared" si="35"/>
+        <v>2289.3718320445514</v>
+      </c>
+      <c r="L26" s="5">
+        <f t="shared" si="13"/>
+        <v>-1.8404526174312454</v>
+      </c>
+      <c r="M26" s="6">
+        <f t="shared" si="14"/>
+        <v>-1924.1085485152089</v>
+      </c>
+      <c r="N26" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>13</v>
+      </c>
+      <c r="B27" s="6">
+        <f t="shared" ref="B27:C27" si="36">B11-B$34</f>
+        <v>0</v>
+      </c>
+      <c r="C27" s="6">
+        <f t="shared" si="36"/>
+        <v>0</v>
+      </c>
+      <c r="D27" s="5" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E27" s="6">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F27" s="6">
+        <f t="shared" ref="F27:G27" si="37">F11-F$34</f>
+        <v>0</v>
+      </c>
+      <c r="G27" s="6">
+        <f t="shared" si="37"/>
+        <v>0</v>
+      </c>
+      <c r="H27" s="5" t="e">
+        <f t="shared" si="10"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I27" s="6">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J27" s="6">
+        <f t="shared" ref="J27:K27" si="38">J11-J$34</f>
+        <v>0</v>
+      </c>
+      <c r="K27" s="6">
+        <f t="shared" si="38"/>
+        <v>0</v>
+      </c>
+      <c r="L27" s="5" t="e">
+        <f t="shared" si="13"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="M27" s="6">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="N27" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>10</v>
+      </c>
+      <c r="B28" s="6">
+        <f t="shared" ref="B28:C28" si="39">B12-B$34</f>
+        <v>-1404.5679010868701</v>
+      </c>
+      <c r="C28" s="6">
+        <f t="shared" si="39"/>
+        <v>30645.9567213056</v>
+      </c>
+      <c r="D28" s="5">
+        <f t="shared" si="7"/>
+        <v>-4.5832078726078411E-2</v>
+      </c>
+      <c r="E28" s="6">
+        <f t="shared" si="8"/>
+        <v>29241.38882021873</v>
+      </c>
+      <c r="F28" s="6">
+        <f t="shared" ref="F28:G28" si="40">F12-F$34</f>
+        <v>-32.085743248811902</v>
+      </c>
+      <c r="G28" s="6">
+        <f t="shared" si="40"/>
+        <v>20766.988076812304</v>
+      </c>
+      <c r="H28" s="5">
+        <f t="shared" si="10"/>
+        <v>-1.5450359546668074E-3</v>
+      </c>
+      <c r="I28" s="6">
+        <f t="shared" si="11"/>
+        <v>20734.902333563492</v>
+      </c>
+      <c r="J28" s="6">
+        <f t="shared" ref="J28:K28" si="41">J12-J$34</f>
+        <v>-227.43782558660999</v>
+      </c>
+      <c r="K28" s="6">
+        <f t="shared" si="41"/>
+        <v>16410.750520843852</v>
+      </c>
+      <c r="L28" s="5">
+        <f t="shared" si="13"/>
+        <v>-1.385907520181563E-2</v>
+      </c>
+      <c r="M28" s="6">
+        <f t="shared" si="14"/>
+        <v>16183.312695257242</v>
+      </c>
+      <c r="N28" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>11</v>
+      </c>
+      <c r="B29" s="6">
+        <f t="shared" ref="B29:C29" si="42">B13-B$34</f>
+        <v>40603.4193094004</v>
+      </c>
+      <c r="C29" s="6">
+        <f t="shared" si="42"/>
+        <v>813683.07561047014</v>
+      </c>
+      <c r="D29" s="5">
+        <f t="shared" si="7"/>
+        <v>4.9900778972129245E-2</v>
+      </c>
+      <c r="E29" s="6">
+        <f t="shared" si="8"/>
+        <v>854286.49491987051</v>
+      </c>
+      <c r="F29" s="6">
+        <f t="shared" ref="F29:G29" si="43">F13-F$34</f>
+        <v>4460.6170443716501</v>
+      </c>
+      <c r="G29" s="6">
+        <f t="shared" si="43"/>
+        <v>210792.00600332531</v>
+      </c>
+      <c r="H29" s="5">
+        <f t="shared" si="10"/>
+        <v>2.116122489152308E-2</v>
+      </c>
+      <c r="I29" s="6">
+        <f t="shared" si="11"/>
+        <v>215252.62304769695</v>
+      </c>
+      <c r="J29" s="6">
+        <f t="shared" ref="J29:K29" si="44">J13-J$34</f>
+        <v>-1031.07110519603</v>
+      </c>
+      <c r="K29" s="6">
+        <f t="shared" si="44"/>
+        <v>98908.904641411849</v>
+      </c>
+      <c r="L29" s="5">
+        <f t="shared" si="13"/>
+        <v>-1.0424451761285952E-2</v>
+      </c>
+      <c r="M29" s="6">
+        <f t="shared" si="14"/>
+        <v>97877.833536215825</v>
+      </c>
+      <c r="N29" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>12</v>
+      </c>
+      <c r="B30" s="6">
+        <f t="shared" ref="B30:C30" si="45">B14-B$34</f>
+        <v>-2626.77829541446</v>
+      </c>
+      <c r="C30" s="6">
+        <f t="shared" si="45"/>
+        <v>11281.197868490701</v>
+      </c>
+      <c r="D30" s="5">
+        <f t="shared" si="7"/>
+        <v>-0.23284568944147896</v>
+      </c>
+      <c r="E30" s="6">
+        <f t="shared" si="8"/>
+        <v>8654.4195730762403</v>
+      </c>
+      <c r="F30" s="6">
+        <f t="shared" ref="F30:G30" si="46">F14-F$34</f>
+        <v>-184.162683612303</v>
+      </c>
+      <c r="G30" s="6">
+        <f t="shared" si="46"/>
+        <v>6318.092648078602</v>
+      </c>
+      <c r="H30" s="5">
+        <f t="shared" si="10"/>
+        <v>-2.9148462023314711E-2</v>
+      </c>
+      <c r="I30" s="6">
+        <f t="shared" si="11"/>
+        <v>6133.9299644662988</v>
+      </c>
+      <c r="J30" s="6">
+        <f t="shared" ref="J30:K30" si="47">J14-J$34</f>
+        <v>-125.237709722896</v>
+      </c>
+      <c r="K30" s="6">
+        <f t="shared" si="47"/>
+        <v>4288.3705311750509</v>
+      </c>
+      <c r="L30" s="5">
+        <f t="shared" si="13"/>
+        <v>-2.9204031884012546E-2</v>
+      </c>
+      <c r="M30" s="6">
+        <f t="shared" si="14"/>
+        <v>4163.1328214521545</v>
+      </c>
+      <c r="N30" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>55</v>
+      </c>
+      <c r="B31" s="6">
+        <f t="shared" ref="B31:C31" si="48">B15-B$34</f>
+        <v>-177560.27976733001</v>
+      </c>
+      <c r="C31" s="6">
+        <f t="shared" si="48"/>
+        <v>70162.474951677606</v>
+      </c>
+      <c r="D31" s="5">
+        <f t="shared" si="7"/>
+        <v>-2.5307014880763479</v>
+      </c>
+      <c r="E31" s="6">
+        <f t="shared" si="8"/>
+        <v>-107397.8048156524</v>
+      </c>
+      <c r="F31" s="6">
+        <f t="shared" ref="F31:G31" si="49">F15-F$34</f>
+        <v>-55394.240300793303</v>
+      </c>
+      <c r="G31" s="6">
+        <f t="shared" si="49"/>
+        <v>32817.166808422196</v>
+      </c>
+      <c r="H31" s="5">
+        <f t="shared" si="10"/>
+        <v>-1.6879653452161181</v>
+      </c>
+      <c r="I31" s="6">
+        <f t="shared" si="11"/>
+        <v>-22577.073492371106</v>
+      </c>
+      <c r="J31" s="6">
+        <f t="shared" ref="J31:K31" si="50">J15-J$34</f>
+        <v>-27847.218892906101</v>
+      </c>
+      <c r="K31" s="6">
+        <f t="shared" si="50"/>
+        <v>19047.796062373549</v>
+      </c>
+      <c r="L31" s="5">
+        <f t="shared" si="13"/>
+        <v>-1.4619654054315854</v>
+      </c>
+      <c r="M31" s="6">
+        <f t="shared" si="14"/>
+        <v>-8799.4228305325523</v>
+      </c>
+      <c r="N31" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>13</v>
+      </c>
+      <c r="B33" t="s">
+        <v>61</v>
+      </c>
+      <c r="C33" t="s">
+        <v>62</v>
+      </c>
+      <c r="F33" t="s">
+        <v>63</v>
+      </c>
+      <c r="G33" t="s">
+        <v>64</v>
+      </c>
+      <c r="J33" t="s">
+        <v>65</v>
+      </c>
+      <c r="K33" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B34" s="1">
+        <v>0</v>
+      </c>
+      <c r="C34" s="1">
+        <v>14486.1268858849</v>
+      </c>
+      <c r="F34" s="1">
+        <v>0</v>
+      </c>
+      <c r="G34" s="1">
+        <v>11511.601320002699</v>
+      </c>
+      <c r="J34" s="1">
+        <v>0</v>
+      </c>
+      <c r="K34" s="1">
+        <v>9874.8984398431494</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:N1" xr:uid="{E1B4DBF1-F2D7-44F8-977D-1BE3C41C10B1}">
@@ -7178,7 +8109,43 @@
       <sortCondition ref="A1"/>
     </sortState>
   </autoFilter>
-  <conditionalFormatting sqref="D2:D15 H2:H15 L2:L14">
+  <conditionalFormatting sqref="D2:D15 H2:H15 L2:L15">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="num" val="-1"/>
+        <cfvo type="max"/>
+        <color theme="6"/>
+        <color theme="0"/>
+        <color rgb="FFC00000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D18:D31">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="num" val="-1"/>
+        <cfvo type="max"/>
+        <color theme="6"/>
+        <color theme="0"/>
+        <color rgb="FFC00000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H18:H31">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="num" val="-1"/>
+        <cfvo type="max"/>
+        <color theme="6"/>
+        <color theme="0"/>
+        <color rgb="FFC00000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L18:L31">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -7196,110 +8163,113 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18025FA5-7769-47FF-9EA0-8E472D7D4015}">
-  <dimension ref="A1:AP16"/>
+  <dimension ref="A1:AP34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="21" style="5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="21" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1" t="s">
         <v>15</v>
       </c>
-      <c r="C1" t="s">
+      <c r="G1" t="s">
         <v>16</v>
       </c>
-      <c r="D1" t="s">
+      <c r="H1" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E1" t="s">
+      <c r="I1" t="s">
         <v>18</v>
       </c>
-      <c r="F1" t="s">
+      <c r="J1" t="s">
         <v>19</v>
       </c>
-      <c r="G1" t="s">
+      <c r="K1" t="s">
         <v>20</v>
       </c>
-      <c r="H1" t="s">
+      <c r="L1" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="I1" t="s">
+      <c r="M1" t="s">
         <v>22</v>
       </c>
-      <c r="J1" t="s">
+      <c r="N1" t="s">
         <v>23</v>
-      </c>
-      <c r="K1" t="s">
-        <v>24</v>
-      </c>
-      <c r="L1" t="s">
-        <v>25</v>
-      </c>
-      <c r="M1" t="s">
-        <v>26</v>
-      </c>
-      <c r="N1" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="6">
         <v>-94864.731470308194</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="6">
         <v>121535.566517909</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="5">
         <v>-0.78055119327006905</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="6">
         <f>B2+C2</f>
         <v>26670.835047600805</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F2" s="6">
         <v>-24012.4014868552</v>
       </c>
-      <c r="G2" s="1">
+      <c r="G2" s="6">
         <v>48730.788212699401</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="5">
         <v>-0.49275627108772002</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="6">
         <f>F2+G2</f>
         <v>24718.386725844201</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="6">
         <v>-9686.1108143464007</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="6">
         <v>27914.545327342599</v>
       </c>
-      <c r="L2">
+      <c r="L2" s="5">
         <v>-0.346991530786594</v>
       </c>
-      <c r="M2" s="1">
+      <c r="M2" s="6">
         <f>J2+K2</f>
         <v>18228.434512996198</v>
       </c>
       <c r="N2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="O2" s="2"/>
       <c r="P2" s="2"/>
@@ -7334,624 +8304,1495 @@
       <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="6">
         <v>-573819.81405192497</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="6">
         <v>815193.62386759603</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="5">
         <v>-0.70390616075908496</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="6">
         <f t="shared" ref="E3:E15" si="0">B3+C3</f>
         <v>241373.80981567106</v>
       </c>
-      <c r="F3" s="1">
+      <c r="F3" s="6">
         <v>-84257.525916830593</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G3" s="6">
         <v>140944.522706794</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="5">
         <v>-0.59780631626324898</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="6">
         <f t="shared" ref="I3:I15" si="1">F3+G3</f>
         <v>56686.996789963407</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="6">
         <v>-23204.8464252616</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="6">
         <v>49651.190773092399</v>
       </c>
-      <c r="L3">
+      <c r="L3" s="5">
         <v>-0.46735729927019298</v>
       </c>
-      <c r="M3" s="1">
+      <c r="M3" s="6">
         <f t="shared" ref="M3:M15" si="2">J3+K3</f>
         <v>26446.3443478308</v>
       </c>
       <c r="N3" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="6">
         <v>-189547.67770812401</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="6">
         <v>81242.480945637202</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="5">
         <v>-2.3331104060566301</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="6">
         <f t="shared" si="0"/>
         <v>-108305.19676248681</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F4" s="6">
         <v>-74162.1476601756</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G4" s="6">
         <v>40207.866336966101</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="5">
         <v>-1.8444686181219401</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="6">
         <f t="shared" si="1"/>
         <v>-33954.2813232095</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="6">
         <v>-41535.203838220703</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="6">
         <v>24697.2770423121</v>
       </c>
-      <c r="L4">
+      <c r="L4" s="5">
         <v>-1.68177260056083</v>
       </c>
-      <c r="M4" s="1">
+      <c r="M4" s="6">
         <f t="shared" si="2"/>
         <v>-16837.926795908603</v>
       </c>
       <c r="N4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="6">
         <v>-1529260.70418628</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="6">
         <v>1535271.1979602601</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="5">
         <v>-0.99608506055349399</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="6">
         <f t="shared" si="0"/>
         <v>6010.4937739800662</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5" s="6">
         <v>-265902.76421105402</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G5" s="6">
         <v>266640.44285571203</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="5">
         <v>-0.99723343302029399</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="6">
         <f t="shared" si="1"/>
         <v>737.67864465800812</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="6">
         <v>-90741.464406757499</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="6">
         <v>89320.816158220798</v>
       </c>
-      <c r="L5">
+      <c r="L5" s="5">
         <v>-1.0159050074735101</v>
       </c>
-      <c r="M5" s="1">
+      <c r="M5" s="6">
         <f t="shared" si="2"/>
         <v>-1420.6482485367014</v>
       </c>
       <c r="N5" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="6">
         <v>0</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="6">
         <v>16454.604553368801</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="5">
         <v>0</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="6">
         <f t="shared" si="0"/>
         <v>16454.604553368801</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F6" s="6">
         <v>0</v>
       </c>
-      <c r="G6" s="1">
+      <c r="G6" s="6">
         <v>12922.5120645157</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="5">
         <v>0</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6" s="6">
         <f t="shared" si="1"/>
         <v>12922.5120645157</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="6">
         <v>0</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="6">
         <v>10988.815786839299</v>
       </c>
-      <c r="L6">
+      <c r="L6" s="5">
         <v>0</v>
       </c>
-      <c r="M6" s="1">
+      <c r="M6" s="6">
         <f t="shared" si="2"/>
         <v>10988.815786839299</v>
       </c>
       <c r="N6" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="1">
+      <c r="B7" s="6">
         <v>-81711.783899172602</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7" s="6">
         <v>22059.733037833099</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="5">
         <v>-3.7041148122252601</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="6">
         <f t="shared" si="0"/>
         <v>-59652.050861339507</v>
       </c>
-      <c r="F7" s="1">
+      <c r="F7" s="6">
         <v>-14041.807010664401</v>
       </c>
-      <c r="G7" s="1">
+      <c r="G7" s="6">
         <v>17381.240704187301</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="5">
         <v>-0.8078713855727</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7" s="6">
         <f t="shared" si="1"/>
         <v>3339.4336935229003</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="6">
         <v>-5067.3328268512496</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="6">
         <v>14808.855061788299</v>
       </c>
-      <c r="L7">
+      <c r="L7" s="5">
         <v>-0.34218262017612899</v>
       </c>
-      <c r="M7" s="1">
+      <c r="M7" s="6">
         <f t="shared" si="2"/>
         <v>9741.5222349370488</v>
       </c>
       <c r="N7" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="1">
+      <c r="B8" s="6">
         <v>-74787.623200904796</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="6">
         <v>19094.971222653399</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="5">
         <v>-3.9166135590809201</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="6">
         <f t="shared" si="0"/>
         <v>-55692.651978251393</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F8" s="6">
         <v>-12795.920628411601</v>
       </c>
-      <c r="G8" s="1">
+      <c r="G8" s="6">
         <v>14128.7206300791</v>
       </c>
-      <c r="H8">
+      <c r="H8" s="5">
         <v>-0.90566732568623198</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8" s="6">
         <f t="shared" si="1"/>
         <v>1332.8000016674996</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="6">
         <v>-4277.3243685469497</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="6">
         <v>11823.3041249241</v>
       </c>
-      <c r="L8">
+      <c r="L8" s="5">
         <v>-0.361770645781675</v>
       </c>
-      <c r="M8" s="1">
+      <c r="M8" s="6">
         <f t="shared" si="2"/>
         <v>7545.9797563771499</v>
       </c>
       <c r="N8" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="1">
+      <c r="B9" s="6">
         <v>-201382.40255214801</v>
       </c>
-      <c r="C9" s="1">
+      <c r="C9" s="6">
         <v>32071.308412600101</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="5">
         <v>-6.2792075696240897</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="6">
         <f t="shared" si="0"/>
         <v>-169311.0941395479</v>
       </c>
-      <c r="F9" s="1">
+      <c r="F9" s="6">
         <v>-38626.101035459098</v>
       </c>
-      <c r="G9" s="1">
+      <c r="G9" s="6">
         <v>19876.195905398199</v>
       </c>
-      <c r="H9">
+      <c r="H9" s="5">
         <v>-1.9433346913716201</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9" s="6">
         <f t="shared" si="1"/>
         <v>-18749.905130060899</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="6">
         <v>-14104.8743016727</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="6">
         <v>15017.4159804518</v>
       </c>
-      <c r="L9">
+      <c r="L9" s="5">
         <v>-0.93923444086739505</v>
       </c>
-      <c r="M9" s="1">
+      <c r="M9" s="6">
         <f t="shared" si="2"/>
         <v>912.54167877910004</v>
       </c>
       <c r="N9" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="1">
+      <c r="B10" s="6">
         <v>-98338.675448048598</v>
       </c>
-      <c r="C10" s="1">
+      <c r="C10" s="6">
         <v>21722.272439247401</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="5">
         <v>-4.5270896828626404</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="6">
         <f t="shared" si="0"/>
         <v>-76616.403008801193</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F10" s="6">
         <v>-17986.986790839499</v>
       </c>
-      <c r="G10" s="1">
+      <c r="G10" s="6">
         <v>15287.094538355101</v>
       </c>
-      <c r="H10">
+      <c r="H10" s="5">
         <v>-1.1766125175526601</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10" s="6">
         <f t="shared" si="1"/>
         <v>-2699.8922524843983</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="6">
         <v>-6302.0903447309802</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="6">
         <v>12370.0600946878</v>
       </c>
-      <c r="L10">
+      <c r="L10" s="5">
         <v>-0.50946319552944896</v>
       </c>
-      <c r="M10" s="1">
+      <c r="M10" s="6">
         <f t="shared" si="2"/>
         <v>6067.9697499568201</v>
       </c>
       <c r="N10" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="1">
+      <c r="B11" s="6">
         <v>-112560.083841115</v>
       </c>
-      <c r="C11" s="1">
+      <c r="C11" s="6">
         <v>24071.699131444799</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="5">
         <v>-4.6760340109967</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="6">
         <f t="shared" si="0"/>
         <v>-88488.384709670208</v>
       </c>
-      <c r="F11" s="1">
+      <c r="F11" s="6">
         <v>-20252.154009836198</v>
       </c>
-      <c r="G11" s="1">
+      <c r="G11" s="6">
         <v>16316.162333554499</v>
       </c>
-      <c r="H11">
+      <c r="H11" s="5">
         <v>-1.2412326866954</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11" s="6">
         <f t="shared" si="1"/>
         <v>-3935.9916762816993</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="6">
         <v>-7133.5598014398502</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="6">
         <v>13309.729450819899</v>
       </c>
-      <c r="L11">
+      <c r="L11" s="5">
         <v>-0.535965800642205</v>
       </c>
-      <c r="M11" s="1">
+      <c r="M11" s="6">
         <f t="shared" si="2"/>
         <v>6176.1696493800491</v>
       </c>
       <c r="N11" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="1">
+      <c r="B12" s="6">
         <v>-20612.841126253501</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12" s="6">
         <v>47147.659759674803</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="5">
         <v>-0.43719754556903001</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="6">
         <f t="shared" si="0"/>
         <v>26534.818633421302</v>
       </c>
-      <c r="F12" s="1">
+      <c r="F12" s="6">
         <v>-2555.2191726661399</v>
       </c>
-      <c r="G12" s="1">
+      <c r="G12" s="6">
         <v>33709.460372616202</v>
       </c>
-      <c r="H12">
+      <c r="H12" s="5">
         <v>-7.58012482081101E-2</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12" s="6">
         <f t="shared" si="1"/>
         <v>31154.241199950062</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="6">
         <v>-817.00285092435604</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="6">
         <v>27410.213109250599</v>
       </c>
-      <c r="L12">
+      <c r="L12" s="5">
         <v>-2.9806512180987999E-2</v>
       </c>
-      <c r="M12" s="1">
+      <c r="M12" s="6">
         <f t="shared" si="2"/>
         <v>26593.210258326242</v>
       </c>
       <c r="N12" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="1">
+      <c r="B13" s="6">
         <v>33750.559282223403</v>
       </c>
-      <c r="C13" s="1">
+      <c r="C13" s="6">
         <v>913639.44245667802</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="5">
         <v>3.6940786172137897E-2</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="6">
         <f t="shared" si="0"/>
         <v>947390.00173890148</v>
       </c>
-      <c r="F13" s="1">
+      <c r="F13" s="6">
         <v>5157.5221174354301</v>
       </c>
-      <c r="G13" s="1">
+      <c r="G13" s="6">
         <v>235929.47854249101</v>
       </c>
-      <c r="H13">
+      <c r="H13" s="5">
         <v>2.1860439608043899E-2</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13" s="6">
         <f t="shared" si="1"/>
         <v>241087.00065992645</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="6">
         <v>-354.46081332431601</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="6">
         <v>113106.55812487499</v>
       </c>
-      <c r="L13">
+      <c r="L13" s="5">
         <v>-3.1338661453474098E-3</v>
       </c>
-      <c r="M13" s="1">
+      <c r="M13" s="6">
         <f t="shared" si="2"/>
         <v>112752.09731155068</v>
       </c>
       <c r="N13" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="1">
+      <c r="B14" s="6">
         <v>-22101.075343330998</v>
       </c>
-      <c r="C14" s="1">
+      <c r="C14" s="6">
         <v>27762.780358668701</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="5">
         <v>-0.79606851539385404</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="6">
         <f t="shared" si="0"/>
         <v>5661.7050153377022</v>
       </c>
-      <c r="F14" s="1">
+      <c r="F14" s="6">
         <v>-2707.91448460225</v>
       </c>
-      <c r="G14" s="1">
+      <c r="G14" s="6">
         <v>19251.584572950102</v>
       </c>
-      <c r="H14">
+      <c r="H14" s="5">
         <v>-0.140659303879175</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14" s="6">
         <f t="shared" si="1"/>
         <v>16543.670088347852</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="6">
         <v>-692.01167725153198</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="6">
         <v>15282.8414246461</v>
       </c>
-      <c r="L14">
+      <c r="L14" s="5">
         <v>-4.5280302139073698E-2</v>
       </c>
-      <c r="M14" s="1">
+      <c r="M14" s="6">
         <f t="shared" si="2"/>
         <v>14590.829747394568</v>
       </c>
       <c r="N14" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>59</v>
-      </c>
-      <c r="B15" s="1">
+        <v>55</v>
+      </c>
+      <c r="B15" s="6">
         <v>-343064.27648368402</v>
       </c>
-      <c r="C15" s="1">
+      <c r="C15" s="6">
         <v>96166.745901482194</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="5">
         <v>-3.5673898837664302</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="6">
         <f t="shared" si="0"/>
         <v>-246897.53058220184</v>
       </c>
-      <c r="F15" s="1">
+      <c r="F15" s="6">
         <v>-100078.99781724501</v>
       </c>
-      <c r="G15" s="1">
+      <c r="G15" s="6">
         <v>46662.644528508899</v>
       </c>
-      <c r="H15">
+      <c r="H15" s="5">
         <v>-2.14473480507734</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15" s="6">
         <f t="shared" si="1"/>
         <v>-53416.353288736107</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="6">
         <v>-49751.588765194501</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="6">
         <v>28330.3209334069</v>
       </c>
-      <c r="L15">
+      <c r="L15" s="5">
         <v>-1.75612513822699</v>
       </c>
-      <c r="M15" s="1">
+      <c r="M15" s="6">
         <f t="shared" si="2"/>
         <v>-21421.267831787602</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="O15" s="1"/>
     </row>
     <row r="16" spans="1:42" x14ac:dyDescent="0.25">
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
-      <c r="J16" s="1"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
+      <c r="G16" s="4"/>
+      <c r="I16" s="4"/>
+      <c r="J16" s="4"/>
+      <c r="K16" s="4"/>
+      <c r="M16" s="4"/>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I17" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="J17" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K17" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="L17" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="M17" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="N17" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B18" s="6">
+        <f>B2-B$34</f>
+        <v>-94864.731470308194</v>
+      </c>
+      <c r="C18" s="6">
+        <f>C2-C$34</f>
+        <v>105080.9619645402</v>
+      </c>
+      <c r="D18" s="5">
+        <f>B18/C18</f>
+        <v>-0.90277753169332908</v>
+      </c>
+      <c r="E18" s="6">
+        <f>B18+C18</f>
+        <v>10216.230494232004</v>
+      </c>
+      <c r="F18" s="6">
+        <f>F2-F$34</f>
+        <v>-24012.4014868552</v>
+      </c>
+      <c r="G18" s="6">
+        <f>G2-G$34</f>
+        <v>35808.276148183701</v>
+      </c>
+      <c r="H18" s="5">
+        <f>F18/G18</f>
+        <v>-0.67058244824424973</v>
+      </c>
+      <c r="I18" s="6">
+        <f>F18+G18</f>
+        <v>11795.8746613285</v>
+      </c>
+      <c r="J18" s="6">
+        <f>J2-J$34</f>
+        <v>-9686.1108143464007</v>
+      </c>
+      <c r="K18" s="6">
+        <f>K2-K$34</f>
+        <v>16925.7295405033</v>
+      </c>
+      <c r="L18" s="5">
+        <f>J18/K18</f>
+        <v>-0.57227139256641912</v>
+      </c>
+      <c r="M18" s="6">
+        <f>J18+K18</f>
+        <v>7239.6187261568994</v>
+      </c>
+      <c r="N18" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>2</v>
+      </c>
+      <c r="B19" s="6">
+        <f t="shared" ref="B19:C31" si="3">B3-B$34</f>
+        <v>-573819.81405192497</v>
+      </c>
+      <c r="C19" s="6">
+        <f t="shared" si="3"/>
+        <v>798739.01931422728</v>
+      </c>
+      <c r="D19" s="5">
+        <f t="shared" ref="D19:D31" si="4">B19/C19</f>
+        <v>-0.71840713947415391</v>
+      </c>
+      <c r="E19" s="6">
+        <f t="shared" ref="E19:E31" si="5">B19+C19</f>
+        <v>224919.2052623023</v>
+      </c>
+      <c r="F19" s="6">
+        <f t="shared" ref="F19:G31" si="6">F3-F$34</f>
+        <v>-84257.525916830593</v>
+      </c>
+      <c r="G19" s="6">
+        <f t="shared" si="6"/>
+        <v>128022.0106422783</v>
+      </c>
+      <c r="H19" s="5">
+        <f t="shared" ref="H19:H31" si="7">F19/G19</f>
+        <v>-0.65814874718898675</v>
+      </c>
+      <c r="I19" s="6">
+        <f t="shared" ref="I19:I31" si="8">F19+G19</f>
+        <v>43764.484725447706</v>
+      </c>
+      <c r="J19" s="6">
+        <f t="shared" ref="J19:K31" si="9">J3-J$34</f>
+        <v>-23204.8464252616</v>
+      </c>
+      <c r="K19" s="6">
+        <f t="shared" si="9"/>
+        <v>38662.374986253097</v>
+      </c>
+      <c r="L19" s="5">
+        <f t="shared" ref="L19:L31" si="10">J19/K19</f>
+        <v>-0.60019195493066269</v>
+      </c>
+      <c r="M19" s="6">
+        <f t="shared" ref="M19:M31" si="11">J19+K19</f>
+        <v>15457.528560991497</v>
+      </c>
+      <c r="N19" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>3</v>
+      </c>
+      <c r="B20" s="6">
+        <f t="shared" si="3"/>
+        <v>-189547.67770812401</v>
+      </c>
+      <c r="C20" s="6">
+        <f t="shared" si="3"/>
+        <v>64787.876392268401</v>
+      </c>
+      <c r="D20" s="5">
+        <f t="shared" si="4"/>
+        <v>-2.9256658539088045</v>
+      </c>
+      <c r="E20" s="6">
+        <f t="shared" si="5"/>
+        <v>-124759.80131585561</v>
+      </c>
+      <c r="F20" s="6">
+        <f t="shared" si="6"/>
+        <v>-74162.1476601756</v>
+      </c>
+      <c r="G20" s="6">
+        <f t="shared" si="6"/>
+        <v>27285.3542724504</v>
+      </c>
+      <c r="H20" s="5">
+        <f t="shared" si="7"/>
+        <v>-2.7180203313341611</v>
+      </c>
+      <c r="I20" s="6">
+        <f t="shared" si="8"/>
+        <v>-46876.7933877252</v>
+      </c>
+      <c r="J20" s="6">
+        <f t="shared" si="9"/>
+        <v>-41535.203838220703</v>
+      </c>
+      <c r="K20" s="6">
+        <f t="shared" si="9"/>
+        <v>13708.461255472801</v>
+      </c>
+      <c r="L20" s="5">
+        <f t="shared" si="10"/>
+        <v>-3.0298954101532503</v>
+      </c>
+      <c r="M20" s="6">
+        <f t="shared" si="11"/>
+        <v>-27826.742582747902</v>
+      </c>
+      <c r="N20" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>4</v>
+      </c>
+      <c r="B21" s="6">
+        <f t="shared" si="3"/>
+        <v>-1529260.70418628</v>
+      </c>
+      <c r="C21" s="6">
+        <f t="shared" si="3"/>
+        <v>1518816.5934068912</v>
+      </c>
+      <c r="D21" s="5">
+        <f t="shared" si="4"/>
+        <v>-1.006876479243594</v>
+      </c>
+      <c r="E21" s="6">
+        <f t="shared" si="5"/>
+        <v>-10444.110779388808</v>
+      </c>
+      <c r="F21" s="6">
+        <f t="shared" si="6"/>
+        <v>-265902.76421105402</v>
+      </c>
+      <c r="G21" s="6">
+        <f t="shared" si="6"/>
+        <v>253717.93079119633</v>
+      </c>
+      <c r="H21" s="5">
+        <f t="shared" si="7"/>
+        <v>-1.0480251174280839</v>
+      </c>
+      <c r="I21" s="6">
+        <f t="shared" si="8"/>
+        <v>-12184.833419857692</v>
+      </c>
+      <c r="J21" s="6">
+        <f t="shared" si="9"/>
+        <v>-90741.464406757499</v>
+      </c>
+      <c r="K21" s="6">
+        <f t="shared" si="9"/>
+        <v>78332.000371381495</v>
+      </c>
+      <c r="L21" s="5">
+        <f t="shared" si="10"/>
+        <v>-1.1584213855964514</v>
+      </c>
+      <c r="M21" s="6">
+        <f t="shared" si="11"/>
+        <v>-12409.464035376004</v>
+      </c>
+      <c r="N21" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>14</v>
+      </c>
+      <c r="B22" s="6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="C22" s="6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="D22" s="5" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="E22" s="6">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="F22" s="6">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="G22" s="6">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="H22" s="5" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="I22" s="6">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J22" s="6">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="K22" s="6">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="L22" s="5" t="e">
+        <f t="shared" si="10"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="M22" s="6">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="N22" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>6</v>
+      </c>
+      <c r="B23" s="6">
+        <f t="shared" si="3"/>
+        <v>-81711.783899172602</v>
+      </c>
+      <c r="C23" s="6">
+        <f t="shared" si="3"/>
+        <v>5605.1284844642978</v>
+      </c>
+      <c r="D23" s="5">
+        <f t="shared" si="4"/>
+        <v>-14.578039401889303</v>
+      </c>
+      <c r="E23" s="6">
+        <f t="shared" si="5"/>
+        <v>-76106.655414708308</v>
+      </c>
+      <c r="F23" s="6">
+        <f t="shared" si="6"/>
+        <v>-14041.807010664401</v>
+      </c>
+      <c r="G23" s="6">
+        <f t="shared" si="6"/>
+        <v>4458.7286396716008</v>
+      </c>
+      <c r="H23" s="5">
+        <f t="shared" si="7"/>
+        <v>-3.1492849521559183</v>
+      </c>
+      <c r="I23" s="6">
+        <f t="shared" si="8"/>
+        <v>-9583.0783709928</v>
+      </c>
+      <c r="J23" s="6">
+        <f t="shared" si="9"/>
+        <v>-5067.3328268512496</v>
+      </c>
+      <c r="K23" s="6">
+        <f t="shared" si="9"/>
+        <v>3820.0392749490002</v>
+      </c>
+      <c r="L23" s="5">
+        <f t="shared" si="10"/>
+        <v>-1.3265132796099071</v>
+      </c>
+      <c r="M23" s="6">
+        <f t="shared" si="11"/>
+        <v>-1247.2935519022494</v>
+      </c>
+      <c r="N23" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>5</v>
+      </c>
+      <c r="B24" s="6">
+        <f t="shared" si="3"/>
+        <v>-74787.623200904796</v>
+      </c>
+      <c r="C24" s="6">
+        <f t="shared" si="3"/>
+        <v>2640.3666692845982</v>
+      </c>
+      <c r="D24" s="5">
+        <f t="shared" si="4"/>
+        <v>-28.324711136112146</v>
+      </c>
+      <c r="E24" s="6">
+        <f t="shared" si="5"/>
+        <v>-72147.256531620194</v>
+      </c>
+      <c r="F24" s="6">
+        <f t="shared" si="6"/>
+        <v>-12795.920628411601</v>
+      </c>
+      <c r="G24" s="6">
+        <f t="shared" si="6"/>
+        <v>1206.2085655634</v>
+      </c>
+      <c r="H24" s="5">
+        <f t="shared" si="7"/>
+        <v>-10.608381496971743</v>
+      </c>
+      <c r="I24" s="6">
+        <f t="shared" si="8"/>
+        <v>-11589.712062848201</v>
+      </c>
+      <c r="J24" s="6">
+        <f t="shared" si="9"/>
+        <v>-4277.3243685469497</v>
+      </c>
+      <c r="K24" s="6">
+        <f t="shared" si="9"/>
+        <v>834.48833808480049</v>
+      </c>
+      <c r="L24" s="5">
+        <f t="shared" si="10"/>
+        <v>-5.125685013602058</v>
+      </c>
+      <c r="M24" s="6">
+        <f t="shared" si="11"/>
+        <v>-3442.8360304621492</v>
+      </c>
+      <c r="N24" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>8</v>
+      </c>
+      <c r="B25" s="6">
+        <f t="shared" si="3"/>
+        <v>-201382.40255214801</v>
+      </c>
+      <c r="C25" s="6">
+        <f t="shared" si="3"/>
+        <v>15616.7038592313</v>
+      </c>
+      <c r="D25" s="5">
+        <f t="shared" si="4"/>
+        <v>-12.895320572600053</v>
+      </c>
+      <c r="E25" s="6">
+        <f t="shared" si="5"/>
+        <v>-185765.69869291672</v>
+      </c>
+      <c r="F25" s="6">
+        <f t="shared" si="6"/>
+        <v>-38626.101035459098</v>
+      </c>
+      <c r="G25" s="6">
+        <f t="shared" si="6"/>
+        <v>6953.6838408824988</v>
+      </c>
+      <c r="H25" s="5">
+        <f t="shared" si="7"/>
+        <v>-5.5547680796711374</v>
+      </c>
+      <c r="I25" s="6">
+        <f t="shared" si="8"/>
+        <v>-31672.417194576599</v>
+      </c>
+      <c r="J25" s="6">
+        <f t="shared" si="9"/>
+        <v>-14104.8743016727</v>
+      </c>
+      <c r="K25" s="6">
+        <f t="shared" si="9"/>
+        <v>4028.6001936125012</v>
+      </c>
+      <c r="L25" s="5">
+        <f t="shared" si="10"/>
+        <v>-3.5011849336741121</v>
+      </c>
+      <c r="M25" s="6">
+        <f t="shared" si="11"/>
+        <v>-10076.274108060199</v>
+      </c>
+      <c r="N25" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>7</v>
+      </c>
+      <c r="B26" s="6">
+        <f t="shared" si="3"/>
+        <v>-98338.675448048598</v>
+      </c>
+      <c r="C26" s="6">
+        <f t="shared" si="3"/>
+        <v>5267.6678858785999</v>
+      </c>
+      <c r="D26" s="5">
+        <f t="shared" si="4"/>
+        <v>-18.668351456186496</v>
+      </c>
+      <c r="E26" s="6">
+        <f t="shared" si="5"/>
+        <v>-93071.007562169994</v>
+      </c>
+      <c r="F26" s="6">
+        <f t="shared" si="6"/>
+        <v>-17986.986790839499</v>
+      </c>
+      <c r="G26" s="6">
+        <f t="shared" si="6"/>
+        <v>2364.5824738394003</v>
+      </c>
+      <c r="H26" s="5">
+        <f t="shared" si="7"/>
+        <v>-7.6068341831333193</v>
+      </c>
+      <c r="I26" s="6">
+        <f t="shared" si="8"/>
+        <v>-15622.404317000099</v>
+      </c>
+      <c r="J26" s="6">
+        <f t="shared" si="9"/>
+        <v>-6302.0903447309802</v>
+      </c>
+      <c r="K26" s="6">
+        <f t="shared" si="9"/>
+        <v>1381.2443078485012</v>
+      </c>
+      <c r="L26" s="5">
+        <f t="shared" si="10"/>
+        <v>-4.5626181472178864</v>
+      </c>
+      <c r="M26" s="6">
+        <f t="shared" si="11"/>
+        <v>-4920.846036882479</v>
+      </c>
+      <c r="N26" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>9</v>
+      </c>
+      <c r="B27" s="6">
+        <f t="shared" si="3"/>
+        <v>-112560.083841115</v>
+      </c>
+      <c r="C27" s="6">
+        <f t="shared" si="3"/>
+        <v>7617.0945780759976</v>
+      </c>
+      <c r="D27" s="5">
+        <f t="shared" si="4"/>
+        <v>-14.777298967127511</v>
+      </c>
+      <c r="E27" s="6">
+        <f t="shared" si="5"/>
+        <v>-104942.98926303901</v>
+      </c>
+      <c r="F27" s="6">
+        <f t="shared" si="6"/>
+        <v>-20252.154009836198</v>
+      </c>
+      <c r="G27" s="6">
+        <f t="shared" si="6"/>
+        <v>3393.6502690387988</v>
+      </c>
+      <c r="H27" s="5">
+        <f t="shared" si="7"/>
+        <v>-5.967660897353551</v>
+      </c>
+      <c r="I27" s="6">
+        <f t="shared" si="8"/>
+        <v>-16858.503740797401</v>
+      </c>
+      <c r="J27" s="6">
+        <f t="shared" si="9"/>
+        <v>-7133.5598014398502</v>
+      </c>
+      <c r="K27" s="6">
+        <f t="shared" si="9"/>
+        <v>2320.9136639806002</v>
+      </c>
+      <c r="L27" s="5">
+        <f t="shared" si="10"/>
+        <v>-3.0735998120693031</v>
+      </c>
+      <c r="M27" s="6">
+        <f t="shared" si="11"/>
+        <v>-4812.64613745925</v>
+      </c>
+      <c r="N27" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>10</v>
+      </c>
+      <c r="B28" s="6">
+        <f t="shared" si="3"/>
+        <v>-20612.841126253501</v>
+      </c>
+      <c r="C28" s="6">
+        <f t="shared" si="3"/>
+        <v>30693.055206306002</v>
+      </c>
+      <c r="D28" s="5">
+        <f t="shared" si="4"/>
+        <v>-0.67157997102935896</v>
+      </c>
+      <c r="E28" s="6">
+        <f t="shared" si="5"/>
+        <v>10080.214080052501</v>
+      </c>
+      <c r="F28" s="6">
+        <f t="shared" si="6"/>
+        <v>-2555.2191726661399</v>
+      </c>
+      <c r="G28" s="6">
+        <f t="shared" si="6"/>
+        <v>20786.948308100502</v>
+      </c>
+      <c r="H28" s="5">
+        <f t="shared" si="7"/>
+        <v>-0.12292420872910874</v>
+      </c>
+      <c r="I28" s="6">
+        <f t="shared" si="8"/>
+        <v>18231.729135434362</v>
+      </c>
+      <c r="J28" s="6">
+        <f t="shared" si="9"/>
+        <v>-817.00285092435604</v>
+      </c>
+      <c r="K28" s="6">
+        <f t="shared" si="9"/>
+        <v>16421.3973224113</v>
+      </c>
+      <c r="L28" s="5">
+        <f t="shared" si="10"/>
+        <v>-4.9752334401491009E-2</v>
+      </c>
+      <c r="M28" s="6">
+        <f t="shared" si="11"/>
+        <v>15604.394471486943</v>
+      </c>
+      <c r="N28" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>11</v>
+      </c>
+      <c r="B29" s="6">
+        <f t="shared" si="3"/>
+        <v>33750.559282223403</v>
+      </c>
+      <c r="C29" s="6">
+        <f t="shared" si="3"/>
+        <v>897184.83790330926</v>
+      </c>
+      <c r="D29" s="5">
+        <f t="shared" si="4"/>
+        <v>3.7618289851060485E-2</v>
+      </c>
+      <c r="E29" s="6">
+        <f t="shared" si="5"/>
+        <v>930935.39718553261</v>
+      </c>
+      <c r="F29" s="6">
+        <f t="shared" si="6"/>
+        <v>5157.5221174354301</v>
+      </c>
+      <c r="G29" s="6">
+        <f t="shared" si="6"/>
+        <v>223006.96647797531</v>
+      </c>
+      <c r="H29" s="5">
+        <f t="shared" si="7"/>
+        <v>2.3127179383182182E-2</v>
+      </c>
+      <c r="I29" s="6">
+        <f t="shared" si="8"/>
+        <v>228164.48859541074</v>
+      </c>
+      <c r="J29" s="6">
+        <f t="shared" si="9"/>
+        <v>-354.46081332431601</v>
+      </c>
+      <c r="K29" s="6">
+        <f t="shared" si="9"/>
+        <v>102117.74233803569</v>
+      </c>
+      <c r="L29" s="5">
+        <f t="shared" si="10"/>
+        <v>-3.4710991959747855E-3</v>
+      </c>
+      <c r="M29" s="6">
+        <f t="shared" si="11"/>
+        <v>101763.28152471138</v>
+      </c>
+      <c r="N29" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>12</v>
+      </c>
+      <c r="B30" s="6">
+        <f t="shared" si="3"/>
+        <v>-22101.075343330998</v>
+      </c>
+      <c r="C30" s="6">
+        <f t="shared" si="3"/>
+        <v>11308.175805299899</v>
+      </c>
+      <c r="D30" s="5">
+        <f t="shared" si="4"/>
+        <v>-1.954433298867948</v>
+      </c>
+      <c r="E30" s="6">
+        <f t="shared" si="5"/>
+        <v>-10792.899538031099</v>
+      </c>
+      <c r="F30" s="6">
+        <f t="shared" si="6"/>
+        <v>-2707.91448460225</v>
+      </c>
+      <c r="G30" s="6">
+        <f t="shared" si="6"/>
+        <v>6329.0725084344012</v>
+      </c>
+      <c r="H30" s="5">
+        <f t="shared" si="7"/>
+        <v>-0.42785328829675495</v>
+      </c>
+      <c r="I30" s="6">
+        <f t="shared" si="8"/>
+        <v>3621.1580238321512</v>
+      </c>
+      <c r="J30" s="6">
+        <f t="shared" si="9"/>
+        <v>-692.01167725153198</v>
+      </c>
+      <c r="K30" s="6">
+        <f t="shared" si="9"/>
+        <v>4294.0256378068007</v>
+      </c>
+      <c r="L30" s="5">
+        <f t="shared" si="10"/>
+        <v>-0.16115685736915653</v>
+      </c>
+      <c r="M30" s="6">
+        <f t="shared" si="11"/>
+        <v>3602.0139605552686</v>
+      </c>
+      <c r="N30" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>55</v>
+      </c>
+      <c r="B31" s="6">
+        <f t="shared" si="3"/>
+        <v>-343064.27648368402</v>
+      </c>
+      <c r="C31" s="6">
+        <f t="shared" si="3"/>
+        <v>79712.141348113393</v>
+      </c>
+      <c r="D31" s="5">
+        <f t="shared" si="4"/>
+        <v>-4.3037894940681278</v>
+      </c>
+      <c r="E31" s="6">
+        <f t="shared" si="5"/>
+        <v>-263352.13513557066</v>
+      </c>
+      <c r="F31" s="6">
+        <f t="shared" si="6"/>
+        <v>-100078.99781724501</v>
+      </c>
+      <c r="G31" s="6">
+        <f t="shared" si="6"/>
+        <v>33740.132463993199</v>
+      </c>
+      <c r="H31" s="5">
+        <f t="shared" si="7"/>
+        <v>-2.966170862667695</v>
+      </c>
+      <c r="I31" s="6">
+        <f t="shared" si="8"/>
+        <v>-66338.865353251807</v>
+      </c>
+      <c r="J31" s="6">
+        <f t="shared" si="9"/>
+        <v>-49751.588765194501</v>
+      </c>
+      <c r="K31" s="6">
+        <f t="shared" si="9"/>
+        <v>17341.505146567601</v>
+      </c>
+      <c r="L31" s="5">
+        <f t="shared" si="10"/>
+        <v>-2.8689314073203054</v>
+      </c>
+      <c r="M31" s="6">
+        <f t="shared" si="11"/>
+        <v>-32410.083618626901</v>
+      </c>
+      <c r="N31" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>13</v>
+      </c>
+      <c r="B33" t="s">
+        <v>61</v>
+      </c>
+      <c r="C33" t="s">
+        <v>62</v>
+      </c>
+      <c r="F33" t="s">
+        <v>63</v>
+      </c>
+      <c r="G33" t="s">
+        <v>64</v>
+      </c>
+      <c r="J33" t="s">
+        <v>65</v>
+      </c>
+      <c r="K33" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B34" s="1">
+        <v>0</v>
+      </c>
+      <c r="C34" s="1">
+        <v>16454.604553368801</v>
+      </c>
+      <c r="F34" s="1">
+        <v>0</v>
+      </c>
+      <c r="G34" s="1">
+        <v>12922.5120645157</v>
+      </c>
+      <c r="J34" s="1">
+        <v>0</v>
+      </c>
+      <c r="K34" s="1">
+        <v>10988.815786839299</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:N1" xr:uid="{18025FA5-7769-47FF-9EA0-8E472D7D4015}">
@@ -7960,6 +9801,42 @@
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="L2:L15 H2:H15 D2:D15">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="num" val="-1"/>
+        <cfvo type="max"/>
+        <color theme="6"/>
+        <color theme="0"/>
+        <color rgb="FFC00000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D18:D31">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="num" val="-1"/>
+        <cfvo type="max"/>
+        <color theme="6"/>
+        <color theme="0"/>
+        <color rgb="FFC00000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H18:H31">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="num" val="-1"/>
+        <cfvo type="max"/>
+        <color theme="6"/>
+        <color theme="0"/>
+        <color rgb="FFC00000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L18:L31">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -7993,7 +9870,7 @@
         <v>Scenario</v>
       </c>
       <c r="B1" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C1" t="str">
         <f>Low!F1</f>
@@ -8004,19 +9881,19 @@
         <v>Costs | 12.0%</v>
       </c>
       <c r="F1" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G1" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="H1" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="I1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="J1" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -8025,7 +9902,7 @@
         <v>45Q-2040</v>
       </c>
       <c r="B2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C2" s="1">
         <f>Low!F2</f>
@@ -8046,7 +9923,7 @@
         <v>45Q-2050</v>
       </c>
       <c r="B3" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C3" s="1">
         <f>Low!F3</f>
@@ -8067,7 +9944,7 @@
         <v>CDRIA-2035</v>
       </c>
       <c r="B4" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C4" s="1">
         <f>Low!F4</f>
@@ -8088,7 +9965,7 @@
         <v>CDRIA-2050</v>
       </c>
       <c r="B5" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C5" s="1">
         <f>Low!F5</f>
@@ -8109,7 +9986,7 @@
         <v>Innovation-DACHubs</v>
       </c>
       <c r="B6" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C6" s="1">
         <f>Low!F6</f>
@@ -8130,7 +10007,7 @@
         <v>Innovation-maintain</v>
       </c>
       <c r="B7" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C7" s="1">
         <f>Low!F7</f>
@@ -8151,7 +10028,7 @@
         <v>Innovation-rhodium18b</v>
       </c>
       <c r="B8" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C8" s="1">
         <f>Low!F8</f>
@@ -8172,7 +10049,7 @@
         <v>Innovation-rhodium6b</v>
       </c>
       <c r="B9" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C9" s="1">
         <f>Low!F9</f>
@@ -8193,7 +10070,7 @@
         <v>Innovation-triple</v>
       </c>
       <c r="B10" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C10" s="1">
         <f>Low!F10</f>
@@ -8214,7 +10091,7 @@
         <v>Low Baseline</v>
       </c>
       <c r="B11" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C11" s="1">
         <f>Low!F11</f>
@@ -8235,7 +10112,7 @@
         <v>Procure3B</v>
       </c>
       <c r="B12" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C12" s="1">
         <f>Low!F12</f>
@@ -8256,7 +10133,7 @@
         <v>ProcureRhodium</v>
       </c>
       <c r="B13" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C13" s="1">
         <f>Low!F13</f>
@@ -8277,7 +10154,7 @@
         <v>ProcureScaling</v>
       </c>
       <c r="B14" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C14" s="1">
         <f>Low!F14</f>
@@ -8298,7 +10175,7 @@
         <v>Optimal</v>
       </c>
       <c r="B15" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C15" s="1">
         <f>Low!F15</f>
@@ -8319,7 +10196,7 @@
         <v>45Q-2040</v>
       </c>
       <c r="B16" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C16" s="1">
         <f>High!F2</f>
@@ -8340,7 +10217,7 @@
         <v>45Q-2050</v>
       </c>
       <c r="B17" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C17" s="1">
         <f>High!F3</f>
@@ -8361,7 +10238,7 @@
         <v>CDRIA-2035</v>
       </c>
       <c r="B18" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C18" s="1">
         <f>High!F4</f>
@@ -8382,7 +10259,7 @@
         <v>CDRIA-2050</v>
       </c>
       <c r="B19" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C19" s="1">
         <f>High!F5</f>
@@ -8403,7 +10280,7 @@
         <v>High Baseline</v>
       </c>
       <c r="B20" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C20" s="1">
         <f>High!F6</f>
@@ -8424,7 +10301,7 @@
         <v>Innovation-DACHubs</v>
       </c>
       <c r="B21" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C21" s="1">
         <f>High!F7</f>
@@ -8445,7 +10322,7 @@
         <v>Innovation-maintain</v>
       </c>
       <c r="B22" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C22" s="1">
         <f>High!F8</f>
@@ -8466,7 +10343,7 @@
         <v>Innovation-rhodium18b</v>
       </c>
       <c r="B23" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C23" s="1">
         <f>High!F9</f>
@@ -8487,7 +10364,7 @@
         <v>Innovation-rhodium6b</v>
       </c>
       <c r="B24" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C24" s="1">
         <f>High!F10</f>
@@ -8508,7 +10385,7 @@
         <v>Innovation-triple</v>
       </c>
       <c r="B25" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C25" s="1">
         <f>High!F11</f>
@@ -8529,7 +10406,7 @@
         <v>Procure3B</v>
       </c>
       <c r="B26" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C26" s="1">
         <f>High!F12</f>
@@ -8550,7 +10427,7 @@
         <v>ProcureRhodium</v>
       </c>
       <c r="B27" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C27" s="1">
         <f>High!F13</f>
@@ -8571,7 +10448,7 @@
         <v>ProcureScaling</v>
       </c>
       <c r="B28" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C28" s="1">
         <f>High!F14</f>
@@ -8592,7 +10469,7 @@
         <v>Optimal</v>
       </c>
       <c r="B29" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C29" s="1">
         <f>High!F15</f>
@@ -8629,39 +10506,39 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C1" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="E1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="G1" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="H1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="I1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="J1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C2">
         <v>5.4175769899473796</v>
@@ -8693,7 +10570,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C3">
         <v>5.4526751392889503</v>
@@ -8725,7 +10602,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C4">
         <v>5.4176986655229298</v>
@@ -8757,7 +10634,7 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C5">
         <v>5.4325606637280597</v>
@@ -8789,7 +10666,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C6">
         <v>5.4675026820248398</v>
@@ -8821,7 +10698,7 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C7">
         <v>5.4690262916548296</v>
@@ -8853,7 +10730,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C8">
         <v>5.4704807351999003</v>
@@ -8885,7 +10762,7 @@
         <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C9">
         <v>5.4684294412951697</v>
@@ -8917,7 +10794,7 @@
         <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C10">
         <v>5.5007324623894398</v>
@@ -8949,7 +10826,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C11">
         <v>5.4984718932521197</v>
@@ -8981,7 +10858,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C12">
         <v>5.7243968175114803</v>
@@ -9013,7 +10890,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C13">
         <v>5.4812879541932098</v>
@@ -9045,7 +10922,7 @@
         <v>1</v>
       </c>
       <c r="B14" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C14">
         <v>5.5417657965940101</v>
@@ -9077,7 +10954,7 @@
         <v>2</v>
       </c>
       <c r="B15" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C15">
         <v>5.5469377878581998</v>
@@ -9109,7 +10986,7 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C16">
         <v>5.6382572848615498</v>
@@ -9141,7 +11018,7 @@
         <v>6</v>
       </c>
       <c r="B17" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C17">
         <v>5.4997560593119497</v>
@@ -9173,7 +11050,7 @@
         <v>5</v>
       </c>
       <c r="B18" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C18">
         <v>5.54833513221618</v>
@@ -9205,7 +11082,7 @@
         <v>8</v>
       </c>
       <c r="B19" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C19">
         <v>5.4635976264752202</v>
@@ -9237,7 +11114,7 @@
         <v>7</v>
       </c>
       <c r="B20" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C20">
         <v>5.5358720502600303</v>
@@ -9269,7 +11146,7 @@
         <v>9</v>
       </c>
       <c r="B21" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C21">
         <v>5.5232699771311804</v>
@@ -9301,7 +11178,7 @@
         <v>10</v>
       </c>
       <c r="B22" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C22">
         <v>5.6119825340455902</v>
@@ -9333,7 +11210,7 @@
         <v>11</v>
       </c>
       <c r="B23" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C23">
         <v>5.8166522657457698</v>
@@ -9365,7 +11242,7 @@
         <v>12</v>
       </c>
       <c r="B24" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C24">
         <v>5.5985806170975803</v>
@@ -9394,10 +11271,10 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B25" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C25">
         <v>5.59858089366009</v>
@@ -9426,10 +11303,10 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B26" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C26">
         <v>5.6764675158573299</v>
@@ -9458,10 +11335,10 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B27" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C27">
         <v>5.3010462151932503</v>
@@ -9490,10 +11367,10 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B28" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C28">
         <v>5.5504529880081197</v>
@@ -9538,19 +11415,19 @@
         <v>Cost Decrease necessary in size of the CDR market in 2050</v>
       </c>
       <c r="E31" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F31" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="G31" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="H31" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="I31" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
@@ -10154,8 +12031,8 @@
     </sortState>
   </autoFilter>
   <phoneticPr fontId="3" type="noConversion"/>
-  <conditionalFormatting sqref="E35:Z35 E36:E39">
-    <cfRule type="colorScale" priority="2">
+  <conditionalFormatting sqref="D2:D28 F2:F28 H2:I28">
+    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="num" val="0"/>
@@ -10166,8 +12043,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D28 F2:F28 H2:I28">
-    <cfRule type="colorScale" priority="1">
+  <conditionalFormatting sqref="E35:Z35 E36:E39">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="num" val="0"/>
@@ -10205,35 +12082,35 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C1" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E1" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F1" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="G1" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="H1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="L1">
         <f>CORREL(D2:D23,F2:F23)</f>
         <v>0.67272727272727262</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="O1">
         <f>CORREL(C2:C23,H2:H23)</f>
@@ -10245,7 +12122,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C2">
         <v>-0.70390616075908496</v>
@@ -10271,7 +12148,7 @@
         <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -10297,7 +12174,7 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C4">
         <v>-0.78055119327006905</v>
@@ -10323,7 +12200,7 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C5">
         <v>-3.7041148122252601</v>
@@ -10349,7 +12226,7 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C6">
         <v>-4.6760340109967</v>
@@ -10375,7 +12252,7 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C7">
         <v>-0.79606851539385404</v>
@@ -10401,7 +12278,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C8">
         <v>-6.2792075696240897</v>
@@ -10427,7 +12304,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C9">
         <v>-4.5270896828626404</v>
@@ -10453,7 +12330,7 @@
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C10">
         <v>-0.43719754556903001</v>
@@ -10479,7 +12356,7 @@
         <v>5</v>
       </c>
       <c r="B11" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C11">
         <v>-3.9166135590809201</v>
@@ -10505,7 +12382,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C12">
         <v>3.6940786172137897E-2</v>
@@ -10531,7 +12408,7 @@
         <v>5</v>
       </c>
       <c r="B13" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C13">
         <v>-1.7952663161307201</v>
@@ -10557,7 +12434,7 @@
         <v>1</v>
       </c>
       <c r="B14" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C14">
         <v>-0.55420087336513202</v>
@@ -10583,7 +12460,7 @@
         <v>8</v>
       </c>
       <c r="B15" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C15">
         <v>-3.2383964853381602</v>
@@ -10609,7 +12486,7 @@
         <v>13</v>
       </c>
       <c r="B16" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -10635,7 +12512,7 @@
         <v>9</v>
       </c>
       <c r="B17" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C17">
         <v>-2.2891584853534401</v>
@@ -10661,7 +12538,7 @@
         <v>7</v>
       </c>
       <c r="B18" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C18">
         <v>-2.2172361920194099</v>
@@ -10687,7 +12564,7 @@
         <v>12</v>
       </c>
       <c r="B19" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C19">
         <v>-0.10194222025196401</v>
@@ -10713,7 +12590,7 @@
         <v>6</v>
       </c>
       <c r="B20" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C20">
         <v>-1.20099872998618</v>
@@ -10739,7 +12616,7 @@
         <v>2</v>
       </c>
       <c r="B21" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C21">
         <v>-0.55690592949661299</v>
@@ -10765,7 +12642,7 @@
         <v>10</v>
       </c>
       <c r="B22" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C22">
         <v>-3.1121273134907899E-2</v>
@@ -10791,7 +12668,7 @@
         <v>11</v>
       </c>
       <c r="B23" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C23">
         <v>4.9027927127704499E-2</v>

</xml_diff>

<commit_message>
some more scenario comparisons
</commit_message>
<xml_diff>
--- a/data/data_analysis/policy_effectiveness.xlsx
+++ b/data/data_analysis/policy_effectiveness.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\data\data_analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4876D8D1-E0E9-48E5-8ABD-177D1C1E9261}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6E389DF-F9AA-40E8-9A37-58DCB08A81F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{5B094011-67C9-461D-BBBF-A6D3FE50B4AB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{5B094011-67C9-461D-BBBF-A6D3FE50B4AB}"/>
   </bookViews>
   <sheets>
     <sheet name="Low" sheetId="1" r:id="rId1"/>
@@ -26,6 +26,14 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Net-Zero Mandate'!$A$1:$H$26</definedName>
     <definedName name="_xlchart.v1.0" hidden="1">'Net-Zero Mandate'!$A$2:$B$28</definedName>
     <definedName name="_xlchart.v1.1" hidden="1">'Net-Zero Mandate'!$D$1</definedName>
+    <definedName name="_xlchart.v1.10" hidden="1">'Net-Zero Mandate'!$D$1</definedName>
+    <definedName name="_xlchart.v1.11" hidden="1">'Net-Zero Mandate'!$D$2:$D$28</definedName>
+    <definedName name="_xlchart.v1.12" hidden="1">'Net-Zero Mandate'!$F$1</definedName>
+    <definedName name="_xlchart.v1.13" hidden="1">'Net-Zero Mandate'!$F$2:$F$28</definedName>
+    <definedName name="_xlchart.v1.14" hidden="1">'Net-Zero Mandate'!$H$1</definedName>
+    <definedName name="_xlchart.v1.15" hidden="1">'Net-Zero Mandate'!$H$2:$H$28</definedName>
+    <definedName name="_xlchart.v1.16" hidden="1">'Net-Zero Mandate'!$I$1</definedName>
+    <definedName name="_xlchart.v1.17" hidden="1">'Net-Zero Mandate'!$I$2:$I$28</definedName>
     <definedName name="_xlchart.v1.2" hidden="1">'Net-Zero Mandate'!$D$2:$D$28</definedName>
     <definedName name="_xlchart.v1.3" hidden="1">'Net-Zero Mandate'!$F$1</definedName>
     <definedName name="_xlchart.v1.4" hidden="1">'Net-Zero Mandate'!$F$2:$F$28</definedName>
@@ -33,6 +41,7 @@
     <definedName name="_xlchart.v1.6" hidden="1">'Net-Zero Mandate'!$H$2:$H$28</definedName>
     <definedName name="_xlchart.v1.7" hidden="1">'Net-Zero Mandate'!$I$1</definedName>
     <definedName name="_xlchart.v1.8" hidden="1">'Net-Zero Mandate'!$I$2:$I$28</definedName>
+    <definedName name="_xlchart.v1.9" hidden="1">'Net-Zero Mandate'!$A$2:$B$28</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -55,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="70">
   <si>
     <t>Scenario</t>
   </si>
@@ -257,6 +266,15 @@
   <si>
     <t>20% Costs</t>
   </si>
+  <si>
+    <t>t C</t>
+  </si>
+  <si>
+    <t>tC</t>
+  </si>
+  <si>
+    <t>tCO2</t>
+  </si>
 </sst>
 </file>
 
@@ -266,7 +284,7 @@
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
-    <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -326,7 +344,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1627,82 +1645,82 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>7.9722193986204699</c:v>
+                  <c:v>0.64785695536394483</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.18215697221197E-2</c:v>
+                  <c:v>2.2459408657409443E-3</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3.27434679522118</c:v>
+                  <c:v>0.27657518865875208</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>11.080702210154501</c:v>
+                  <c:v>0.9215502090713279</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>13.3924163736789</c:v>
+                  <c:v>0.94967366043744428</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>12.090518117610101</c:v>
+                  <c:v>0.97652041402801693</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>11.804833462263</c:v>
+                  <c:v>0.93865673606761379</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>17.279164053851499</c:v>
+                  <c:v>1.5349199946093965</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>16.858636173362701</c:v>
+                  <c:v>1.4931934230901602</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>58.794583510587898</c:v>
+                  <c:v>5.6634142557350327</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>13.3113794026041</c:v>
+                  <c:v>1.176004777856402</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>10.5657233468163</c:v>
+                  <c:v>2.2923311819484971</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>18.574625943324801</c:v>
+                  <c:v>2.3877980534629502</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>17.3728711500404</c:v>
+                  <c:v>4.073413175736218</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>6.9142507501659596</c:v>
+                  <c:v>1.5168971205588402</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>10.9377981211906</c:v>
+                  <c:v>2.4135908453433994</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>4.3055182785194903</c:v>
+                  <c:v>0.84946898979441365</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>10.094129555691</c:v>
+                  <c:v>2.1835418404233824</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>9.1295821492606297</c:v>
+                  <c:v>1.950927275789899</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>15.5568590322536</c:v>
+                  <c:v>3.5884223603825314</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>30.603730057832198</c:v>
+                  <c:v>7.3663055742243611</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>14.5016716897262</c:v>
+                  <c:v>3.341043929529071</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>8.9909705744803396</c:v>
+                  <c:v>3.3410490344405526</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>7.5077860222692498</c:v>
+                  <c:v>4.778714292207316</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>-38.3720249610137</c:v>
+                  <c:v>-2.1509758877512724</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>14.3309846710661</c:v>
+                  <c:v>2.4526831516616943</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1717,82 +1735,82 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.1065459229826602</c:v>
+                  <c:v>0.21249703186680166</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-32.193007747667103</c:v>
+                  <c:v>-1.3655573070193403</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-4.7661224787360901</c:v>
+                  <c:v>-0.46376197004718345</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-1.6578001841819501</c:v>
+                  <c:v>-0.15840906711694819</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-17.610796138934401</c:v>
+                  <c:v>-1.4997785764247658</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-4.2330036189303399</c:v>
+                  <c:v>-0.39769251330281402</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-5.6982743163725003</c:v>
+                  <c:v>-0.52357713726908883</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>10.550045036612699</c:v>
+                  <c:v>1.0818447048699995</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>3.6313721464693201</c:v>
+                  <c:v>0.36638009527595833</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>11.060630810043</c:v>
+                  <c:v>1.1959723569841303</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>3.6008171018680599</c:v>
+                  <c:v>0.36328086889841033</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2.9193308209991198</c:v>
+                  <c:v>1.0676371229122197</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2.9106502559085001</c:v>
+                  <c:v>0.46865683829263816</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>6.3225799064404198</c:v>
+                  <c:v>2.3727693973872075</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>-3.1562896930530902</c:v>
+                  <c:v>-1.0959771479748042</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>-1.91250657480905</c:v>
+                  <c:v>-0.67455579376899111</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>-14.256171407604199</c:v>
+                  <c:v>-4.6305696962614666</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>-3.7834628368867498</c:v>
+                  <c:v>-1.319407624914968</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>-5.5231217389472302</c:v>
+                  <c:v>-1.897612583824104</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2.8341151029912499</c:v>
+                  <c:v>1.0363250084620061</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>7.8453238562851402</c:v>
+                  <c:v>2.923407082508354</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>2.51401455023696</c:v>
+                  <c:v>0.91897387304034173</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>-5.8747233323781796</c:v>
+                  <c:v>-3.8617004313604051</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>18.9014044107759</c:v>
+                  <c:v>23.306697574041493</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>-16.938204157826199</c:v>
+                  <c:v>-1.4445409002888128</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>-14.693518666643</c:v>
+                  <c:v>-4.7728156685049763</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1998,39 +2016,19 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:chart>
-    <c:title>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
+    <c:autoTitleDeleted val="1"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="8.7487789964051293E-2"/>
+          <c:y val="9.5648818834036059E-2"/>
+          <c:w val="0.86045319240557017"/>
+          <c:h val="0.82694066899082042"/>
+        </c:manualLayout>
+      </c:layout>
       <c:scatterChart>
         <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
@@ -2080,82 +2078,82 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.1065459229826602</c:v>
+                  <c:v>0.21249703186680166</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-32.193007747667103</c:v>
+                  <c:v>-1.3655573070193403</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-4.7661224787360901</c:v>
+                  <c:v>-0.46376197004718345</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-1.6578001841819501</c:v>
+                  <c:v>-0.15840906711694819</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-17.610796138934401</c:v>
+                  <c:v>-1.4997785764247658</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-4.2330036189303399</c:v>
+                  <c:v>-0.39769251330281402</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-5.6982743163725003</c:v>
+                  <c:v>-0.52357713726908883</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>10.550045036612699</c:v>
+                  <c:v>1.0818447048699995</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>3.6313721464693201</c:v>
+                  <c:v>0.36638009527595833</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>11.060630810043</c:v>
+                  <c:v>1.1959723569841303</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>3.6008171018680599</c:v>
+                  <c:v>0.36328086889841033</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2.9193308209991198</c:v>
+                  <c:v>1.0676371229122197</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2.9106502559085001</c:v>
+                  <c:v>0.46865683829263816</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>6.3225799064404198</c:v>
+                  <c:v>2.3727693973872075</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>-3.1562896930530902</c:v>
+                  <c:v>-1.0959771479748042</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>-1.91250657480905</c:v>
+                  <c:v>-0.67455579376899111</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>-14.256171407604199</c:v>
+                  <c:v>-4.6305696962614666</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>-3.7834628368867498</c:v>
+                  <c:v>-1.319407624914968</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>-5.5231217389472302</c:v>
+                  <c:v>-1.897612583824104</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2.8341151029912499</c:v>
+                  <c:v>1.0363250084620061</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>7.8453238562851402</c:v>
+                  <c:v>2.923407082508354</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>2.51401455023696</c:v>
+                  <c:v>0.91897387304034173</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>-5.8747233323781796</c:v>
+                  <c:v>-3.8617004313604051</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>18.9014044107759</c:v>
+                  <c:v>23.306697574041493</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>-16.938204157826199</c:v>
+                  <c:v>-1.4445409002888128</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>-14.693518666643</c:v>
+                  <c:v>-4.7728156685049763</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2167,34 +2165,34 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="27"/>
                 <c:pt idx="3">
-                  <c:v>3.27434679522118</c:v>
+                  <c:v>0.27657518865875208</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>11.080702210154501</c:v>
+                  <c:v>0.9215502090713279</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>13.3924163736789</c:v>
+                  <c:v>0.94967366043744428</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>12.090518117610101</c:v>
+                  <c:v>0.97652041402801693</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>11.804833462263</c:v>
+                  <c:v>0.93865673606761379</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>6.9142507501659596</c:v>
+                  <c:v>1.5168971205588402</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>10.9377981211906</c:v>
+                  <c:v>2.4135908453433994</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>4.3055182785194903</c:v>
+                  <c:v>0.84946898979441365</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>10.094129555691</c:v>
+                  <c:v>2.1835418404233824</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>9.1295821492606297</c:v>
+                  <c:v>1.950927275789899</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2252,82 +2250,82 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.1065459229826602</c:v>
+                  <c:v>0.21249703186680166</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-32.193007747667103</c:v>
+                  <c:v>-1.3655573070193403</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-4.7661224787360901</c:v>
+                  <c:v>-0.46376197004718345</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-1.6578001841819501</c:v>
+                  <c:v>-0.15840906711694819</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-17.610796138934401</c:v>
+                  <c:v>-1.4997785764247658</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-4.2330036189303399</c:v>
+                  <c:v>-0.39769251330281402</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-5.6982743163725003</c:v>
+                  <c:v>-0.52357713726908883</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>10.550045036612699</c:v>
+                  <c:v>1.0818447048699995</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>3.6313721464693201</c:v>
+                  <c:v>0.36638009527595833</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>11.060630810043</c:v>
+                  <c:v>1.1959723569841303</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>3.6008171018680599</c:v>
+                  <c:v>0.36328086889841033</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2.9193308209991198</c:v>
+                  <c:v>1.0676371229122197</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2.9106502559085001</c:v>
+                  <c:v>0.46865683829263816</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>6.3225799064404198</c:v>
+                  <c:v>2.3727693973872075</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>-3.1562896930530902</c:v>
+                  <c:v>-1.0959771479748042</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>-1.91250657480905</c:v>
+                  <c:v>-0.67455579376899111</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>-14.256171407604199</c:v>
+                  <c:v>-4.6305696962614666</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>-3.7834628368867498</c:v>
+                  <c:v>-1.319407624914968</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>-5.5231217389472302</c:v>
+                  <c:v>-1.897612583824104</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2.8341151029912499</c:v>
+                  <c:v>1.0363250084620061</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>7.8453238562851402</c:v>
+                  <c:v>2.923407082508354</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>2.51401455023696</c:v>
+                  <c:v>0.91897387304034173</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>-5.8747233323781796</c:v>
+                  <c:v>-3.8617004313604051</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>18.9014044107759</c:v>
+                  <c:v>23.306697574041493</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>-16.938204157826199</c:v>
+                  <c:v>-1.4445409002888128</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>-14.693518666643</c:v>
+                  <c:v>-4.7728156685049763</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2339,16 +2337,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="27"/>
                 <c:pt idx="1">
-                  <c:v>7.9722193986204699</c:v>
+                  <c:v>0.64785695536394483</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.18215697221197E-2</c:v>
+                  <c:v>2.2459408657409443E-3</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>10.5657233468163</c:v>
+                  <c:v>2.2923311819484971</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>18.574625943324801</c:v>
+                  <c:v>2.3877980534629502</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2406,82 +2404,82 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.1065459229826602</c:v>
+                  <c:v>0.21249703186680166</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-32.193007747667103</c:v>
+                  <c:v>-1.3655573070193403</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-4.7661224787360901</c:v>
+                  <c:v>-0.46376197004718345</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-1.6578001841819501</c:v>
+                  <c:v>-0.15840906711694819</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-17.610796138934401</c:v>
+                  <c:v>-1.4997785764247658</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-4.2330036189303399</c:v>
+                  <c:v>-0.39769251330281402</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-5.6982743163725003</c:v>
+                  <c:v>-0.52357713726908883</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>10.550045036612699</c:v>
+                  <c:v>1.0818447048699995</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>3.6313721464693201</c:v>
+                  <c:v>0.36638009527595833</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>11.060630810043</c:v>
+                  <c:v>1.1959723569841303</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>3.6008171018680599</c:v>
+                  <c:v>0.36328086889841033</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2.9193308209991198</c:v>
+                  <c:v>1.0676371229122197</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2.9106502559085001</c:v>
+                  <c:v>0.46865683829263816</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>6.3225799064404198</c:v>
+                  <c:v>2.3727693973872075</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>-3.1562896930530902</c:v>
+                  <c:v>-1.0959771479748042</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>-1.91250657480905</c:v>
+                  <c:v>-0.67455579376899111</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>-14.256171407604199</c:v>
+                  <c:v>-4.6305696962614666</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>-3.7834628368867498</c:v>
+                  <c:v>-1.319407624914968</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>-5.5231217389472302</c:v>
+                  <c:v>-1.897612583824104</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2.8341151029912499</c:v>
+                  <c:v>1.0363250084620061</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>7.8453238562851402</c:v>
+                  <c:v>2.923407082508354</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>2.51401455023696</c:v>
+                  <c:v>0.91897387304034173</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>-5.8747233323781796</c:v>
+                  <c:v>-3.8617004313604051</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>18.9014044107759</c:v>
+                  <c:v>23.306697574041493</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>-16.938204157826199</c:v>
+                  <c:v>-1.4445409002888128</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>-14.693518666643</c:v>
+                  <c:v>-4.7728156685049763</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2493,22 +2491,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="27"/>
                 <c:pt idx="9">
-                  <c:v>16.858636173362701</c:v>
+                  <c:v>1.4931934230901602</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>58.794583510587898</c:v>
+                  <c:v>5.6634142557350327</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>13.3113794026041</c:v>
+                  <c:v>1.176004777856402</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>15.5568590322536</c:v>
+                  <c:v>3.5884223603825314</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>30.603730057832198</c:v>
+                  <c:v>7.3663055742243611</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>14.5016716897262</c:v>
+                  <c:v>3.341043929529071</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2566,82 +2564,82 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.1065459229826602</c:v>
+                  <c:v>0.21249703186680166</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-32.193007747667103</c:v>
+                  <c:v>-1.3655573070193403</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-4.7661224787360901</c:v>
+                  <c:v>-0.46376197004718345</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-1.6578001841819501</c:v>
+                  <c:v>-0.15840906711694819</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-17.610796138934401</c:v>
+                  <c:v>-1.4997785764247658</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-4.2330036189303399</c:v>
+                  <c:v>-0.39769251330281402</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-5.6982743163725003</c:v>
+                  <c:v>-0.52357713726908883</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>10.550045036612699</c:v>
+                  <c:v>1.0818447048699995</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>3.6313721464693201</c:v>
+                  <c:v>0.36638009527595833</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>11.060630810043</c:v>
+                  <c:v>1.1959723569841303</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>3.6008171018680599</c:v>
+                  <c:v>0.36328086889841033</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2.9193308209991198</c:v>
+                  <c:v>1.0676371229122197</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2.9106502559085001</c:v>
+                  <c:v>0.46865683829263816</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>6.3225799064404198</c:v>
+                  <c:v>2.3727693973872075</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>-3.1562896930530902</c:v>
+                  <c:v>-1.0959771479748042</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>-1.91250657480905</c:v>
+                  <c:v>-0.67455579376899111</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>-14.256171407604199</c:v>
+                  <c:v>-4.6305696962614666</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>-3.7834628368867498</c:v>
+                  <c:v>-1.319407624914968</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>-5.5231217389472302</c:v>
+                  <c:v>-1.897612583824104</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2.8341151029912499</c:v>
+                  <c:v>1.0363250084620061</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>7.8453238562851402</c:v>
+                  <c:v>2.923407082508354</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>2.51401455023696</c:v>
+                  <c:v>0.91897387304034173</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>-5.8747233323781796</c:v>
+                  <c:v>-3.8617004313604051</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>18.9014044107759</c:v>
+                  <c:v>23.306697574041493</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>-16.938204157826199</c:v>
+                  <c:v>-1.4445409002888128</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>-14.693518666643</c:v>
+                  <c:v>-4.7728156685049763</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2653,10 +2651,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="27"/>
                 <c:pt idx="25">
-                  <c:v>-38.3720249610137</c:v>
+                  <c:v>-2.1509758877512724</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>14.3309846710661</c:v>
+                  <c:v>2.4526831516616943</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2714,82 +2712,82 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.1065459229826602</c:v>
+                  <c:v>0.21249703186680166</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-32.193007747667103</c:v>
+                  <c:v>-1.3655573070193403</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-4.7661224787360901</c:v>
+                  <c:v>-0.46376197004718345</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-1.6578001841819501</c:v>
+                  <c:v>-0.15840906711694819</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-17.610796138934401</c:v>
+                  <c:v>-1.4997785764247658</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-4.2330036189303399</c:v>
+                  <c:v>-0.39769251330281402</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-5.6982743163725003</c:v>
+                  <c:v>-0.52357713726908883</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>10.550045036612699</c:v>
+                  <c:v>1.0818447048699995</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>3.6313721464693201</c:v>
+                  <c:v>0.36638009527595833</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>11.060630810043</c:v>
+                  <c:v>1.1959723569841303</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>3.6008171018680599</c:v>
+                  <c:v>0.36328086889841033</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2.9193308209991198</c:v>
+                  <c:v>1.0676371229122197</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2.9106502559085001</c:v>
+                  <c:v>0.46865683829263816</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>6.3225799064404198</c:v>
+                  <c:v>2.3727693973872075</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>-3.1562896930530902</c:v>
+                  <c:v>-1.0959771479748042</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>-1.91250657480905</c:v>
+                  <c:v>-0.67455579376899111</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>-14.256171407604199</c:v>
+                  <c:v>-4.6305696962614666</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>-3.7834628368867498</c:v>
+                  <c:v>-1.319407624914968</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>-5.5231217389472302</c:v>
+                  <c:v>-1.897612583824104</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2.8341151029912499</c:v>
+                  <c:v>1.0363250084620061</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>7.8453238562851402</c:v>
+                  <c:v>2.923407082508354</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>2.51401455023696</c:v>
+                  <c:v>0.91897387304034173</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>-5.8747233323781796</c:v>
+                  <c:v>-3.8617004313604051</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>18.9014044107759</c:v>
+                  <c:v>23.306697574041493</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>-16.938204157826199</c:v>
+                  <c:v>-1.4445409002888128</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>-14.693518666643</c:v>
+                  <c:v>-4.7728156685049763</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2804,16 +2802,16 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>17.279164053851499</c:v>
+                  <c:v>1.5349199946093965</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>17.3728711500404</c:v>
+                  <c:v>4.073413175736218</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>8.9909705744803396</c:v>
+                  <c:v>3.3410490344405526</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>7.5077860222692498</c:v>
+                  <c:v>4.778714292207316</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2864,7 +2862,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="65000"/>
@@ -2877,14 +2875,14 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="en-US"/>
+                  <a:rPr lang="en-US" sz="1400"/>
                   <a:t>Change in 2050 cost effectiveness from</a:t>
                 </a:r>
                 <a:r>
-                  <a:rPr lang="en-US" baseline="0"/>
-                  <a:t> baseline</a:t>
+                  <a:rPr lang="en-US" sz="1400" baseline="0"/>
+                  <a:t> efficient scenario (%)</a:t>
                 </a:r>
-                <a:endParaRPr lang="en-US"/>
+                <a:endParaRPr lang="en-US" sz="1400"/>
               </a:p>
             </c:rich>
           </c:tx>
@@ -2901,7 +2899,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
                     <a:schemeClr val="tx1">
                       <a:lumMod val="65000"/>
@@ -2939,7 +2937,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -2986,7 +2984,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="65000"/>
@@ -2999,12 +2997,28 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="en-US"/>
-                  <a:t>Change in NPV from Baseline</a:t>
+                  <a:rPr lang="en-US" sz="1400"/>
+                  <a:t>Change in NPV from efficient</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1400" baseline="0"/>
+                  <a:t> scenario</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1400"/>
+                  <a:t> (%)</a:t>
                 </a:r>
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="3.2156184287128318E-2"/>
+              <c:y val="0.2133207649709703"/>
+            </c:manualLayout>
+          </c:layout>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -3018,7 +3032,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
                     <a:schemeClr val="tx1">
                       <a:lumMod val="65000"/>
@@ -3056,7 +3070,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -3085,9 +3099,23 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.5898129642232609"/>
+          <c:y val="0.38244392172116509"/>
+          <c:w val="0.18739061607306434"/>
+          <c:h val="0.25525532296155895"/>
+        </c:manualLayout>
+      </c:layout>
       <c:overlay val="0"/>
       <c:spPr>
-        <a:noFill/>
+        <a:solidFill>
+          <a:schemeClr val="bg1">
+            <a:alpha val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
         <a:ln>
           <a:noFill/>
         </a:ln>
@@ -3098,7 +3126,7 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+            <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="65000"/>
@@ -3260,10 +3288,10 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr algn="ctr" rtl="0">
-                <a:defRPr/>
+                <a:defRPr sz="1400"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:sysClr val="windowText" lastClr="000000">
                       <a:lumMod val="65000"/>
@@ -3278,13 +3306,31 @@
           </cx:txPr>
         </cx:title>
         <cx:tickLabels/>
+        <cx:txPr>
+          <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr" rtl="0">
+              <a:defRPr sz="1200"/>
+            </a:pPr>
+            <a:endParaRPr lang="en-US" sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+              <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+            </a:endParaRPr>
+          </a:p>
+        </cx:txPr>
       </cx:axis>
       <cx:axis id="1">
         <cx:valScaling/>
         <cx:title>
           <cx:tx>
             <cx:txData>
-              <cx:v>% of the size of the CDR market</cx:v>
+              <cx:v>% of NPV of efficient pathway</cx:v>
             </cx:txData>
           </cx:tx>
           <cx:txPr>
@@ -3292,10 +3338,10 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr algn="ctr" rtl="0">
-                <a:defRPr/>
+                <a:defRPr sz="1400"/>
               </a:pPr>
               <a:r>
-                <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
                   <a:solidFill>
                     <a:sysClr val="windowText" lastClr="000000">
                       <a:lumMod val="65000"/>
@@ -3304,16 +3350,53 @@
                   </a:solidFill>
                   <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
                 </a:rPr>
-                <a:t>% of the size of the CDR market</a:t>
+                <a:t>% of NPV of efficient pathway</a:t>
               </a:r>
             </a:p>
           </cx:txPr>
         </cx:title>
         <cx:majorGridlines/>
         <cx:tickLabels/>
+        <cx:txPr>
+          <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr" rtl="0">
+              <a:defRPr sz="1200"/>
+            </a:pPr>
+            <a:endParaRPr lang="en-US" sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+              <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+            </a:endParaRPr>
+          </a:p>
+        </cx:txPr>
       </cx:axis>
     </cx:plotArea>
-    <cx:legend pos="t" align="ctr" overlay="0"/>
+    <cx:legend pos="t" align="ctr" overlay="0">
+      <cx:txPr>
+        <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr sz="1050"/>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="1050" b="0" i="0" u="none" strike="noStrike" baseline="0">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000">
+                <a:lumMod val="65000"/>
+                <a:lumOff val="35000"/>
+              </a:sysClr>
+            </a:solidFill>
+            <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+          </a:endParaRPr>
+        </a:p>
+      </cx:txPr>
+    </cx:legend>
   </cx:chart>
 </cx:chartSpace>
 </file>
@@ -5736,16 +5819,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>552450</xdr:colOff>
-      <xdr:row>53</xdr:row>
-      <xdr:rowOff>161925</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>457200</xdr:colOff>
-      <xdr:row>56</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>400050</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -5760,13 +5843,17 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8934450" y="10258425"/>
-          <a:ext cx="1733550" cy="438150"/>
+          <a:off x="9067800" y="9505950"/>
+          <a:ext cx="933450" cy="1143000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
+        <a:solidFill>
+          <a:schemeClr val="bg1">
+            <a:alpha val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
         <a:ln w="9525" cmpd="sng">
           <a:solidFill>
             <a:schemeClr val="lt1">
@@ -5809,16 +5896,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>476250</xdr:colOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
       <xdr:row>33</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>381000</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -5833,13 +5920,17 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11296650" y="6410325"/>
+          <a:off x="12087225" y="6438900"/>
           <a:ext cx="1733550" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
+        <a:solidFill>
+          <a:schemeClr val="bg1">
+            <a:alpha val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
         <a:ln w="9525" cmpd="sng">
           <a:solidFill>
             <a:schemeClr val="lt1">
@@ -5882,16 +5973,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>542925</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>85725</xdr:colOff>
       <xdr:row>33</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
+      <xdr:rowOff>152399</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>447675</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>419100</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -5906,13 +5997,17 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8924925" y="6419850"/>
-          <a:ext cx="1733550" cy="438150"/>
+          <a:off x="9077325" y="6438899"/>
+          <a:ext cx="942975" cy="1019176"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
+        <a:solidFill>
+          <a:schemeClr val="bg1">
+            <a:alpha val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
         <a:ln w="9525" cmpd="sng">
           <a:solidFill>
             <a:schemeClr val="lt1">
@@ -5955,16 +6050,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>495300</xdr:colOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
       <xdr:row>53</xdr:row>
-      <xdr:rowOff>161925</xdr:rowOff>
+      <xdr:rowOff>104775</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>400050</xdr:colOff>
-      <xdr:row>56</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>552450</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -5979,13 +6074,17 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11315700" y="10258425"/>
+          <a:off x="12077700" y="10201275"/>
           <a:ext cx="1733550" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
+        <a:solidFill>
+          <a:schemeClr val="bg1">
+            <a:alpha val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
         <a:ln w="9525" cmpd="sng">
           <a:solidFill>
             <a:schemeClr val="lt1">
@@ -9800,18 +9899,6 @@
       <sortCondition ref="A1"/>
     </sortState>
   </autoFilter>
-  <conditionalFormatting sqref="L2:L15 H2:H15 D2:D15">
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="num" val="-1"/>
-        <cfvo type="max"/>
-        <color theme="6"/>
-        <color theme="0"/>
-        <color rgb="FFC00000"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="D18:D31">
     <cfRule type="colorScale" priority="3">
       <colorScale>
@@ -9826,6 +9913,18 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="H18:H31">
     <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="num" val="-1"/>
+        <cfvo type="max"/>
+        <color theme="6"/>
+        <color theme="0"/>
+        <color rgb="FFC00000"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L2:L15 H2:H15 D2:D15">
+    <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="num" val="-1"/>
@@ -9854,7 +9953,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A1C2576-3F3B-4E71-BDB4-1E4541BB8CBE}">
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:N30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="15.140625" bestFit="1" customWidth="1"/>
@@ -10211,7 +10310,7 @@
         <v>-24012.4014868552</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" t="str">
         <f>High!A3</f>
         <v>45Q-2050</v>
@@ -10232,7 +10331,7 @@
         <v>-84257.525916830593</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" t="str">
         <f>High!A4</f>
         <v>CDRIA-2035</v>
@@ -10253,7 +10352,7 @@
         <v>-74162.1476601756</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" t="str">
         <f>High!A5</f>
         <v>CDRIA-2050</v>
@@ -10274,7 +10373,7 @@
         <v>-265902.76421105402</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" t="str">
         <f>High!A6</f>
         <v>High Baseline</v>
@@ -10295,7 +10394,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" t="str">
         <f>High!A7</f>
         <v>Innovation-DACHubs</v>
@@ -10316,7 +10415,7 @@
         <v>-14041.807010664401</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" t="str">
         <f>High!A8</f>
         <v>Innovation-maintain</v>
@@ -10337,7 +10436,7 @@
         <v>-12795.920628411601</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" t="str">
         <f>High!A9</f>
         <v>Innovation-rhodium18b</v>
@@ -10358,7 +10457,7 @@
         <v>-38626.101035459098</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" t="str">
         <f>High!A10</f>
         <v>Innovation-rhodium6b</v>
@@ -10379,7 +10478,7 @@
         <v>-17986.986790839499</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" t="str">
         <f>High!A11</f>
         <v>Innovation-triple</v>
@@ -10400,7 +10499,7 @@
         <v>-20252.154009836198</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" t="str">
         <f>High!A12</f>
         <v>Procure3B</v>
@@ -10421,7 +10520,7 @@
         <v>-2555.2191726661399</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" t="str">
         <f>High!A13</f>
         <v>ProcureRhodium</v>
@@ -10442,7 +10541,7 @@
         <v>5157.5221174354301</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" t="str">
         <f>High!A14</f>
         <v>ProcureScaling</v>
@@ -10463,7 +10562,7 @@
         <v>-2707.91448460225</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" t="str">
         <f>High!A15</f>
         <v>Optimal</v>
@@ -10482,6 +10581,26 @@
       <c r="I29" s="1">
         <f>C29</f>
         <v>-100078.99781724501</v>
+      </c>
+      <c r="L29">
+        <v>1990</v>
+      </c>
+      <c r="M29">
+        <v>2025</v>
+      </c>
+      <c r="N29" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="L30" t="s">
+        <v>67</v>
+      </c>
+      <c r="M30">
+        <v>1990</v>
+      </c>
+      <c r="N30" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -10544,21 +10663,25 @@
         <v>5.4175769899473796</v>
       </c>
       <c r="D2">
+        <f>100*(C2-C$2)/C$2</f>
         <v>0</v>
       </c>
       <c r="E2">
         <v>1.21462324059764</v>
       </c>
       <c r="F2">
+        <f>100*(E2-E$2)/E$2</f>
         <v>0</v>
       </c>
       <c r="G2">
         <v>0.50517645710506498</v>
       </c>
       <c r="H2">
+        <f>100*(G2-G$2)/G$2</f>
         <v>0</v>
       </c>
       <c r="I2">
+        <f>100*(J2-J$2)/J$2</f>
         <v>0</v>
       </c>
       <c r="J2">
@@ -10576,22 +10699,26 @@
         <v>5.4526751392889503</v>
       </c>
       <c r="D3">
-        <v>7.9722193986204699</v>
+        <f t="shared" ref="D3:F28" si="0">100*(C3-C$2)/C$2</f>
+        <v>0.64785695536394483</v>
       </c>
       <c r="E3">
         <v>1.2265993616247699</v>
       </c>
       <c r="F3">
-        <v>12.943976807287701</v>
+        <f t="shared" si="0"/>
+        <v>0.98599472057171911</v>
       </c>
       <c r="G3">
         <v>0.51196546571708901</v>
       </c>
       <c r="H3">
-        <v>17.3256530369916</v>
+        <f t="shared" ref="H3" si="1">100*(G3-G$2)/G$2</f>
+        <v>1.3438885594409384</v>
       </c>
       <c r="I3">
-        <v>2.1065459229826602</v>
+        <f t="shared" ref="I3:I28" si="2">100*(J3-J$2)/J$2</f>
+        <v>0.21249703186680166</v>
       </c>
       <c r="J3">
         <v>0.84470017355869997</v>
@@ -10608,22 +10735,26 @@
         <v>5.4176986655229298</v>
       </c>
       <c r="D4">
-        <v>4.18215697221197E-2</v>
+        <f t="shared" si="0"/>
+        <v>2.2459408657409443E-3</v>
       </c>
       <c r="E4">
         <v>1.2200220480936199</v>
       </c>
       <c r="F4">
-        <v>7.3634914210611901</v>
+        <f t="shared" si="0"/>
+        <v>0.44448412606722876</v>
       </c>
       <c r="G4">
         <v>0.50945647219154799</v>
       </c>
       <c r="H4">
-        <v>12.3014623706724</v>
+        <f t="shared" ref="H4" si="3">100*(G4-G$2)/G$2</f>
+        <v>0.84723170018844907</v>
       </c>
       <c r="I4">
-        <v>-32.193007747667103</v>
+        <f t="shared" si="2"/>
+        <v>-1.3655573070193403</v>
       </c>
       <c r="J4">
         <v>0.83139861124438796</v>
@@ -10640,22 +10771,26 @@
         <v>5.4325606637280597</v>
       </c>
       <c r="D5">
-        <v>3.27434679522118</v>
+        <f t="shared" si="0"/>
+        <v>0.27657518865875208</v>
       </c>
       <c r="E5">
         <v>1.2224848613141599</v>
       </c>
       <c r="F5">
-        <v>7.9854624669163199</v>
+        <f t="shared" si="0"/>
+        <v>0.64724767761331869</v>
       </c>
       <c r="G5">
         <v>0.51069933585084104</v>
       </c>
       <c r="H5">
-        <v>13.341427664723501</v>
+        <f t="shared" ref="H5" si="4">100*(G5-G$2)/G$2</f>
+        <v>1.0932573496051559</v>
       </c>
       <c r="I5">
-        <v>-4.7661224787360901</v>
+        <f t="shared" si="2"/>
+        <v>-0.46376197004718345</v>
       </c>
       <c r="J5">
         <v>0.83899992545385804</v>
@@ -10672,22 +10807,26 @@
         <v>5.4675026820248398</v>
       </c>
       <c r="D6">
-        <v>11.080702210154501</v>
+        <f t="shared" si="0"/>
+        <v>0.9215502090713279</v>
       </c>
       <c r="E6">
         <v>1.23111451544623</v>
       </c>
       <c r="F6">
-        <v>16.816335761750899</v>
+        <f t="shared" si="0"/>
+        <v>1.3577275897072081</v>
       </c>
       <c r="G6">
         <v>0.513737215902481</v>
       </c>
       <c r="H6">
-        <v>20.4675390471334</v>
+        <f t="shared" ref="H6" si="5">100*(G6-G$2)/G$2</f>
+        <v>1.6946076320487724</v>
       </c>
       <c r="I6">
-        <v>-1.6578001841819501</v>
+        <f t="shared" si="2"/>
+        <v>-0.15840906711694819</v>
       </c>
       <c r="J6">
         <v>0.84157377260607302</v>
@@ -10704,22 +10843,26 @@
         <v>5.4690262916548296</v>
       </c>
       <c r="D7">
-        <v>13.3924163736789</v>
+        <f t="shared" si="0"/>
+        <v>0.94967366043744428</v>
       </c>
       <c r="E7">
         <v>1.24274587562168</v>
       </c>
       <c r="F7">
-        <v>33.8032802979519</v>
+        <f t="shared" si="0"/>
+        <v>2.3153381298881297</v>
       </c>
       <c r="G7">
         <v>0.52159577509564503</v>
       </c>
       <c r="H7">
-        <v>45.889149664641799</v>
+        <f t="shared" ref="H7" si="6">100*(G7-G$2)/G$2</f>
+        <v>3.2502144071938046</v>
       </c>
       <c r="I7">
-        <v>-17.610796138934401</v>
+        <f t="shared" si="2"/>
+        <v>-1.4997785764247658</v>
       </c>
       <c r="J7">
         <v>0.83026724806194996</v>
@@ -10736,22 +10879,26 @@
         <v>5.4704807351999003</v>
       </c>
       <c r="D8">
-        <v>12.090518117610101</v>
+        <f t="shared" si="0"/>
+        <v>0.97652041402801693</v>
       </c>
       <c r="E8">
         <v>1.2344805645724799</v>
       </c>
       <c r="F8">
-        <v>20.904336245338801</v>
+        <f t="shared" si="0"/>
+        <v>1.6348546043849213</v>
       </c>
       <c r="G8">
         <v>0.51580994167138305</v>
       </c>
       <c r="H8">
-        <v>26.205814883550801</v>
+        <f t="shared" ref="H8" si="7">100*(G8-G$2)/G$2</f>
+        <v>2.1049050122513044</v>
       </c>
       <c r="I8">
-        <v>-4.2330036189303399</v>
+        <f t="shared" si="2"/>
+        <v>-0.39769251330281402</v>
       </c>
       <c r="J8">
         <v>0.83955683086218402</v>
@@ -10768,22 +10915,26 @@
         <v>5.4684294412951697</v>
       </c>
       <c r="D9">
-        <v>11.804833462263</v>
+        <f t="shared" si="0"/>
+        <v>0.93865673606761379</v>
       </c>
       <c r="E9">
         <v>1.23469984643818</v>
       </c>
       <c r="F9">
-        <v>21.4277299143567</v>
+        <f t="shared" si="0"/>
+        <v>1.6529080927729902</v>
       </c>
       <c r="G9">
         <v>0.51633662594582996</v>
       </c>
       <c r="H9">
-        <v>27.919026065915698</v>
+        <f t="shared" ref="H9" si="8">100*(G9-G$2)/G$2</f>
+        <v>2.2091624983315339</v>
       </c>
       <c r="I9">
-        <v>-5.6982743163725003</v>
+        <f t="shared" si="2"/>
+        <v>-0.52357713726908883</v>
       </c>
       <c r="J9">
         <v>0.83849573801586097</v>
@@ -10800,22 +10951,26 @@
         <v>5.5007324623894398</v>
       </c>
       <c r="D10">
-        <v>17.279164053851499</v>
+        <f t="shared" si="0"/>
+        <v>1.5349199946093965</v>
       </c>
       <c r="E10">
         <v>1.2333937815064</v>
       </c>
       <c r="F10">
-        <v>18.019593931069998</v>
+        <f t="shared" si="0"/>
+        <v>1.5453796931733457</v>
       </c>
       <c r="G10">
         <v>0.513172389200656</v>
       </c>
       <c r="H10">
-        <v>18.0957375351921</v>
+        <f t="shared" ref="H10" si="9">100*(G10-G$2)/G$2</f>
+        <v>1.5827998282841693</v>
       </c>
       <c r="I10">
-        <v>10.550045036612699</v>
+        <f t="shared" si="2"/>
+        <v>1.0818447048699995</v>
       </c>
       <c r="J10">
         <v>0.85202798348279696</v>
@@ -10832,22 +10987,26 @@
         <v>5.4984718932521197</v>
       </c>
       <c r="D11">
-        <v>16.858636173362701</v>
+        <f t="shared" si="0"/>
+        <v>1.4931934230901602</v>
       </c>
       <c r="E11">
         <v>1.2461970757383001</v>
       </c>
       <c r="F11">
-        <v>30.32001009859</v>
+        <f t="shared" si="0"/>
+        <v>2.5994756304123183</v>
       </c>
       <c r="G11">
         <v>0.52572239246154995</v>
       </c>
       <c r="H11">
-        <v>46.738446809391498</v>
+        <f t="shared" ref="H11" si="10">100*(G11-G$2)/G$2</f>
+        <v>4.0670809313292864</v>
       </c>
       <c r="I11">
-        <v>3.6313721464693201</v>
+        <f t="shared" si="2"/>
+        <v>0.36638009527595833</v>
       </c>
       <c r="J11">
         <v>0.84599726777568296</v>
@@ -10864,22 +11023,26 @@
         <v>5.7243968175114803</v>
       </c>
       <c r="D12">
-        <v>58.794583510587898</v>
+        <f t="shared" si="0"/>
+        <v>5.6634142557350327</v>
       </c>
       <c r="E12">
         <v>1.3160625148040399</v>
       </c>
       <c r="F12">
-        <v>93.382246268824602</v>
+        <f t="shared" si="0"/>
+        <v>8.3515011746760219</v>
       </c>
       <c r="G12">
         <v>0.56052492044233604</v>
       </c>
       <c r="H12">
-        <v>128.25279781669599</v>
+        <f t="shared" ref="H12" si="11">100*(G12-G$2)/G$2</f>
+        <v>10.956263412283258</v>
       </c>
       <c r="I12">
-        <v>11.060630810043</v>
+        <f t="shared" si="2"/>
+        <v>1.1959723569841303</v>
       </c>
       <c r="J12">
         <v>0.85298997575326196</v>
@@ -10896,22 +11059,26 @@
         <v>5.4812879541932098</v>
       </c>
       <c r="D13">
-        <v>13.3113794026041</v>
+        <f t="shared" si="0"/>
+        <v>1.176004777856402</v>
       </c>
       <c r="E13">
         <v>1.2334114219814001</v>
       </c>
       <c r="F13">
-        <v>18.068472816125901</v>
+        <f t="shared" si="0"/>
+        <v>1.5468320344764317</v>
       </c>
       <c r="G13">
         <v>0.51482952026028495</v>
       </c>
       <c r="H13">
-        <v>21.908114265485199</v>
+        <f t="shared" ref="H13" si="12">100*(G13-G$2)/G$2</f>
+        <v>1.9108299722709272</v>
       </c>
       <c r="I13">
-        <v>3.6008171018680599</v>
+        <f t="shared" si="2"/>
+        <v>0.36328086889841033</v>
       </c>
       <c r="J13">
         <v>0.84597114411709196</v>
@@ -10928,22 +11095,26 @@
         <v>5.5417657965940101</v>
       </c>
       <c r="D14">
-        <v>10.5657233468163</v>
+        <f t="shared" si="0"/>
+        <v>2.2923311819484971</v>
       </c>
       <c r="E14">
         <v>1.2457635282608599</v>
       </c>
       <c r="F14">
-        <v>15.427706085558601</v>
+        <f t="shared" si="0"/>
+        <v>2.5637816421080228</v>
       </c>
       <c r="G14">
         <v>0.51994929271492896</v>
       </c>
       <c r="H14">
-        <v>21.036516548608301</v>
+        <f t="shared" ref="H14" si="13">100*(G14-G$2)/G$2</f>
+        <v>2.9242921759498324</v>
       </c>
       <c r="I14">
-        <v>2.9193308209991198</v>
+        <f t="shared" si="2"/>
+        <v>1.0676371229122197</v>
       </c>
       <c r="J14">
         <v>0.85190822649338904</v>
@@ -10960,22 +11131,26 @@
         <v>5.5469377878581998</v>
       </c>
       <c r="D15">
-        <v>18.574625943324801</v>
+        <f t="shared" si="0"/>
+        <v>2.3877980534629502</v>
       </c>
       <c r="E15">
         <v>1.24906589704301</v>
       </c>
       <c r="F15">
-        <v>24.3236703991907</v>
+        <f t="shared" si="0"/>
+        <v>2.8356658504593448</v>
       </c>
       <c r="G15">
         <v>0.52138261081502402</v>
       </c>
       <c r="H15">
-        <v>28.5792634483009</v>
+        <f t="shared" ref="H15" si="14">100*(G15-G$2)/G$2</f>
+        <v>3.2080184026842988</v>
       </c>
       <c r="I15">
-        <v>2.9106502559085001</v>
+        <f t="shared" si="2"/>
+        <v>0.46865683829263816</v>
       </c>
       <c r="J15">
         <v>0.84685936766477898</v>
@@ -10992,22 +11167,26 @@
         <v>5.6382572848615498</v>
       </c>
       <c r="D16">
-        <v>17.3728711500404</v>
+        <f t="shared" si="0"/>
+        <v>4.073413175736218</v>
       </c>
       <c r="E16">
         <v>1.26406672926263</v>
       </c>
       <c r="F16">
-        <v>21.891315429941098</v>
+        <f t="shared" si="0"/>
+        <v>4.0706852143436585</v>
       </c>
       <c r="G16">
         <v>0.52557117328980196</v>
       </c>
       <c r="H16">
-        <v>25.521841091825902</v>
+        <f t="shared" ref="H16" si="15">100*(G16-G$2)/G$2</f>
+        <v>4.0371470003985861</v>
       </c>
       <c r="I16">
-        <v>6.3225799064404198</v>
+        <f t="shared" si="2"/>
+        <v>2.3727693973872075</v>
       </c>
       <c r="J16">
         <v>0.86290930411762501</v>
@@ -11024,22 +11203,26 @@
         <v>5.4997560593119497</v>
       </c>
       <c r="D17">
-        <v>6.9142507501659596</v>
+        <f t="shared" si="0"/>
+        <v>1.5168971205588402</v>
       </c>
       <c r="E17">
         <v>1.2403987076644101</v>
       </c>
       <c r="F17">
-        <v>12.1687368263228</v>
+        <f t="shared" si="0"/>
+        <v>2.1220956593986737</v>
       </c>
       <c r="G17">
         <v>0.51878134271989196</v>
       </c>
       <c r="H17">
-        <v>18.177778055381498</v>
+        <f t="shared" ref="H17" si="16">100*(G17-G$2)/G$2</f>
+        <v>2.693095733872942</v>
       </c>
       <c r="I17">
-        <v>-3.1562896930530902</v>
+        <f t="shared" si="2"/>
+        <v>-1.0959771479748042</v>
       </c>
       <c r="J17">
         <v>0.83367092671279197</v>
@@ -11056,22 +11239,26 @@
         <v>5.54833513221618</v>
       </c>
       <c r="D18">
-        <v>10.9377981211906</v>
+        <f t="shared" si="0"/>
+        <v>2.4135908453433994</v>
       </c>
       <c r="E18">
         <v>1.2520633936749701</v>
       </c>
       <c r="F18">
-        <v>17.572339232378901</v>
+        <f t="shared" si="0"/>
+        <v>3.0824499174664326</v>
       </c>
       <c r="G18">
         <v>0.52294039663778702</v>
       </c>
       <c r="H18">
-        <v>23.486863841748999</v>
+        <f t="shared" ref="H18" si="17">100*(G18-G$2)/G$2</f>
+        <v>3.5163830940418412</v>
       </c>
       <c r="I18">
-        <v>-1.91250657480905</v>
+        <f t="shared" si="2"/>
+        <v>-0.67455579376899111</v>
       </c>
       <c r="J18">
         <v>0.83722312530660403</v>
@@ -11088,22 +11275,26 @@
         <v>5.4635976264752202</v>
       </c>
       <c r="D19">
-        <v>4.3055182785194903</v>
+        <f t="shared" si="0"/>
+        <v>0.84946898979441365</v>
       </c>
       <c r="E19">
         <v>1.24990611993794</v>
       </c>
       <c r="F19">
-        <v>18.844388223606401</v>
+        <f t="shared" si="0"/>
+        <v>2.9048414488544982</v>
       </c>
       <c r="G19">
         <v>0.52663439663696598</v>
       </c>
       <c r="H19">
-        <v>32.607896734475098</v>
+        <f t="shared" ref="H19" si="18">100*(G19-G$2)/G$2</f>
+        <v>4.2476127361252409</v>
       </c>
       <c r="I19">
-        <v>-14.256171407604199</v>
+        <f t="shared" si="2"/>
+        <v>-4.6305696962614666</v>
       </c>
       <c r="J19">
         <v>0.803877527412028</v>
@@ -11120,22 +11311,26 @@
         <v>5.5358720502600303</v>
       </c>
       <c r="D20">
-        <v>10.094129555691</v>
+        <f t="shared" si="0"/>
+        <v>2.1835418404233824</v>
       </c>
       <c r="E20">
         <v>1.2527627412573199</v>
       </c>
       <c r="F20">
-        <v>18.347595088783098</v>
+        <f t="shared" si="0"/>
+        <v>3.1400272434202559</v>
       </c>
       <c r="G20">
         <v>0.52415207638914296</v>
       </c>
       <c r="H20">
-        <v>25.7790287192941</v>
+        <f t="shared" ref="H20" si="19">100*(G20-G$2)/G$2</f>
+        <v>3.7562358691096911</v>
       </c>
       <c r="I20">
-        <v>-3.7834628368867498</v>
+        <f t="shared" si="2"/>
+        <v>-1.319407624914968</v>
       </c>
       <c r="J20">
         <v>0.83178761107612398</v>
@@ -11152,22 +11347,26 @@
         <v>5.5232699771311804</v>
       </c>
       <c r="D21">
-        <v>9.1295821492606297</v>
+        <f t="shared" si="0"/>
+        <v>1.950927275789899</v>
       </c>
       <c r="E21">
         <v>1.2516020094135401</v>
       </c>
       <c r="F21">
-        <v>17.985190607705601</v>
+        <f t="shared" si="0"/>
+        <v>3.0444641251640361</v>
       </c>
       <c r="G21">
         <v>0.52434373084310903</v>
       </c>
       <c r="H21">
-        <v>26.336894077588902</v>
+        <f t="shared" ref="H21" si="20">100*(G21-G$2)/G$2</f>
+        <v>3.7941739897941655</v>
       </c>
       <c r="I21">
-        <v>-5.5231217389472302</v>
+        <f t="shared" si="2"/>
+        <v>-1.897612583824104</v>
       </c>
       <c r="J21">
         <v>0.82691386934122102</v>
@@ -11184,22 +11383,26 @@
         <v>5.6119825340455902</v>
       </c>
       <c r="D22">
-        <v>15.5568590322536</v>
+        <f t="shared" si="0"/>
+        <v>3.5884223603825314</v>
       </c>
       <c r="E22">
         <v>1.2719189458234801</v>
       </c>
       <c r="F22">
-        <v>25.6581977557504</v>
+        <f t="shared" si="0"/>
+        <v>4.7171586472895424</v>
       </c>
       <c r="G22">
         <v>0.53623613968750194</v>
       </c>
       <c r="H22">
-        <v>39.269411978856098</v>
+        <f t="shared" ref="H22" si="21">100*(G22-G$2)/G$2</f>
+        <v>6.1482838611335504</v>
       </c>
       <c r="I22">
-        <v>2.8341151029912499</v>
+        <f t="shared" si="2"/>
+        <v>1.0363250084620061</v>
       </c>
       <c r="J22">
         <v>0.851644293857301</v>
@@ -11216,22 +11419,26 @@
         <v>5.8166522657457698</v>
       </c>
       <c r="D23">
-        <v>30.603730057832198</v>
+        <f t="shared" si="0"/>
+        <v>7.3663055742243611</v>
       </c>
       <c r="E23">
         <v>1.3364385232365401</v>
       </c>
       <c r="F23">
-        <v>52.730135299082299</v>
+        <f t="shared" si="0"/>
+        <v>10.029059099755278</v>
       </c>
       <c r="G23">
         <v>0.56914999220891305</v>
       </c>
       <c r="H23">
-        <v>80.412834541766998</v>
+        <f t="shared" ref="H23" si="22">100*(G23-G$2)/G$2</f>
+        <v>12.663601837356222</v>
       </c>
       <c r="I23">
-        <v>7.8453238562851402</v>
+        <f t="shared" si="2"/>
+        <v>2.923407082508354</v>
       </c>
       <c r="J23">
         <v>0.86755067881605097</v>
@@ -11248,22 +11455,26 @@
         <v>5.5985806170975803</v>
       </c>
       <c r="D24">
-        <v>14.5016716897262</v>
+        <f t="shared" si="0"/>
+        <v>3.341043929529071</v>
       </c>
       <c r="E24">
         <v>1.2617380288169799</v>
       </c>
       <c r="F24">
-        <v>21.1134106483448</v>
+        <f t="shared" si="0"/>
+        <v>3.8789631751289115</v>
       </c>
       <c r="G24">
         <v>0.52686850022717402</v>
       </c>
       <c r="H24">
-        <v>27.382435589819298</v>
+        <f t="shared" ref="H24" si="23">100*(G24-G$2)/G$2</f>
+        <v>4.293953690244436</v>
       </c>
       <c r="I24">
-        <v>2.51401455023696</v>
+        <f t="shared" si="2"/>
+        <v>0.91897387304034173</v>
       </c>
       <c r="J24">
         <v>0.850655130555378</v>
@@ -11280,22 +11491,26 @@
         <v>5.59858089366009</v>
       </c>
       <c r="D25">
-        <v>8.9909705744803396</v>
+        <f t="shared" si="0"/>
+        <v>3.3410490344405526</v>
       </c>
       <c r="E25">
         <v>1.26706396066733</v>
       </c>
       <c r="F25">
-        <v>15.740247717615199</v>
+        <f t="shared" si="0"/>
+        <v>4.3174474451754374</v>
       </c>
       <c r="G25">
         <v>0.52914280295609695</v>
       </c>
       <c r="H25">
-        <v>21.9644485184402</v>
+        <f t="shared" ref="H25" si="24">100*(G25-G$2)/G$2</f>
+        <v>4.7441533574965318</v>
       </c>
       <c r="I25">
-        <v>-5.8747233323781796</v>
+        <f t="shared" si="2"/>
+        <v>-3.8617004313604051</v>
       </c>
       <c r="J25">
         <v>0.81035839577417801</v>
@@ -11312,22 +11527,26 @@
         <v>5.6764675158573299</v>
       </c>
       <c r="D26">
-        <v>7.5077860222692498</v>
+        <f t="shared" si="0"/>
+        <v>4.778714292207316</v>
       </c>
       <c r="E26">
         <v>1.2753904629780699</v>
       </c>
       <c r="F26">
-        <v>11.388571489914501</v>
+        <f t="shared" si="0"/>
+        <v>5.0029688506972843</v>
       </c>
       <c r="G26">
         <v>0.53294102312719405</v>
       </c>
       <c r="H26">
-        <v>17.1908399626004</v>
+        <f t="shared" ref="H26" si="25">100*(G26-G$2)/G$2</f>
+        <v>5.4960134486937662</v>
       </c>
       <c r="I26">
-        <v>18.9014044107759</v>
+        <f t="shared" si="2"/>
+        <v>23.306697574041493</v>
       </c>
       <c r="J26">
         <v>1.03936327231345</v>
@@ -11344,22 +11563,26 @@
         <v>5.3010462151932503</v>
       </c>
       <c r="D27">
-        <v>-38.3720249610137</v>
+        <f t="shared" si="0"/>
+        <v>-2.1509758877512724</v>
       </c>
       <c r="E27">
         <v>1.1731321959108101</v>
       </c>
       <c r="F27">
-        <v>-85.069436552493201</v>
+        <f t="shared" si="0"/>
+        <v>-3.4159600524698353</v>
       </c>
       <c r="G27">
         <v>0.48426792383517298</v>
       </c>
       <c r="H27">
-        <v>-127.962275149492</v>
+        <f t="shared" ref="H27" si="26">100*(G27-G$2)/G$2</f>
+        <v>-4.1388574181998177</v>
       </c>
       <c r="I27">
-        <v>-16.938204157826199</v>
+        <f t="shared" si="2"/>
+        <v>-1.4445409002888128</v>
       </c>
       <c r="J27">
         <v>0.83073285141483499</v>
@@ -11376,22 +11599,26 @@
         <v>5.5504529880081197</v>
       </c>
       <c r="D28">
-        <v>14.3309846710661</v>
+        <f t="shared" si="0"/>
+        <v>2.4526831516616943</v>
       </c>
       <c r="E28">
         <v>1.28812765278595</v>
       </c>
       <c r="F28">
-        <v>58.438907219487298</v>
+        <f t="shared" si="0"/>
+        <v>6.0516224069731308</v>
       </c>
       <c r="G28">
         <v>0.54364839445570401</v>
       </c>
       <c r="H28">
-        <v>127.562664353183</v>
+        <f t="shared" ref="H28" si="27">100*(G28-G$2)/G$2</f>
+        <v>7.6155443923701611</v>
       </c>
       <c r="I28">
-        <v>-14.693518666643</v>
+        <f t="shared" si="2"/>
+        <v>-4.7728156685049763</v>
       </c>
       <c r="J28">
         <v>0.80267852328578704</v>
@@ -11432,19 +11659,19 @@
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="str">
-        <f t="shared" ref="A32:B32" si="0">A2</f>
+        <f t="shared" ref="A32:B32" si="28">A2</f>
         <v>100 Mt Baseline</v>
       </c>
       <c r="B32" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="28"/>
         <v>100 Mt</v>
       </c>
       <c r="C32">
-        <f t="shared" ref="C32:C58" si="1">D2</f>
+        <f t="shared" ref="C32:C58" si="29">D2</f>
         <v>0</v>
       </c>
       <c r="D32">
-        <f t="shared" ref="D32:D56" si="2">I2</f>
+        <f t="shared" ref="D32:D56" si="30">I2</f>
         <v>0</v>
       </c>
       <c r="I32">
@@ -11454,530 +11681,530 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="str">
-        <f t="shared" ref="A33:B33" si="3">A3</f>
+        <f t="shared" ref="A33:B33" si="31">A3</f>
         <v>45Q-2040</v>
       </c>
       <c r="B33" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="31"/>
         <v>500 Mt</v>
       </c>
       <c r="C33">
-        <f t="shared" si="1"/>
-        <v>7.9722193986204699</v>
+        <f t="shared" si="29"/>
+        <v>0.64785695536394483</v>
       </c>
       <c r="D33">
-        <f t="shared" si="2"/>
-        <v>2.1065459229826602</v>
+        <f t="shared" si="30"/>
+        <v>0.21249703186680166</v>
       </c>
       <c r="F33">
         <f>C33</f>
-        <v>7.9722193986204699</v>
+        <v>0.64785695536394483</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="str">
-        <f t="shared" ref="A34:B34" si="4">A4</f>
+        <f t="shared" ref="A34:B34" si="32">A4</f>
         <v>45Q-2050</v>
       </c>
       <c r="B34" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="32"/>
         <v>500 Mt</v>
       </c>
       <c r="C34">
-        <f t="shared" si="1"/>
-        <v>4.18215697221197E-2</v>
+        <f t="shared" si="29"/>
+        <v>2.2459408657409443E-3</v>
       </c>
       <c r="D34">
-        <f t="shared" si="2"/>
-        <v>-32.193007747667103</v>
+        <f t="shared" si="30"/>
+        <v>-1.3655573070193403</v>
       </c>
       <c r="F34">
         <f>C34</f>
-        <v>4.18215697221197E-2</v>
+        <v>2.2459408657409443E-3</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="str">
-        <f t="shared" ref="A35:B35" si="5">A5</f>
+        <f t="shared" ref="A35:B35" si="33">A5</f>
         <v>Innovation-DACHubs</v>
       </c>
       <c r="B35" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="33"/>
         <v>500 Mt</v>
       </c>
       <c r="C35">
-        <f t="shared" si="1"/>
-        <v>3.27434679522118</v>
+        <f t="shared" si="29"/>
+        <v>0.27657518865875208</v>
       </c>
       <c r="D35">
-        <f t="shared" si="2"/>
-        <v>-4.7661224787360901</v>
+        <f t="shared" si="30"/>
+        <v>-0.46376197004718345</v>
       </c>
       <c r="E35">
         <f>C35</f>
-        <v>3.27434679522118</v>
+        <v>0.27657518865875208</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="str">
-        <f t="shared" ref="A36:B36" si="6">A6</f>
+        <f t="shared" ref="A36:B36" si="34">A6</f>
         <v>Innovation-maintain</v>
       </c>
       <c r="B36" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="34"/>
         <v>500 Mt</v>
       </c>
       <c r="C36">
-        <f t="shared" si="1"/>
-        <v>11.080702210154501</v>
+        <f t="shared" si="29"/>
+        <v>0.9215502090713279</v>
       </c>
       <c r="D36">
-        <f t="shared" si="2"/>
-        <v>-1.6578001841819501</v>
+        <f t="shared" si="30"/>
+        <v>-0.15840906711694819</v>
       </c>
       <c r="E36">
-        <f t="shared" ref="E36:E39" si="7">C36</f>
-        <v>11.080702210154501</v>
+        <f t="shared" ref="E36:E39" si="35">C36</f>
+        <v>0.9215502090713279</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="str">
-        <f t="shared" ref="A37:B37" si="8">A7</f>
+        <f t="shared" ref="A37:B37" si="36">A7</f>
         <v>Innovation-rhodium18b</v>
       </c>
       <c r="B37" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="36"/>
         <v>500 Mt</v>
       </c>
       <c r="C37">
-        <f t="shared" si="1"/>
-        <v>13.3924163736789</v>
+        <f t="shared" si="29"/>
+        <v>0.94967366043744428</v>
       </c>
       <c r="D37">
-        <f t="shared" si="2"/>
-        <v>-17.610796138934401</v>
+        <f t="shared" si="30"/>
+        <v>-1.4997785764247658</v>
       </c>
       <c r="E37">
-        <f t="shared" si="7"/>
-        <v>13.3924163736789</v>
+        <f t="shared" si="35"/>
+        <v>0.94967366043744428</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="str">
-        <f t="shared" ref="A38:B38" si="9">A8</f>
+        <f t="shared" ref="A38:B38" si="37">A8</f>
         <v>Innovation-rhodium6b</v>
       </c>
       <c r="B38" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="37"/>
         <v>500 Mt</v>
       </c>
       <c r="C38">
-        <f t="shared" si="1"/>
-        <v>12.090518117610101</v>
+        <f t="shared" si="29"/>
+        <v>0.97652041402801693</v>
       </c>
       <c r="D38">
-        <f t="shared" si="2"/>
-        <v>-4.2330036189303399</v>
+        <f t="shared" si="30"/>
+        <v>-0.39769251330281402</v>
       </c>
       <c r="E38">
-        <f t="shared" si="7"/>
-        <v>12.090518117610101</v>
+        <f t="shared" si="35"/>
+        <v>0.97652041402801693</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="str">
-        <f t="shared" ref="A39:B39" si="10">A9</f>
+        <f t="shared" ref="A39:B39" si="38">A9</f>
         <v>Innovation-triple</v>
       </c>
       <c r="B39" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="38"/>
         <v>500 Mt</v>
       </c>
       <c r="C39">
-        <f t="shared" si="1"/>
-        <v>11.804833462263</v>
+        <f t="shared" si="29"/>
+        <v>0.93865673606761379</v>
       </c>
       <c r="D39">
-        <f t="shared" si="2"/>
-        <v>-5.6982743163725003</v>
+        <f t="shared" si="30"/>
+        <v>-0.52357713726908883</v>
       </c>
       <c r="E39">
-        <f t="shared" si="7"/>
-        <v>11.804833462263</v>
+        <f t="shared" si="35"/>
+        <v>0.93865673606761379</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="str">
-        <f t="shared" ref="A40:B40" si="11">A10</f>
+        <f t="shared" ref="A40:B40" si="39">A10</f>
         <v>Low Baseline</v>
       </c>
       <c r="B40" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="39"/>
         <v>500 Mt</v>
       </c>
       <c r="C40">
-        <f t="shared" si="1"/>
-        <v>17.279164053851499</v>
+        <f t="shared" si="29"/>
+        <v>1.5349199946093965</v>
       </c>
       <c r="D40">
-        <f t="shared" si="2"/>
-        <v>10.550045036612699</v>
+        <f t="shared" si="30"/>
+        <v>1.0818447048699995</v>
       </c>
       <c r="I40">
         <f>C40</f>
-        <v>17.279164053851499</v>
+        <v>1.5349199946093965</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="str">
-        <f t="shared" ref="A41:B41" si="12">A11</f>
+        <f t="shared" ref="A41:B41" si="40">A11</f>
         <v>Procure3B</v>
       </c>
       <c r="B41" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="40"/>
         <v>500 Mt</v>
       </c>
       <c r="C41">
-        <f t="shared" si="1"/>
-        <v>16.858636173362701</v>
+        <f t="shared" si="29"/>
+        <v>1.4931934230901602</v>
       </c>
       <c r="D41">
-        <f t="shared" si="2"/>
-        <v>3.6313721464693201</v>
+        <f t="shared" si="30"/>
+        <v>0.36638009527595833</v>
       </c>
       <c r="G41">
         <f>C41</f>
-        <v>16.858636173362701</v>
+        <v>1.4931934230901602</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="str">
-        <f t="shared" ref="A42:B42" si="13">A12</f>
+        <f t="shared" ref="A42:B42" si="41">A12</f>
         <v>ProcureRhodium</v>
       </c>
       <c r="B42" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="41"/>
         <v>500 Mt</v>
       </c>
       <c r="C42">
-        <f t="shared" si="1"/>
-        <v>58.794583510587898</v>
+        <f t="shared" si="29"/>
+        <v>5.6634142557350327</v>
       </c>
       <c r="D42">
-        <f t="shared" si="2"/>
-        <v>11.060630810043</v>
+        <f t="shared" si="30"/>
+        <v>1.1959723569841303</v>
       </c>
       <c r="G42">
         <f>C42</f>
-        <v>58.794583510587898</v>
+        <v>5.6634142557350327</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="str">
-        <f t="shared" ref="A43:B43" si="14">A13</f>
+        <f t="shared" ref="A43:B43" si="42">A13</f>
         <v>ProcureScaling</v>
       </c>
       <c r="B43" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="42"/>
         <v>500 Mt</v>
       </c>
       <c r="C43">
-        <f t="shared" si="1"/>
-        <v>13.3113794026041</v>
+        <f t="shared" si="29"/>
+        <v>1.176004777856402</v>
       </c>
       <c r="D43">
-        <f t="shared" si="2"/>
-        <v>3.6008171018680599</v>
+        <f t="shared" si="30"/>
+        <v>0.36328086889841033</v>
       </c>
       <c r="G43">
         <f>C43</f>
-        <v>13.3113794026041</v>
+        <v>1.176004777856402</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="str">
-        <f t="shared" ref="A44:B44" si="15">A14</f>
+        <f t="shared" ref="A44:B44" si="43">A14</f>
         <v>45Q-2040</v>
       </c>
       <c r="B44" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="43"/>
         <v>1.5 Gt</v>
       </c>
       <c r="C44">
-        <f t="shared" si="1"/>
-        <v>10.5657233468163</v>
+        <f t="shared" si="29"/>
+        <v>2.2923311819484971</v>
       </c>
       <c r="D44">
-        <f t="shared" si="2"/>
-        <v>2.9193308209991198</v>
+        <f t="shared" si="30"/>
+        <v>1.0676371229122197</v>
       </c>
       <c r="F44">
         <f>C44</f>
-        <v>10.5657233468163</v>
+        <v>2.2923311819484971</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="str">
-        <f t="shared" ref="A45:B45" si="16">A15</f>
+        <f t="shared" ref="A45:B45" si="44">A15</f>
         <v>45Q-2050</v>
       </c>
       <c r="B45" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="44"/>
         <v>1.5 Gt</v>
       </c>
       <c r="C45">
-        <f t="shared" si="1"/>
-        <v>18.574625943324801</v>
+        <f t="shared" si="29"/>
+        <v>2.3877980534629502</v>
       </c>
       <c r="D45">
-        <f t="shared" si="2"/>
-        <v>2.9106502559085001</v>
+        <f t="shared" si="30"/>
+        <v>0.46865683829263816</v>
       </c>
       <c r="F45">
         <f>C45</f>
-        <v>18.574625943324801</v>
+        <v>2.3877980534629502</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="str">
-        <f t="shared" ref="A46:B46" si="17">A16</f>
+        <f t="shared" ref="A46:B46" si="45">A16</f>
         <v>High Baseline</v>
       </c>
       <c r="B46" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="45"/>
         <v>1.5 Gt</v>
       </c>
       <c r="C46">
-        <f t="shared" si="1"/>
-        <v>17.3728711500404</v>
+        <f t="shared" si="29"/>
+        <v>4.073413175736218</v>
       </c>
       <c r="D46">
-        <f t="shared" si="2"/>
-        <v>6.3225799064404198</v>
+        <f t="shared" si="30"/>
+        <v>2.3727693973872075</v>
       </c>
       <c r="I46">
         <f>C46</f>
-        <v>17.3728711500404</v>
+        <v>4.073413175736218</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="str">
-        <f t="shared" ref="A47:B47" si="18">A17</f>
+        <f t="shared" ref="A47:B47" si="46">A17</f>
         <v>Innovation-DACHubs</v>
       </c>
       <c r="B47" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="46"/>
         <v>1.5 Gt</v>
       </c>
       <c r="C47">
-        <f t="shared" si="1"/>
-        <v>6.9142507501659596</v>
+        <f t="shared" si="29"/>
+        <v>1.5168971205588402</v>
       </c>
       <c r="D47">
-        <f t="shared" si="2"/>
-        <v>-3.1562896930530902</v>
+        <f t="shared" si="30"/>
+        <v>-1.0959771479748042</v>
       </c>
       <c r="E47">
         <f>C47</f>
-        <v>6.9142507501659596</v>
+        <v>1.5168971205588402</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="str">
-        <f t="shared" ref="A48:B48" si="19">A18</f>
+        <f t="shared" ref="A48:B48" si="47">A18</f>
         <v>Innovation-maintain</v>
       </c>
       <c r="B48" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="47"/>
         <v>1.5 Gt</v>
       </c>
       <c r="C48">
-        <f t="shared" si="1"/>
-        <v>10.9377981211906</v>
+        <f t="shared" si="29"/>
+        <v>2.4135908453433994</v>
       </c>
       <c r="D48">
-        <f t="shared" si="2"/>
-        <v>-1.91250657480905</v>
+        <f t="shared" si="30"/>
+        <v>-0.67455579376899111</v>
       </c>
       <c r="E48">
-        <f t="shared" ref="E48:E51" si="20">C48</f>
-        <v>10.9377981211906</v>
+        <f t="shared" ref="E48:E51" si="48">C48</f>
+        <v>2.4135908453433994</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="str">
-        <f t="shared" ref="A49:B49" si="21">A19</f>
+        <f t="shared" ref="A49:B49" si="49">A19</f>
         <v>Innovation-rhodium18b</v>
       </c>
       <c r="B49" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="49"/>
         <v>1.5 Gt</v>
       </c>
       <c r="C49">
-        <f t="shared" si="1"/>
-        <v>4.3055182785194903</v>
+        <f t="shared" si="29"/>
+        <v>0.84946898979441365</v>
       </c>
       <c r="D49">
-        <f t="shared" si="2"/>
-        <v>-14.256171407604199</v>
+        <f t="shared" si="30"/>
+        <v>-4.6305696962614666</v>
       </c>
       <c r="E49">
-        <f t="shared" si="20"/>
-        <v>4.3055182785194903</v>
+        <f t="shared" si="48"/>
+        <v>0.84946898979441365</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="str">
-        <f t="shared" ref="A50:B50" si="22">A20</f>
+        <f t="shared" ref="A50:B50" si="50">A20</f>
         <v>Innovation-rhodium6b</v>
       </c>
       <c r="B50" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="50"/>
         <v>1.5 Gt</v>
       </c>
       <c r="C50">
-        <f t="shared" si="1"/>
-        <v>10.094129555691</v>
+        <f t="shared" si="29"/>
+        <v>2.1835418404233824</v>
       </c>
       <c r="D50">
-        <f t="shared" si="2"/>
-        <v>-3.7834628368867498</v>
+        <f t="shared" si="30"/>
+        <v>-1.319407624914968</v>
       </c>
       <c r="E50">
-        <f t="shared" si="20"/>
-        <v>10.094129555691</v>
+        <f t="shared" si="48"/>
+        <v>2.1835418404233824</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="str">
-        <f t="shared" ref="A51:B51" si="23">A21</f>
+        <f t="shared" ref="A51:B51" si="51">A21</f>
         <v>Innovation-triple</v>
       </c>
       <c r="B51" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="51"/>
         <v>1.5 Gt</v>
       </c>
       <c r="C51">
-        <f t="shared" si="1"/>
-        <v>9.1295821492606297</v>
+        <f t="shared" si="29"/>
+        <v>1.950927275789899</v>
       </c>
       <c r="D51">
-        <f t="shared" si="2"/>
-        <v>-5.5231217389472302</v>
+        <f t="shared" si="30"/>
+        <v>-1.897612583824104</v>
       </c>
       <c r="E51">
-        <f t="shared" si="20"/>
-        <v>9.1295821492606297</v>
+        <f t="shared" si="48"/>
+        <v>1.950927275789899</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" t="str">
-        <f t="shared" ref="A52:B52" si="24">A22</f>
+        <f t="shared" ref="A52:B52" si="52">A22</f>
         <v>Procure3B</v>
       </c>
       <c r="B52" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="52"/>
         <v>1.5 Gt</v>
       </c>
       <c r="C52">
-        <f t="shared" si="1"/>
-        <v>15.5568590322536</v>
+        <f t="shared" si="29"/>
+        <v>3.5884223603825314</v>
       </c>
       <c r="D52">
-        <f t="shared" si="2"/>
-        <v>2.8341151029912499</v>
+        <f t="shared" si="30"/>
+        <v>1.0363250084620061</v>
       </c>
       <c r="G52">
         <f>C52</f>
-        <v>15.5568590322536</v>
+        <v>3.5884223603825314</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" t="str">
-        <f t="shared" ref="A53:B53" si="25">A23</f>
+        <f t="shared" ref="A53:B53" si="53">A23</f>
         <v>ProcureRhodium</v>
       </c>
       <c r="B53" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="53"/>
         <v>1.5 Gt</v>
       </c>
       <c r="C53">
-        <f t="shared" si="1"/>
-        <v>30.603730057832198</v>
+        <f t="shared" si="29"/>
+        <v>7.3663055742243611</v>
       </c>
       <c r="D53">
-        <f t="shared" si="2"/>
-        <v>7.8453238562851402</v>
+        <f t="shared" si="30"/>
+        <v>2.923407082508354</v>
       </c>
       <c r="G53">
         <f>C53</f>
-        <v>30.603730057832198</v>
+        <v>7.3663055742243611</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" t="str">
-        <f t="shared" ref="A54:B54" si="26">A24</f>
+        <f t="shared" ref="A54:B54" si="54">A24</f>
         <v>ProcureScaling</v>
       </c>
       <c r="B54" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="54"/>
         <v>1.5 Gt</v>
       </c>
       <c r="C54">
-        <f t="shared" si="1"/>
-        <v>14.5016716897262</v>
+        <f t="shared" si="29"/>
+        <v>3.341043929529071</v>
       </c>
       <c r="D54">
-        <f t="shared" si="2"/>
-        <v>2.51401455023696</v>
+        <f t="shared" si="30"/>
+        <v>0.91897387304034173</v>
       </c>
       <c r="G54">
         <f>C54</f>
-        <v>14.5016716897262</v>
+        <v>3.341043929529071</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" t="str">
-        <f t="shared" ref="A55:B55" si="27">A25</f>
+        <f t="shared" ref="A55:B55" si="55">A25</f>
         <v>2.4 Gt Baseline</v>
       </c>
       <c r="B55" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="55"/>
         <v>2.4 Gt</v>
       </c>
       <c r="C55">
-        <f t="shared" si="1"/>
-        <v>8.9909705744803396</v>
+        <f t="shared" si="29"/>
+        <v>3.3410490344405526</v>
       </c>
       <c r="D55">
-        <f t="shared" si="2"/>
-        <v>-5.8747233323781796</v>
+        <f t="shared" si="30"/>
+        <v>-3.8617004313604051</v>
       </c>
       <c r="I55">
         <f>C55</f>
-        <v>8.9909705744803396</v>
+        <v>3.3410490344405526</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" t="str">
-        <f t="shared" ref="A56:B56" si="28">A26</f>
+        <f t="shared" ref="A56:B56" si="56">A26</f>
         <v>4.1 Gt Baseline</v>
       </c>
       <c r="B56" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="56"/>
         <v>4.1 Gt</v>
       </c>
       <c r="C56">
-        <f t="shared" si="1"/>
-        <v>7.5077860222692498</v>
+        <f t="shared" si="29"/>
+        <v>4.778714292207316</v>
       </c>
       <c r="D56">
-        <f t="shared" si="2"/>
-        <v>18.9014044107759</v>
+        <f t="shared" si="30"/>
+        <v>23.306697574041493</v>
       </c>
       <c r="I56">
         <f>C56</f>
-        <v>7.5077860222692498</v>
+        <v>4.778714292207316</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -11991,37 +12218,37 @@
       </c>
       <c r="C57">
         <f>D27</f>
-        <v>-38.3720249610137</v>
+        <v>-2.1509758877512724</v>
       </c>
       <c r="D57">
         <f>I27</f>
-        <v>-16.938204157826199</v>
+        <v>-1.4445409002888128</v>
       </c>
       <c r="H57">
         <f>C57</f>
-        <v>-38.3720249610137</v>
+        <v>-2.1509758877512724</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" t="str">
-        <f t="shared" ref="A58:B58" si="29">A28</f>
+        <f t="shared" ref="A58:B58" si="57">A28</f>
         <v>CDRIA-Rhodium18b</v>
       </c>
       <c r="B58" t="str">
+        <f t="shared" si="57"/>
+        <v>1.5 Gt</v>
+      </c>
+      <c r="C58">
         <f t="shared" si="29"/>
-        <v>1.5 Gt</v>
-      </c>
-      <c r="C58">
-        <f t="shared" si="1"/>
-        <v>14.3309846710661</v>
+        <v>2.4526831516616943</v>
       </c>
       <c r="D58">
-        <f t="shared" ref="D58" si="30">I28</f>
-        <v>-14.693518666643</v>
+        <f t="shared" ref="D58" si="58">I28</f>
+        <v>-4.7728156685049763</v>
       </c>
       <c r="H58">
         <f>C58</f>
-        <v>14.3309846710661</v>
+        <v>2.4526831516616943</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
make more plots for comparing effectiveness of trajectory
</commit_message>
<xml_diff>
--- a/data/data_analysis/policy_effectiveness.xlsx
+++ b/data/data_analysis/policy_effectiveness.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\data\data_analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6E389DF-F9AA-40E8-9A37-58DCB08A81F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{122D0F23-43B5-41C3-97B3-3086EABE55FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{5B094011-67C9-461D-BBBF-A6D3FE50B4AB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{5B094011-67C9-461D-BBBF-A6D3FE50B4AB}"/>
   </bookViews>
   <sheets>
     <sheet name="Low" sheetId="1" r:id="rId1"/>
@@ -26,14 +26,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Net-Zero Mandate'!$A$1:$H$26</definedName>
     <definedName name="_xlchart.v1.0" hidden="1">'Net-Zero Mandate'!$A$2:$B$28</definedName>
     <definedName name="_xlchart.v1.1" hidden="1">'Net-Zero Mandate'!$D$1</definedName>
-    <definedName name="_xlchart.v1.10" hidden="1">'Net-Zero Mandate'!$D$1</definedName>
-    <definedName name="_xlchart.v1.11" hidden="1">'Net-Zero Mandate'!$D$2:$D$28</definedName>
-    <definedName name="_xlchart.v1.12" hidden="1">'Net-Zero Mandate'!$F$1</definedName>
-    <definedName name="_xlchart.v1.13" hidden="1">'Net-Zero Mandate'!$F$2:$F$28</definedName>
-    <definedName name="_xlchart.v1.14" hidden="1">'Net-Zero Mandate'!$H$1</definedName>
-    <definedName name="_xlchart.v1.15" hidden="1">'Net-Zero Mandate'!$H$2:$H$28</definedName>
-    <definedName name="_xlchart.v1.16" hidden="1">'Net-Zero Mandate'!$I$1</definedName>
-    <definedName name="_xlchart.v1.17" hidden="1">'Net-Zero Mandate'!$I$2:$I$28</definedName>
     <definedName name="_xlchart.v1.2" hidden="1">'Net-Zero Mandate'!$D$2:$D$28</definedName>
     <definedName name="_xlchart.v1.3" hidden="1">'Net-Zero Mandate'!$F$1</definedName>
     <definedName name="_xlchart.v1.4" hidden="1">'Net-Zero Mandate'!$F$2:$F$28</definedName>
@@ -41,7 +33,6 @@
     <definedName name="_xlchart.v1.6" hidden="1">'Net-Zero Mandate'!$H$2:$H$28</definedName>
     <definedName name="_xlchart.v1.7" hidden="1">'Net-Zero Mandate'!$I$1</definedName>
     <definedName name="_xlchart.v1.8" hidden="1">'Net-Zero Mandate'!$I$2:$I$28</definedName>
-    <definedName name="_xlchart.v1.9" hidden="1">'Net-Zero Mandate'!$A$2:$B$28</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -64,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="70">
   <si>
     <t>Scenario</t>
   </si>
@@ -337,7 +328,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -345,6 +336,8 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2916,6 +2909,2374 @@
           </c:txPr>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="688359152"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="688359152"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1400"/>
+                  <a:t>Change in NPV from efficient</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1400" baseline="0"/>
+                  <a:t> scenario</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1400"/>
+                  <a:t> (%)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="3.2156184287128318E-2"/>
+              <c:y val="0.2133207649709703"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="688358192"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.5898129642232609"/>
+          <c:y val="0.38244392172116509"/>
+          <c:w val="0.18739061607306434"/>
+          <c:h val="0.25525532296155895"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:solidFill>
+          <a:schemeClr val="bg1">
+            <a:alpha val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="8.7487789964051293E-2"/>
+          <c:y val="9.5648818834036059E-2"/>
+          <c:w val="0.86045319240557017"/>
+          <c:h val="0.82694066899082042"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Net-Zero Mandate'!$E$31</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Innovation</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FF0000"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Net-Zero Mandate'!$D$61:$D$87</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="27"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.21249703186680166</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-1.3655573070193403</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-0.46376197004718345</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-0.15840906711694819</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-1.4997785764247658</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-0.39769251330281402</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-0.52357713726908883</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.0818447048699995</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.36638009527595833</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.1959723569841303</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.36328086889841033</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.0676371229122197</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.46865683829263816</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2.3727693973872075</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>-1.0959771479748042</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>-0.67455579376899111</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>-4.6305696962614666</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>-1.319407624914968</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>-1.897612583824104</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1.0363250084620061</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2.923407082508354</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.91897387304034173</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>-3.8617004313604051</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>23.306697574041493</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>-1.4445409002888128</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>-4.7728156685049763</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Net-Zero Mandate'!$E$61:$E$87</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="27"/>
+                <c:pt idx="3" formatCode="0.00">
+                  <c:v>0.64724767761331869</c:v>
+                </c:pt>
+                <c:pt idx="4" formatCode="0.00">
+                  <c:v>1.3577275897072081</c:v>
+                </c:pt>
+                <c:pt idx="5" formatCode="0.00">
+                  <c:v>2.3153381298881297</c:v>
+                </c:pt>
+                <c:pt idx="6" formatCode="0.00">
+                  <c:v>1.6348546043849213</c:v>
+                </c:pt>
+                <c:pt idx="7" formatCode="0.00">
+                  <c:v>1.6529080927729902</c:v>
+                </c:pt>
+                <c:pt idx="15" formatCode="0.00">
+                  <c:v>2.1220956593986737</c:v>
+                </c:pt>
+                <c:pt idx="16" formatCode="0.00">
+                  <c:v>3.0824499174664326</c:v>
+                </c:pt>
+                <c:pt idx="17" formatCode="0.00">
+                  <c:v>2.9048414488544982</c:v>
+                </c:pt>
+                <c:pt idx="18" formatCode="0.00">
+                  <c:v>3.1400272434202559</c:v>
+                </c:pt>
+                <c:pt idx="19" formatCode="0.00">
+                  <c:v>3.0444641251640361</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-D746-4562-9FAE-205B641F3911}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Net-Zero Mandate'!$F$31</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Subsidy</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Net-Zero Mandate'!$D$61:$D$87</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="27"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.21249703186680166</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-1.3655573070193403</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-0.46376197004718345</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-0.15840906711694819</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-1.4997785764247658</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-0.39769251330281402</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-0.52357713726908883</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.0818447048699995</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.36638009527595833</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.1959723569841303</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.36328086889841033</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.0676371229122197</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.46865683829263816</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2.3727693973872075</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>-1.0959771479748042</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>-0.67455579376899111</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>-4.6305696962614666</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>-1.319407624914968</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>-1.897612583824104</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1.0363250084620061</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2.923407082508354</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.91897387304034173</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>-3.8617004313604051</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>23.306697574041493</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>-1.4445409002888128</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>-4.7728156685049763</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Net-Zero Mandate'!$F$61:$F$87</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="27"/>
+                <c:pt idx="1">
+                  <c:v>0.98599472057171911</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.44448412606722876</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2.5637816421080228</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2.8356658504593448</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-D746-4562-9FAE-205B641F3911}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Net-Zero Mandate'!$G$31</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Procurement</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Net-Zero Mandate'!$D$61:$D$87</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="27"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.21249703186680166</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-1.3655573070193403</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-0.46376197004718345</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-0.15840906711694819</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-1.4997785764247658</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-0.39769251330281402</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-0.52357713726908883</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.0818447048699995</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.36638009527595833</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.1959723569841303</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.36328086889841033</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.0676371229122197</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.46865683829263816</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2.3727693973872075</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>-1.0959771479748042</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>-0.67455579376899111</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>-4.6305696962614666</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>-1.319407624914968</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>-1.897612583824104</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1.0363250084620061</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2.923407082508354</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.91897387304034173</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>-3.8617004313604051</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>23.306697574041493</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>-1.4445409002888128</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>-4.7728156685049763</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Net-Zero Mandate'!$G$61:$G$87</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="27"/>
+                <c:pt idx="9" formatCode="0.00">
+                  <c:v>2.5994756304123183</c:v>
+                </c:pt>
+                <c:pt idx="10" formatCode="0.00">
+                  <c:v>8.3515011746760219</c:v>
+                </c:pt>
+                <c:pt idx="11" formatCode="0.00">
+                  <c:v>1.5468320344764317</c:v>
+                </c:pt>
+                <c:pt idx="20" formatCode="0.00">
+                  <c:v>4.7171586472895424</c:v>
+                </c:pt>
+                <c:pt idx="21" formatCode="0.00">
+                  <c:v>10.029059099755278</c:v>
+                </c:pt>
+                <c:pt idx="22" formatCode="0.00">
+                  <c:v>3.8789631751289115</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-D746-4562-9FAE-205B641F3911}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Net-Zero Mandate'!$H$31</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Optimal</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent4"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Net-Zero Mandate'!$D$61:$D$87</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="27"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.21249703186680166</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-1.3655573070193403</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-0.46376197004718345</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-0.15840906711694819</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-1.4997785764247658</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-0.39769251330281402</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-0.52357713726908883</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.0818447048699995</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.36638009527595833</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.1959723569841303</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.36328086889841033</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.0676371229122197</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.46865683829263816</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2.3727693973872075</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>-1.0959771479748042</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>-0.67455579376899111</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>-4.6305696962614666</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>-1.319407624914968</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>-1.897612583824104</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1.0363250084620061</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2.923407082508354</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.91897387304034173</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>-3.8617004313604051</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>23.306697574041493</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>-1.4445409002888128</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>-4.7728156685049763</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Net-Zero Mandate'!$H$61:$H$87</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="27"/>
+                <c:pt idx="25" formatCode="0.00">
+                  <c:v>-3.4159600524698353</c:v>
+                </c:pt>
+                <c:pt idx="26" formatCode="0.00">
+                  <c:v>6.0516224069731308</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-D746-4562-9FAE-205B641F3911}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Net-Zero Mandate'!$I$31</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Baseline</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent5"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Net-Zero Mandate'!$D$61:$D$87</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="27"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.21249703186680166</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-1.3655573070193403</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-0.46376197004718345</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-0.15840906711694819</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-1.4997785764247658</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-0.39769251330281402</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-0.52357713726908883</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.0818447048699995</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.36638009527595833</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.1959723569841303</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.36328086889841033</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.0676371229122197</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.46865683829263816</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2.3727693973872075</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>-1.0959771479748042</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>-0.67455579376899111</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>-4.6305696962614666</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>-1.319407624914968</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>-1.897612583824104</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1.0363250084620061</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2.923407082508354</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.91897387304034173</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>-3.8617004313604051</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>23.306697574041493</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>-1.4445409002888128</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>-4.7728156685049763</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Net-Zero Mandate'!$I$61:$I$87</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="27"/>
+                <c:pt idx="0" formatCode="0.00">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="8" formatCode="0.00">
+                  <c:v>1.5453796931733457</c:v>
+                </c:pt>
+                <c:pt idx="14" formatCode="0.00">
+                  <c:v>4.0706852143436585</c:v>
+                </c:pt>
+                <c:pt idx="23" formatCode="0.00">
+                  <c:v>4.3174474451754374</c:v>
+                </c:pt>
+                <c:pt idx="24" formatCode="0.00">
+                  <c:v>5.0029688506972843</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000004-D746-4562-9FAE-205B641F3911}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="688358192"/>
+        <c:axId val="688359152"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="688358192"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1400"/>
+                  <a:t>Change in 2050 cost effectiveness from</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1400" baseline="0"/>
+                  <a:t> efficient scenario (%)</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US" sz="1400"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="688359152"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="688359152"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1400"/>
+                  <a:t>Change in NPV from efficient</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1400" baseline="0"/>
+                  <a:t> scenario</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1400"/>
+                  <a:t> (%)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="3.2156184287128318E-2"/>
+              <c:y val="0.2133207649709703"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="688358192"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.5898129642232609"/>
+          <c:y val="0.38244392172116509"/>
+          <c:w val="0.18739061607306434"/>
+          <c:h val="0.25525532296155895"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:solidFill>
+          <a:schemeClr val="bg1">
+            <a:alpha val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="8.7487789964051293E-2"/>
+          <c:y val="9.5648818834036059E-2"/>
+          <c:w val="0.86045319240557017"/>
+          <c:h val="0.82694066899082042"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Net-Zero Mandate'!$E$31</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Innovation</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FF0000"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Net-Zero Mandate'!$D$90:$D$116</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="27"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.21249703186680166</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-1.3655573070193403</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-0.46376197004718345</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-0.15840906711694819</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-1.4997785764247658</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-0.39769251330281402</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-0.52357713726908883</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.0818447048699995</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.36638009527595833</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.1959723569841303</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.36328086889841033</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.0676371229122197</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.46865683829263816</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2.3727693973872075</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>-1.0959771479748042</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>-0.67455579376899111</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>-4.6305696962614666</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>-1.319407624914968</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>-1.897612583824104</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1.0363250084620061</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2.923407082508354</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.91897387304034173</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>-3.8617004313604051</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>23.306697574041493</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>-1.4445409002888128</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>-4.7728156685049763</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Net-Zero Mandate'!$E$90:$E$116</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="27"/>
+                <c:pt idx="3" formatCode="0.00">
+                  <c:v>1.0932573496051559</c:v>
+                </c:pt>
+                <c:pt idx="4" formatCode="0.00">
+                  <c:v>1.6946076320487724</c:v>
+                </c:pt>
+                <c:pt idx="5" formatCode="0.00">
+                  <c:v>3.2502144071938046</c:v>
+                </c:pt>
+                <c:pt idx="6" formatCode="0.00">
+                  <c:v>2.1049050122513044</c:v>
+                </c:pt>
+                <c:pt idx="7" formatCode="0.00">
+                  <c:v>2.2091624983315339</c:v>
+                </c:pt>
+                <c:pt idx="15" formatCode="0.00">
+                  <c:v>2.693095733872942</c:v>
+                </c:pt>
+                <c:pt idx="16" formatCode="0.00">
+                  <c:v>3.5163830940418412</c:v>
+                </c:pt>
+                <c:pt idx="17" formatCode="0.00">
+                  <c:v>4.2476127361252409</c:v>
+                </c:pt>
+                <c:pt idx="18" formatCode="0.00">
+                  <c:v>3.7562358691096911</c:v>
+                </c:pt>
+                <c:pt idx="19" formatCode="0.00">
+                  <c:v>3.7941739897941655</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-573D-4403-A039-27329D583A2E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Net-Zero Mandate'!$F$31</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Subsidy</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Net-Zero Mandate'!$D$90:$D$116</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="27"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.21249703186680166</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-1.3655573070193403</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-0.46376197004718345</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-0.15840906711694819</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-1.4997785764247658</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-0.39769251330281402</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-0.52357713726908883</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.0818447048699995</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.36638009527595833</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.1959723569841303</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.36328086889841033</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.0676371229122197</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.46865683829263816</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2.3727693973872075</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>-1.0959771479748042</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>-0.67455579376899111</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>-4.6305696962614666</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>-1.319407624914968</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>-1.897612583824104</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1.0363250084620061</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2.923407082508354</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.91897387304034173</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>-3.8617004313604051</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>23.306697574041493</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>-1.4445409002888128</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>-4.7728156685049763</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Net-Zero Mandate'!$F$90:$F$116</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="27"/>
+                <c:pt idx="1">
+                  <c:v>1.3438885594409384</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.84723170018844907</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2.9242921759498324</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>3.2080184026842988</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-573D-4403-A039-27329D583A2E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Net-Zero Mandate'!$G$31</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Procurement</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Net-Zero Mandate'!$D$90:$D$116</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="27"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.21249703186680166</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-1.3655573070193403</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-0.46376197004718345</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-0.15840906711694819</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-1.4997785764247658</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-0.39769251330281402</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-0.52357713726908883</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.0818447048699995</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.36638009527595833</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.1959723569841303</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.36328086889841033</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.0676371229122197</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.46865683829263816</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2.3727693973872075</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>-1.0959771479748042</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>-0.67455579376899111</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>-4.6305696962614666</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>-1.319407624914968</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>-1.897612583824104</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1.0363250084620061</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2.923407082508354</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.91897387304034173</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>-3.8617004313604051</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>23.306697574041493</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>-1.4445409002888128</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>-4.7728156685049763</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Net-Zero Mandate'!$G$90:$G$116</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="27"/>
+                <c:pt idx="9" formatCode="0.00">
+                  <c:v>4.0670809313292864</c:v>
+                </c:pt>
+                <c:pt idx="10" formatCode="0.00">
+                  <c:v>10.956263412283258</c:v>
+                </c:pt>
+                <c:pt idx="11" formatCode="0.00">
+                  <c:v>1.9108299722709272</c:v>
+                </c:pt>
+                <c:pt idx="20" formatCode="0.00">
+                  <c:v>6.1482838611335504</c:v>
+                </c:pt>
+                <c:pt idx="21" formatCode="0.00">
+                  <c:v>12.663601837356222</c:v>
+                </c:pt>
+                <c:pt idx="22" formatCode="0.00">
+                  <c:v>4.293953690244436</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-573D-4403-A039-27329D583A2E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Net-Zero Mandate'!$H$31</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Optimal</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent4"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Net-Zero Mandate'!$D$90:$D$116</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="27"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.21249703186680166</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-1.3655573070193403</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-0.46376197004718345</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-0.15840906711694819</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-1.4997785764247658</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-0.39769251330281402</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-0.52357713726908883</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.0818447048699995</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.36638009527595833</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.1959723569841303</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.36328086889841033</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.0676371229122197</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.46865683829263816</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2.3727693973872075</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>-1.0959771479748042</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>-0.67455579376899111</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>-4.6305696962614666</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>-1.319407624914968</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>-1.897612583824104</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1.0363250084620061</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2.923407082508354</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.91897387304034173</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>-3.8617004313604051</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>23.306697574041493</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>-1.4445409002888128</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>-4.7728156685049763</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Net-Zero Mandate'!$H$90:$H$116</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="27"/>
+                <c:pt idx="25" formatCode="0.00">
+                  <c:v>-4.1388574181998177</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>7.6155443923701611</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-573D-4403-A039-27329D583A2E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Net-Zero Mandate'!$I$31</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Baseline</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent5"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Net-Zero Mandate'!$D$90:$D$116</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="27"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.21249703186680166</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-1.3655573070193403</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-0.46376197004718345</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-0.15840906711694819</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-1.4997785764247658</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-0.39769251330281402</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-0.52357713726908883</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.0818447048699995</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.36638009527595833</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.1959723569841303</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.36328086889841033</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.0676371229122197</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.46865683829263816</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2.3727693973872075</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>-1.0959771479748042</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>-0.67455579376899111</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>-4.6305696962614666</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>-1.319407624914968</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>-1.897612583824104</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1.0363250084620061</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2.923407082508354</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.91897387304034173</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>-3.8617004313604051</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>23.306697574041493</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>-1.4445409002888128</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>-4.7728156685049763</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Net-Zero Mandate'!$I$90:$I$116</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="27"/>
+                <c:pt idx="0" formatCode="0.00">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="8" formatCode="0.00">
+                  <c:v>1.5827998282841693</c:v>
+                </c:pt>
+                <c:pt idx="14" formatCode="0.00">
+                  <c:v>4.0371470003985861</c:v>
+                </c:pt>
+                <c:pt idx="23" formatCode="0.00">
+                  <c:v>4.7441533574965318</c:v>
+                </c:pt>
+                <c:pt idx="24" formatCode="0.00">
+                  <c:v>5.4960134486937662</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000004-573D-4403-A039-27329D583A2E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="688358192"/>
+        <c:axId val="688359152"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="688358192"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1400"/>
+                  <a:t>Change in 2050 cost effectiveness from</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1400" baseline="0"/>
+                  <a:t> efficient scenario (%)</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US" sz="1400"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -3561,6 +5922,86 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors6.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -5109,6 +7550,1038 @@
 </file>
 
 <file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style6.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -6125,6 +9598,82 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>217714</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>81643</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>260577</xdr:colOff>
+      <xdr:row>86</xdr:row>
+      <xdr:rowOff>38781</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CD220C49-AEBE-4CDA-8478-06D535AEBA9E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>435429</xdr:colOff>
+      <xdr:row>88</xdr:row>
+      <xdr:rowOff>108857</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>478292</xdr:colOff>
+      <xdr:row>115</xdr:row>
+      <xdr:rowOff>65995</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{45FFBF60-479F-456B-919C-CC27930EACA4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -10611,13 +14160,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66EF8D6B-AAC7-4D47-8A22-E3B6AC50568B}">
-  <dimension ref="A1:J58"/>
+  <dimension ref="A1:J116"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.28515625" customWidth="1"/>
-    <col min="4" max="4" width="23.5703125" customWidth="1"/>
+    <col min="3" max="3" width="66.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="70.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -11625,9 +15174,8 @@
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A31" t="str">
-        <f>A1</f>
-        <v>Scenario</v>
+      <c r="A31" s="7">
+        <v>0.02</v>
       </c>
       <c r="B31" t="str">
         <f>B1</f>
@@ -12249,6 +15797,1263 @@
       <c r="H58">
         <f>C58</f>
         <v>2.4526831516616943</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A60" s="7">
+        <v>0.12</v>
+      </c>
+      <c r="B60" s="7" t="str">
+        <f t="shared" ref="B60:I61" si="59">B31</f>
+        <v>Baseline</v>
+      </c>
+      <c r="C60" s="7" t="str">
+        <f>F1</f>
+        <v>Cost Decrease necessary in NPV of CDR market | 12.0% discount rate</v>
+      </c>
+      <c r="D60" s="7" t="str">
+        <f t="shared" si="59"/>
+        <v>Cost Decrease necessary in size of the CDR market in 2050</v>
+      </c>
+      <c r="E60" s="7" t="str">
+        <f t="shared" si="59"/>
+        <v>Innovation</v>
+      </c>
+      <c r="F60" s="7" t="str">
+        <f t="shared" si="59"/>
+        <v>Subsidy</v>
+      </c>
+      <c r="G60" s="7" t="str">
+        <f t="shared" si="59"/>
+        <v>Procurement</v>
+      </c>
+      <c r="H60" s="7" t="str">
+        <f t="shared" si="59"/>
+        <v>Optimal</v>
+      </c>
+      <c r="I60" s="7" t="str">
+        <f t="shared" si="59"/>
+        <v>Baseline</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A61" s="7" t="str">
+        <f>A32</f>
+        <v>100 Mt Baseline</v>
+      </c>
+      <c r="B61" s="7" t="str">
+        <f t="shared" si="59"/>
+        <v>100 Mt</v>
+      </c>
+      <c r="C61" s="8">
+        <f t="shared" ref="C61:C86" si="60">F2</f>
+        <v>0</v>
+      </c>
+      <c r="D61">
+        <f t="shared" si="59"/>
+        <v>0</v>
+      </c>
+      <c r="I61" s="8">
+        <f>C61</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A62" s="7" t="str">
+        <f t="shared" ref="A62:I62" si="61">A33</f>
+        <v>45Q-2040</v>
+      </c>
+      <c r="B62" s="7" t="str">
+        <f t="shared" si="61"/>
+        <v>500 Mt</v>
+      </c>
+      <c r="C62" s="8">
+        <f t="shared" si="60"/>
+        <v>0.98599472057171911</v>
+      </c>
+      <c r="D62">
+        <f t="shared" si="61"/>
+        <v>0.21249703186680166</v>
+      </c>
+      <c r="F62" s="8">
+        <f>C62</f>
+        <v>0.98599472057171911</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A63" s="7" t="str">
+        <f t="shared" ref="A63:I63" si="62">A34</f>
+        <v>45Q-2050</v>
+      </c>
+      <c r="B63" s="7" t="str">
+        <f t="shared" si="62"/>
+        <v>500 Mt</v>
+      </c>
+      <c r="C63" s="8">
+        <f t="shared" si="60"/>
+        <v>0.44448412606722876</v>
+      </c>
+      <c r="D63">
+        <f t="shared" si="62"/>
+        <v>-1.3655573070193403</v>
+      </c>
+      <c r="F63" s="8">
+        <f>C63</f>
+        <v>0.44448412606722876</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A64" s="7" t="str">
+        <f t="shared" ref="A64:I64" si="63">A35</f>
+        <v>Innovation-DACHubs</v>
+      </c>
+      <c r="B64" s="7" t="str">
+        <f t="shared" si="63"/>
+        <v>500 Mt</v>
+      </c>
+      <c r="C64" s="8">
+        <f t="shared" si="60"/>
+        <v>0.64724767761331869</v>
+      </c>
+      <c r="D64">
+        <f t="shared" si="63"/>
+        <v>-0.46376197004718345</v>
+      </c>
+      <c r="E64" s="8">
+        <f>C64</f>
+        <v>0.64724767761331869</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A65" s="7" t="str">
+        <f t="shared" ref="A65:I65" si="64">A36</f>
+        <v>Innovation-maintain</v>
+      </c>
+      <c r="B65" s="7" t="str">
+        <f t="shared" si="64"/>
+        <v>500 Mt</v>
+      </c>
+      <c r="C65" s="8">
+        <f t="shared" si="60"/>
+        <v>1.3577275897072081</v>
+      </c>
+      <c r="D65">
+        <f t="shared" si="64"/>
+        <v>-0.15840906711694819</v>
+      </c>
+      <c r="E65" s="8">
+        <f>C65</f>
+        <v>1.3577275897072081</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A66" s="7" t="str">
+        <f t="shared" ref="A66:I66" si="65">A37</f>
+        <v>Innovation-rhodium18b</v>
+      </c>
+      <c r="B66" s="7" t="str">
+        <f t="shared" si="65"/>
+        <v>500 Mt</v>
+      </c>
+      <c r="C66" s="8">
+        <f t="shared" si="60"/>
+        <v>2.3153381298881297</v>
+      </c>
+      <c r="D66">
+        <f t="shared" si="65"/>
+        <v>-1.4997785764247658</v>
+      </c>
+      <c r="E66" s="8">
+        <f>C66</f>
+        <v>2.3153381298881297</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A67" s="7" t="str">
+        <f t="shared" ref="A67:I67" si="66">A38</f>
+        <v>Innovation-rhodium6b</v>
+      </c>
+      <c r="B67" s="7" t="str">
+        <f t="shared" si="66"/>
+        <v>500 Mt</v>
+      </c>
+      <c r="C67" s="8">
+        <f t="shared" si="60"/>
+        <v>1.6348546043849213</v>
+      </c>
+      <c r="D67">
+        <f t="shared" si="66"/>
+        <v>-0.39769251330281402</v>
+      </c>
+      <c r="E67" s="8">
+        <f>C67</f>
+        <v>1.6348546043849213</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A68" s="7" t="str">
+        <f t="shared" ref="A68:I68" si="67">A39</f>
+        <v>Innovation-triple</v>
+      </c>
+      <c r="B68" s="7" t="str">
+        <f t="shared" si="67"/>
+        <v>500 Mt</v>
+      </c>
+      <c r="C68" s="8">
+        <f t="shared" si="60"/>
+        <v>1.6529080927729902</v>
+      </c>
+      <c r="D68">
+        <f t="shared" si="67"/>
+        <v>-0.52357713726908883</v>
+      </c>
+      <c r="E68" s="8">
+        <f>C68</f>
+        <v>1.6529080927729902</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A69" s="7" t="str">
+        <f t="shared" ref="A69:I69" si="68">A40</f>
+        <v>Low Baseline</v>
+      </c>
+      <c r="B69" s="7" t="str">
+        <f t="shared" si="68"/>
+        <v>500 Mt</v>
+      </c>
+      <c r="C69" s="8">
+        <f t="shared" si="60"/>
+        <v>1.5453796931733457</v>
+      </c>
+      <c r="D69">
+        <f t="shared" si="68"/>
+        <v>1.0818447048699995</v>
+      </c>
+      <c r="I69" s="8">
+        <f>C69</f>
+        <v>1.5453796931733457</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A70" s="7" t="str">
+        <f t="shared" ref="A70:I70" si="69">A41</f>
+        <v>Procure3B</v>
+      </c>
+      <c r="B70" s="7" t="str">
+        <f t="shared" si="69"/>
+        <v>500 Mt</v>
+      </c>
+      <c r="C70" s="8">
+        <f t="shared" si="60"/>
+        <v>2.5994756304123183</v>
+      </c>
+      <c r="D70">
+        <f t="shared" si="69"/>
+        <v>0.36638009527595833</v>
+      </c>
+      <c r="G70" s="8">
+        <f>C70</f>
+        <v>2.5994756304123183</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A71" s="7" t="str">
+        <f t="shared" ref="A71:I71" si="70">A42</f>
+        <v>ProcureRhodium</v>
+      </c>
+      <c r="B71" s="7" t="str">
+        <f t="shared" si="70"/>
+        <v>500 Mt</v>
+      </c>
+      <c r="C71" s="8">
+        <f t="shared" si="60"/>
+        <v>8.3515011746760219</v>
+      </c>
+      <c r="D71">
+        <f t="shared" si="70"/>
+        <v>1.1959723569841303</v>
+      </c>
+      <c r="G71" s="8">
+        <f>C71</f>
+        <v>8.3515011746760219</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A72" s="7" t="str">
+        <f t="shared" ref="A72:I72" si="71">A43</f>
+        <v>ProcureScaling</v>
+      </c>
+      <c r="B72" s="7" t="str">
+        <f t="shared" si="71"/>
+        <v>500 Mt</v>
+      </c>
+      <c r="C72" s="8">
+        <f t="shared" si="60"/>
+        <v>1.5468320344764317</v>
+      </c>
+      <c r="D72">
+        <f t="shared" si="71"/>
+        <v>0.36328086889841033</v>
+      </c>
+      <c r="G72" s="8">
+        <f>C72</f>
+        <v>1.5468320344764317</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A73" s="7" t="str">
+        <f t="shared" ref="A73:I73" si="72">A44</f>
+        <v>45Q-2040</v>
+      </c>
+      <c r="B73" s="7" t="str">
+        <f t="shared" si="72"/>
+        <v>1.5 Gt</v>
+      </c>
+      <c r="C73" s="8">
+        <f t="shared" si="60"/>
+        <v>2.5637816421080228</v>
+      </c>
+      <c r="D73">
+        <f t="shared" si="72"/>
+        <v>1.0676371229122197</v>
+      </c>
+      <c r="F73" s="8">
+        <f>C73</f>
+        <v>2.5637816421080228</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A74" s="7" t="str">
+        <f t="shared" ref="A74:I74" si="73">A45</f>
+        <v>45Q-2050</v>
+      </c>
+      <c r="B74" s="7" t="str">
+        <f t="shared" si="73"/>
+        <v>1.5 Gt</v>
+      </c>
+      <c r="C74" s="8">
+        <f t="shared" si="60"/>
+        <v>2.8356658504593448</v>
+      </c>
+      <c r="D74">
+        <f t="shared" si="73"/>
+        <v>0.46865683829263816</v>
+      </c>
+      <c r="F74" s="8">
+        <f>C74</f>
+        <v>2.8356658504593448</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A75" s="7" t="str">
+        <f t="shared" ref="A75:I75" si="74">A46</f>
+        <v>High Baseline</v>
+      </c>
+      <c r="B75" s="7" t="str">
+        <f t="shared" si="74"/>
+        <v>1.5 Gt</v>
+      </c>
+      <c r="C75" s="8">
+        <f t="shared" si="60"/>
+        <v>4.0706852143436585</v>
+      </c>
+      <c r="D75">
+        <f t="shared" si="74"/>
+        <v>2.3727693973872075</v>
+      </c>
+      <c r="I75" s="8">
+        <f>C75</f>
+        <v>4.0706852143436585</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A76" s="7" t="str">
+        <f t="shared" ref="A76:I76" si="75">A47</f>
+        <v>Innovation-DACHubs</v>
+      </c>
+      <c r="B76" s="7" t="str">
+        <f t="shared" si="75"/>
+        <v>1.5 Gt</v>
+      </c>
+      <c r="C76" s="8">
+        <f t="shared" si="60"/>
+        <v>2.1220956593986737</v>
+      </c>
+      <c r="D76">
+        <f t="shared" si="75"/>
+        <v>-1.0959771479748042</v>
+      </c>
+      <c r="E76" s="8">
+        <f>C76</f>
+        <v>2.1220956593986737</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A77" s="7" t="str">
+        <f t="shared" ref="A77:I77" si="76">A48</f>
+        <v>Innovation-maintain</v>
+      </c>
+      <c r="B77" s="7" t="str">
+        <f t="shared" si="76"/>
+        <v>1.5 Gt</v>
+      </c>
+      <c r="C77" s="8">
+        <f t="shared" si="60"/>
+        <v>3.0824499174664326</v>
+      </c>
+      <c r="D77">
+        <f t="shared" si="76"/>
+        <v>-0.67455579376899111</v>
+      </c>
+      <c r="E77" s="8">
+        <f>C77</f>
+        <v>3.0824499174664326</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A78" s="7" t="str">
+        <f t="shared" ref="A78:I78" si="77">A49</f>
+        <v>Innovation-rhodium18b</v>
+      </c>
+      <c r="B78" s="7" t="str">
+        <f t="shared" si="77"/>
+        <v>1.5 Gt</v>
+      </c>
+      <c r="C78" s="8">
+        <f t="shared" si="60"/>
+        <v>2.9048414488544982</v>
+      </c>
+      <c r="D78">
+        <f t="shared" si="77"/>
+        <v>-4.6305696962614666</v>
+      </c>
+      <c r="E78" s="8">
+        <f>C78</f>
+        <v>2.9048414488544982</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A79" s="7" t="str">
+        <f t="shared" ref="A79:I79" si="78">A50</f>
+        <v>Innovation-rhodium6b</v>
+      </c>
+      <c r="B79" s="7" t="str">
+        <f t="shared" si="78"/>
+        <v>1.5 Gt</v>
+      </c>
+      <c r="C79" s="8">
+        <f t="shared" si="60"/>
+        <v>3.1400272434202559</v>
+      </c>
+      <c r="D79">
+        <f t="shared" si="78"/>
+        <v>-1.319407624914968</v>
+      </c>
+      <c r="E79" s="8">
+        <f>C79</f>
+        <v>3.1400272434202559</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A80" s="7" t="str">
+        <f t="shared" ref="A80:I80" si="79">A51</f>
+        <v>Innovation-triple</v>
+      </c>
+      <c r="B80" s="7" t="str">
+        <f t="shared" si="79"/>
+        <v>1.5 Gt</v>
+      </c>
+      <c r="C80" s="8">
+        <f t="shared" si="60"/>
+        <v>3.0444641251640361</v>
+      </c>
+      <c r="D80">
+        <f t="shared" si="79"/>
+        <v>-1.897612583824104</v>
+      </c>
+      <c r="E80" s="8">
+        <f>C80</f>
+        <v>3.0444641251640361</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A81" s="7" t="str">
+        <f t="shared" ref="A81:I81" si="80">A52</f>
+        <v>Procure3B</v>
+      </c>
+      <c r="B81" s="7" t="str">
+        <f t="shared" si="80"/>
+        <v>1.5 Gt</v>
+      </c>
+      <c r="C81" s="8">
+        <f t="shared" si="60"/>
+        <v>4.7171586472895424</v>
+      </c>
+      <c r="D81">
+        <f t="shared" si="80"/>
+        <v>1.0363250084620061</v>
+      </c>
+      <c r="G81" s="8">
+        <f>C81</f>
+        <v>4.7171586472895424</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A82" s="7" t="str">
+        <f t="shared" ref="A82:I82" si="81">A53</f>
+        <v>ProcureRhodium</v>
+      </c>
+      <c r="B82" s="7" t="str">
+        <f t="shared" si="81"/>
+        <v>1.5 Gt</v>
+      </c>
+      <c r="C82" s="8">
+        <f t="shared" si="60"/>
+        <v>10.029059099755278</v>
+      </c>
+      <c r="D82">
+        <f t="shared" si="81"/>
+        <v>2.923407082508354</v>
+      </c>
+      <c r="G82" s="8">
+        <f>C82</f>
+        <v>10.029059099755278</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A83" s="7" t="str">
+        <f t="shared" ref="A83:I83" si="82">A54</f>
+        <v>ProcureScaling</v>
+      </c>
+      <c r="B83" s="7" t="str">
+        <f t="shared" si="82"/>
+        <v>1.5 Gt</v>
+      </c>
+      <c r="C83" s="8">
+        <f t="shared" si="60"/>
+        <v>3.8789631751289115</v>
+      </c>
+      <c r="D83">
+        <f t="shared" si="82"/>
+        <v>0.91897387304034173</v>
+      </c>
+      <c r="G83" s="8">
+        <f>C83</f>
+        <v>3.8789631751289115</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A84" s="7" t="str">
+        <f t="shared" ref="A84:I84" si="83">A55</f>
+        <v>2.4 Gt Baseline</v>
+      </c>
+      <c r="B84" s="7" t="str">
+        <f t="shared" si="83"/>
+        <v>2.4 Gt</v>
+      </c>
+      <c r="C84" s="8">
+        <f t="shared" si="60"/>
+        <v>4.3174474451754374</v>
+      </c>
+      <c r="D84">
+        <f t="shared" si="83"/>
+        <v>-3.8617004313604051</v>
+      </c>
+      <c r="I84" s="8">
+        <f>C84</f>
+        <v>4.3174474451754374</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A85" s="7" t="str">
+        <f t="shared" ref="A85:I85" si="84">A56</f>
+        <v>4.1 Gt Baseline</v>
+      </c>
+      <c r="B85" s="7" t="str">
+        <f t="shared" si="84"/>
+        <v>4.1 Gt</v>
+      </c>
+      <c r="C85" s="8">
+        <f t="shared" si="60"/>
+        <v>5.0029688506972843</v>
+      </c>
+      <c r="D85">
+        <f t="shared" si="84"/>
+        <v>23.306697574041493</v>
+      </c>
+      <c r="I85" s="8">
+        <f>C85</f>
+        <v>5.0029688506972843</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A86" s="7" t="str">
+        <f t="shared" ref="A86:I87" si="85">A57</f>
+        <v>CDRIA-Rhodium18b</v>
+      </c>
+      <c r="B86" s="7" t="str">
+        <f t="shared" si="85"/>
+        <v>500 Mt</v>
+      </c>
+      <c r="C86" s="8">
+        <f t="shared" si="60"/>
+        <v>-3.4159600524698353</v>
+      </c>
+      <c r="D86">
+        <f t="shared" si="85"/>
+        <v>-1.4445409002888128</v>
+      </c>
+      <c r="H86" s="8">
+        <f>C86</f>
+        <v>-3.4159600524698353</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A87" s="7" t="str">
+        <f t="shared" si="85"/>
+        <v>CDRIA-Rhodium18b</v>
+      </c>
+      <c r="B87" s="7" t="str">
+        <f t="shared" si="85"/>
+        <v>1.5 Gt</v>
+      </c>
+      <c r="C87" s="8">
+        <f t="shared" ref="C87" si="86">F28</f>
+        <v>6.0516224069731308</v>
+      </c>
+      <c r="D87">
+        <f t="shared" si="85"/>
+        <v>-4.7728156685049763</v>
+      </c>
+      <c r="H87" s="8">
+        <f>C87</f>
+        <v>6.0516224069731308</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A89" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="B89" t="str">
+        <f>B1</f>
+        <v>Baseline</v>
+      </c>
+      <c r="C89" t="str">
+        <f>H1</f>
+        <v>Cost Decrease necessary in NPV of CDR market | 20.0% discount rate</v>
+      </c>
+      <c r="D89" s="7" t="str">
+        <f t="shared" ref="D89" si="87">D60</f>
+        <v>Cost Decrease necessary in size of the CDR market in 2050</v>
+      </c>
+      <c r="E89" t="s">
+        <v>56</v>
+      </c>
+      <c r="F89" t="s">
+        <v>57</v>
+      </c>
+      <c r="G89" t="s">
+        <v>58</v>
+      </c>
+      <c r="H89" t="s">
+        <v>55</v>
+      </c>
+      <c r="I89" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A90" s="7" t="str">
+        <f>A61</f>
+        <v>100 Mt Baseline</v>
+      </c>
+      <c r="B90" s="7" t="str">
+        <f>B61</f>
+        <v>100 Mt</v>
+      </c>
+      <c r="C90">
+        <f>H2</f>
+        <v>0</v>
+      </c>
+      <c r="D90" s="8">
+        <f>D61</f>
+        <v>0</v>
+      </c>
+      <c r="I90" s="8">
+        <f>C90</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A91" s="7" t="str">
+        <f t="shared" ref="A91:B91" si="88">A62</f>
+        <v>45Q-2040</v>
+      </c>
+      <c r="B91" s="7" t="str">
+        <f t="shared" si="88"/>
+        <v>500 Mt</v>
+      </c>
+      <c r="C91">
+        <f t="shared" ref="C91:C116" si="89">H3</f>
+        <v>1.3438885594409384</v>
+      </c>
+      <c r="D91" s="8">
+        <f t="shared" ref="D91:D116" si="90">D62</f>
+        <v>0.21249703186680166</v>
+      </c>
+      <c r="F91" s="8">
+        <f>C91</f>
+        <v>1.3438885594409384</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A92" s="7" t="str">
+        <f t="shared" ref="A92:B92" si="91">A63</f>
+        <v>45Q-2050</v>
+      </c>
+      <c r="B92" s="7" t="str">
+        <f t="shared" si="91"/>
+        <v>500 Mt</v>
+      </c>
+      <c r="C92">
+        <f t="shared" si="89"/>
+        <v>0.84723170018844907</v>
+      </c>
+      <c r="D92" s="8">
+        <f t="shared" si="90"/>
+        <v>-1.3655573070193403</v>
+      </c>
+      <c r="F92" s="8">
+        <f>C92</f>
+        <v>0.84723170018844907</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A93" s="7" t="str">
+        <f t="shared" ref="A93:B93" si="92">A64</f>
+        <v>Innovation-DACHubs</v>
+      </c>
+      <c r="B93" s="7" t="str">
+        <f t="shared" si="92"/>
+        <v>500 Mt</v>
+      </c>
+      <c r="C93">
+        <f t="shared" si="89"/>
+        <v>1.0932573496051559</v>
+      </c>
+      <c r="D93" s="8">
+        <f t="shared" si="90"/>
+        <v>-0.46376197004718345</v>
+      </c>
+      <c r="E93" s="8">
+        <f>C93</f>
+        <v>1.0932573496051559</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A94" s="7" t="str">
+        <f t="shared" ref="A94:B94" si="93">A65</f>
+        <v>Innovation-maintain</v>
+      </c>
+      <c r="B94" s="7" t="str">
+        <f t="shared" si="93"/>
+        <v>500 Mt</v>
+      </c>
+      <c r="C94">
+        <f t="shared" si="89"/>
+        <v>1.6946076320487724</v>
+      </c>
+      <c r="D94" s="8">
+        <f t="shared" si="90"/>
+        <v>-0.15840906711694819</v>
+      </c>
+      <c r="E94" s="8">
+        <f>C94</f>
+        <v>1.6946076320487724</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A95" s="7" t="str">
+        <f t="shared" ref="A95:B95" si="94">A66</f>
+        <v>Innovation-rhodium18b</v>
+      </c>
+      <c r="B95" s="7" t="str">
+        <f t="shared" si="94"/>
+        <v>500 Mt</v>
+      </c>
+      <c r="C95">
+        <f t="shared" si="89"/>
+        <v>3.2502144071938046</v>
+      </c>
+      <c r="D95" s="8">
+        <f t="shared" si="90"/>
+        <v>-1.4997785764247658</v>
+      </c>
+      <c r="E95" s="8">
+        <f>C95</f>
+        <v>3.2502144071938046</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A96" s="7" t="str">
+        <f t="shared" ref="A96:B96" si="95">A67</f>
+        <v>Innovation-rhodium6b</v>
+      </c>
+      <c r="B96" s="7" t="str">
+        <f t="shared" si="95"/>
+        <v>500 Mt</v>
+      </c>
+      <c r="C96">
+        <f t="shared" si="89"/>
+        <v>2.1049050122513044</v>
+      </c>
+      <c r="D96" s="8">
+        <f t="shared" si="90"/>
+        <v>-0.39769251330281402</v>
+      </c>
+      <c r="E96" s="8">
+        <f>C96</f>
+        <v>2.1049050122513044</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A97" s="7" t="str">
+        <f t="shared" ref="A97:B97" si="96">A68</f>
+        <v>Innovation-triple</v>
+      </c>
+      <c r="B97" s="7" t="str">
+        <f t="shared" si="96"/>
+        <v>500 Mt</v>
+      </c>
+      <c r="C97">
+        <f t="shared" si="89"/>
+        <v>2.2091624983315339</v>
+      </c>
+      <c r="D97" s="8">
+        <f t="shared" si="90"/>
+        <v>-0.52357713726908883</v>
+      </c>
+      <c r="E97" s="8">
+        <f>C97</f>
+        <v>2.2091624983315339</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A98" s="7" t="str">
+        <f t="shared" ref="A98:B98" si="97">A69</f>
+        <v>Low Baseline</v>
+      </c>
+      <c r="B98" s="7" t="str">
+        <f t="shared" si="97"/>
+        <v>500 Mt</v>
+      </c>
+      <c r="C98">
+        <f t="shared" si="89"/>
+        <v>1.5827998282841693</v>
+      </c>
+      <c r="D98" s="8">
+        <f t="shared" si="90"/>
+        <v>1.0818447048699995</v>
+      </c>
+      <c r="I98" s="8">
+        <f>C98</f>
+        <v>1.5827998282841693</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A99" s="7" t="str">
+        <f t="shared" ref="A99:B99" si="98">A70</f>
+        <v>Procure3B</v>
+      </c>
+      <c r="B99" s="7" t="str">
+        <f t="shared" si="98"/>
+        <v>500 Mt</v>
+      </c>
+      <c r="C99">
+        <f t="shared" si="89"/>
+        <v>4.0670809313292864</v>
+      </c>
+      <c r="D99" s="8">
+        <f t="shared" si="90"/>
+        <v>0.36638009527595833</v>
+      </c>
+      <c r="G99" s="8">
+        <f>C99</f>
+        <v>4.0670809313292864</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A100" s="7" t="str">
+        <f t="shared" ref="A100:B100" si="99">A71</f>
+        <v>ProcureRhodium</v>
+      </c>
+      <c r="B100" s="7" t="str">
+        <f t="shared" si="99"/>
+        <v>500 Mt</v>
+      </c>
+      <c r="C100">
+        <f t="shared" si="89"/>
+        <v>10.956263412283258</v>
+      </c>
+      <c r="D100" s="8">
+        <f t="shared" si="90"/>
+        <v>1.1959723569841303</v>
+      </c>
+      <c r="G100" s="8">
+        <f>C100</f>
+        <v>10.956263412283258</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A101" s="7" t="str">
+        <f t="shared" ref="A101:B101" si="100">A72</f>
+        <v>ProcureScaling</v>
+      </c>
+      <c r="B101" s="7" t="str">
+        <f t="shared" si="100"/>
+        <v>500 Mt</v>
+      </c>
+      <c r="C101">
+        <f t="shared" si="89"/>
+        <v>1.9108299722709272</v>
+      </c>
+      <c r="D101" s="8">
+        <f t="shared" si="90"/>
+        <v>0.36328086889841033</v>
+      </c>
+      <c r="G101" s="8">
+        <f>C101</f>
+        <v>1.9108299722709272</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A102" s="7" t="str">
+        <f t="shared" ref="A102:B102" si="101">A73</f>
+        <v>45Q-2040</v>
+      </c>
+      <c r="B102" s="7" t="str">
+        <f t="shared" si="101"/>
+        <v>1.5 Gt</v>
+      </c>
+      <c r="C102">
+        <f t="shared" si="89"/>
+        <v>2.9242921759498324</v>
+      </c>
+      <c r="D102" s="8">
+        <f t="shared" si="90"/>
+        <v>1.0676371229122197</v>
+      </c>
+      <c r="F102" s="8">
+        <f>C102</f>
+        <v>2.9242921759498324</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A103" s="7" t="str">
+        <f t="shared" ref="A103:B103" si="102">A74</f>
+        <v>45Q-2050</v>
+      </c>
+      <c r="B103" s="7" t="str">
+        <f t="shared" si="102"/>
+        <v>1.5 Gt</v>
+      </c>
+      <c r="C103">
+        <f t="shared" si="89"/>
+        <v>3.2080184026842988</v>
+      </c>
+      <c r="D103" s="8">
+        <f t="shared" si="90"/>
+        <v>0.46865683829263816</v>
+      </c>
+      <c r="F103" s="8">
+        <f>C103</f>
+        <v>3.2080184026842988</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A104" s="7" t="str">
+        <f t="shared" ref="A104:B104" si="103">A75</f>
+        <v>High Baseline</v>
+      </c>
+      <c r="B104" s="7" t="str">
+        <f t="shared" si="103"/>
+        <v>1.5 Gt</v>
+      </c>
+      <c r="C104">
+        <f t="shared" si="89"/>
+        <v>4.0371470003985861</v>
+      </c>
+      <c r="D104" s="8">
+        <f t="shared" si="90"/>
+        <v>2.3727693973872075</v>
+      </c>
+      <c r="I104" s="8">
+        <f>C104</f>
+        <v>4.0371470003985861</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A105" s="7" t="str">
+        <f t="shared" ref="A105:B105" si="104">A76</f>
+        <v>Innovation-DACHubs</v>
+      </c>
+      <c r="B105" s="7" t="str">
+        <f t="shared" si="104"/>
+        <v>1.5 Gt</v>
+      </c>
+      <c r="C105">
+        <f t="shared" si="89"/>
+        <v>2.693095733872942</v>
+      </c>
+      <c r="D105" s="8">
+        <f t="shared" si="90"/>
+        <v>-1.0959771479748042</v>
+      </c>
+      <c r="E105" s="8">
+        <f>C105</f>
+        <v>2.693095733872942</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A106" s="7" t="str">
+        <f t="shared" ref="A106:B106" si="105">A77</f>
+        <v>Innovation-maintain</v>
+      </c>
+      <c r="B106" s="7" t="str">
+        <f t="shared" si="105"/>
+        <v>1.5 Gt</v>
+      </c>
+      <c r="C106">
+        <f t="shared" si="89"/>
+        <v>3.5163830940418412</v>
+      </c>
+      <c r="D106" s="8">
+        <f t="shared" si="90"/>
+        <v>-0.67455579376899111</v>
+      </c>
+      <c r="E106" s="8">
+        <f>C106</f>
+        <v>3.5163830940418412</v>
+      </c>
+    </row>
+    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A107" s="7" t="str">
+        <f t="shared" ref="A107:B107" si="106">A78</f>
+        <v>Innovation-rhodium18b</v>
+      </c>
+      <c r="B107" s="7" t="str">
+        <f t="shared" si="106"/>
+        <v>1.5 Gt</v>
+      </c>
+      <c r="C107">
+        <f t="shared" si="89"/>
+        <v>4.2476127361252409</v>
+      </c>
+      <c r="D107" s="8">
+        <f t="shared" si="90"/>
+        <v>-4.6305696962614666</v>
+      </c>
+      <c r="E107" s="8">
+        <f>C107</f>
+        <v>4.2476127361252409</v>
+      </c>
+    </row>
+    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A108" s="7" t="str">
+        <f t="shared" ref="A108:B108" si="107">A79</f>
+        <v>Innovation-rhodium6b</v>
+      </c>
+      <c r="B108" s="7" t="str">
+        <f t="shared" si="107"/>
+        <v>1.5 Gt</v>
+      </c>
+      <c r="C108">
+        <f t="shared" si="89"/>
+        <v>3.7562358691096911</v>
+      </c>
+      <c r="D108" s="8">
+        <f t="shared" si="90"/>
+        <v>-1.319407624914968</v>
+      </c>
+      <c r="E108" s="8">
+        <f>C108</f>
+        <v>3.7562358691096911</v>
+      </c>
+    </row>
+    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A109" s="7" t="str">
+        <f t="shared" ref="A109:B109" si="108">A80</f>
+        <v>Innovation-triple</v>
+      </c>
+      <c r="B109" s="7" t="str">
+        <f t="shared" si="108"/>
+        <v>1.5 Gt</v>
+      </c>
+      <c r="C109">
+        <f t="shared" si="89"/>
+        <v>3.7941739897941655</v>
+      </c>
+      <c r="D109" s="8">
+        <f t="shared" si="90"/>
+        <v>-1.897612583824104</v>
+      </c>
+      <c r="E109" s="8">
+        <f>C109</f>
+        <v>3.7941739897941655</v>
+      </c>
+    </row>
+    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A110" s="7" t="str">
+        <f t="shared" ref="A110:B110" si="109">A81</f>
+        <v>Procure3B</v>
+      </c>
+      <c r="B110" s="7" t="str">
+        <f t="shared" si="109"/>
+        <v>1.5 Gt</v>
+      </c>
+      <c r="C110">
+        <f t="shared" si="89"/>
+        <v>6.1482838611335504</v>
+      </c>
+      <c r="D110" s="8">
+        <f t="shared" si="90"/>
+        <v>1.0363250084620061</v>
+      </c>
+      <c r="G110" s="8">
+        <f>C110</f>
+        <v>6.1482838611335504</v>
+      </c>
+    </row>
+    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A111" s="7" t="str">
+        <f t="shared" ref="A111:B111" si="110">A82</f>
+        <v>ProcureRhodium</v>
+      </c>
+      <c r="B111" s="7" t="str">
+        <f t="shared" si="110"/>
+        <v>1.5 Gt</v>
+      </c>
+      <c r="C111">
+        <f t="shared" si="89"/>
+        <v>12.663601837356222</v>
+      </c>
+      <c r="D111" s="8">
+        <f t="shared" si="90"/>
+        <v>2.923407082508354</v>
+      </c>
+      <c r="G111" s="8">
+        <f>C111</f>
+        <v>12.663601837356222</v>
+      </c>
+    </row>
+    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A112" s="7" t="str">
+        <f t="shared" ref="A112:B112" si="111">A83</f>
+        <v>ProcureScaling</v>
+      </c>
+      <c r="B112" s="7" t="str">
+        <f t="shared" si="111"/>
+        <v>1.5 Gt</v>
+      </c>
+      <c r="C112">
+        <f t="shared" si="89"/>
+        <v>4.293953690244436</v>
+      </c>
+      <c r="D112" s="8">
+        <f t="shared" si="90"/>
+        <v>0.91897387304034173</v>
+      </c>
+      <c r="G112" s="8">
+        <f>C112</f>
+        <v>4.293953690244436</v>
+      </c>
+    </row>
+    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A113" s="7" t="str">
+        <f t="shared" ref="A113:B113" si="112">A84</f>
+        <v>2.4 Gt Baseline</v>
+      </c>
+      <c r="B113" s="7" t="str">
+        <f t="shared" si="112"/>
+        <v>2.4 Gt</v>
+      </c>
+      <c r="C113">
+        <f t="shared" si="89"/>
+        <v>4.7441533574965318</v>
+      </c>
+      <c r="D113" s="8">
+        <f t="shared" si="90"/>
+        <v>-3.8617004313604051</v>
+      </c>
+      <c r="I113" s="8">
+        <f>C113</f>
+        <v>4.7441533574965318</v>
+      </c>
+    </row>
+    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A114" s="7" t="str">
+        <f t="shared" ref="A114:B114" si="113">A85</f>
+        <v>4.1 Gt Baseline</v>
+      </c>
+      <c r="B114" s="7" t="str">
+        <f t="shared" si="113"/>
+        <v>4.1 Gt</v>
+      </c>
+      <c r="C114">
+        <f t="shared" si="89"/>
+        <v>5.4960134486937662</v>
+      </c>
+      <c r="D114" s="8">
+        <f t="shared" si="90"/>
+        <v>23.306697574041493</v>
+      </c>
+      <c r="I114" s="8">
+        <f>C114</f>
+        <v>5.4960134486937662</v>
+      </c>
+    </row>
+    <row r="115" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A115" s="7" t="str">
+        <f t="shared" ref="A115:B115" si="114">A86</f>
+        <v>CDRIA-Rhodium18b</v>
+      </c>
+      <c r="B115" s="7" t="str">
+        <f t="shared" si="114"/>
+        <v>500 Mt</v>
+      </c>
+      <c r="C115">
+        <f t="shared" si="89"/>
+        <v>-4.1388574181998177</v>
+      </c>
+      <c r="D115" s="8">
+        <f t="shared" si="90"/>
+        <v>-1.4445409002888128</v>
+      </c>
+      <c r="H115" s="8">
+        <f>C115</f>
+        <v>-4.1388574181998177</v>
+      </c>
+    </row>
+    <row r="116" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A116" s="7" t="str">
+        <f t="shared" ref="A116:B116" si="115">A87</f>
+        <v>CDRIA-Rhodium18b</v>
+      </c>
+      <c r="B116" s="7" t="str">
+        <f t="shared" si="115"/>
+        <v>1.5 Gt</v>
+      </c>
+      <c r="C116">
+        <f t="shared" si="89"/>
+        <v>7.6155443923701611</v>
+      </c>
+      <c r="D116" s="8">
+        <f t="shared" si="90"/>
+        <v>-4.7728156685049763</v>
+      </c>
+      <c r="H116">
+        <f>C116</f>
+        <v>7.6155443923701611</v>
       </c>
     </row>
   </sheetData>
@@ -12259,7 +17064,7 @@
   </autoFilter>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="D2:D28 F2:F28 H2:I28">
-    <cfRule type="colorScale" priority="1">
+    <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="num" val="0"/>
@@ -12271,7 +17076,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E35:Z35 E36:E39">
-    <cfRule type="colorScale" priority="2">
+    <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="num" val="0"/>

</xml_diff>

<commit_message>
optimal scenario config files
</commit_message>
<xml_diff>
--- a/data/data_analysis/policy_effectiveness.xlsx
+++ b/data/data_analysis/policy_effectiveness.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\PycharmProjects\GCAM-CDR-policy\data\data_analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF9D5C8E-A71E-4428-A8F4-67EC550AA7E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5345F5C3-691B-42EC-9114-60FC3EA57057}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-15" yWindow="3525" windowWidth="28740" windowHeight="13845" activeTab="1" xr2:uid="{5B094011-67C9-461D-BBBF-A6D3FE50B4AB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{5B094011-67C9-461D-BBBF-A6D3FE50B4AB}"/>
   </bookViews>
   <sheets>
     <sheet name="Low" sheetId="1" r:id="rId1"/>
@@ -30577,15 +30577,42 @@
       <c r="A5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6"/>
-      <c r="K5" s="6"/>
-      <c r="M5" s="6"/>
+      <c r="B5" s="6">
+        <v>-1464989.78716154</v>
+      </c>
+      <c r="C5" s="6">
+        <v>1485429.39379307</v>
+      </c>
+      <c r="D5" s="5">
+        <v>-0.98623993390938702</v>
+      </c>
+      <c r="E5" s="6">
+        <v>20439.606631531598</v>
+      </c>
+      <c r="F5" s="6">
+        <v>-244021.109044115</v>
+      </c>
+      <c r="G5" s="6">
+        <v>269761.83991016098</v>
+      </c>
+      <c r="H5" s="5">
+        <v>-0.90457979203204397</v>
+      </c>
+      <c r="I5" s="6">
+        <v>25740.730866045898</v>
+      </c>
+      <c r="J5" s="6">
+        <v>-77084.450851909904</v>
+      </c>
+      <c r="K5" s="6">
+        <v>96376.642356775497</v>
+      </c>
+      <c r="L5" s="5">
+        <v>-0.79982502987136495</v>
+      </c>
+      <c r="M5" s="6">
+        <v>19292.191504865601</v>
+      </c>
       <c r="N5" t="s">
         <v>24</v>
       </c>
@@ -31233,51 +31260,51 @@
       </c>
       <c r="B21" s="6">
         <f>B5-B$33</f>
-        <v>0</v>
+        <v>-1464989.78716154</v>
       </c>
       <c r="C21" s="6">
         <f>C5-C$33</f>
-        <v>-15116.4576849762</v>
+        <v>1470312.9361080937</v>
       </c>
       <c r="D21" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-0.99637958096142165</v>
       </c>
       <c r="E21" s="6">
         <f t="shared" si="1"/>
-        <v>-15116.4576849762</v>
+        <v>5323.1489465537015</v>
       </c>
       <c r="F21" s="6">
         <f>F5-F$33</f>
-        <v>0</v>
+        <v>-244021.109044115</v>
       </c>
       <c r="G21" s="6">
         <f>G5-G$33</f>
-        <v>-11664.787219482399</v>
+        <v>258097.0526906786</v>
       </c>
       <c r="H21" s="5">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-0.94546259440074587</v>
       </c>
       <c r="I21" s="6">
         <f t="shared" si="3"/>
-        <v>-11664.787219482399</v>
+        <v>14075.943646563595</v>
       </c>
       <c r="J21" s="6">
         <f>J5-J$33</f>
-        <v>0</v>
+        <v>-77084.450851909904</v>
       </c>
       <c r="K21" s="6">
         <f>K5-K$33</f>
-        <v>-9787.7637750826798</v>
+        <v>86588.878581692814</v>
       </c>
       <c r="L21" s="5">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>-0.89023500609473882</v>
       </c>
       <c r="M21" s="6">
         <f t="shared" si="5"/>
-        <v>-9787.7637750826798</v>
+        <v>9504.4277297829103</v>
       </c>
       <c r="N21" t="s">
         <v>24</v>

</xml_diff>